<commit_message>
feat(P7): Naming Rule 통일 + Candidate Concepts 시트 (Stage 1 LOCK)
- Feature Naming Rule 전면 통일: [Object] [Attribute] (Phase)
  · Open Pelvis At Impact → Pelvis Open (P7) 등 16개 Feature 표시명/ID 정규화
  · Pattern Feature 예외(Standing Up/Chicken Wing 명칭 유지) + Hand Position Axes 규칙
  · Mechanism 'Used In' ID 참조 일괄 remap
- DOH Candidate Concepts 시트 신설(Definition/First Found/Status/Example, Repeated 공백)
  · Club Path Out-To-In·In-To-Out, Face Closure Late, Trail Elbow Out, Forward COM 등록
  · 후보 노드 재분류 로그(Derived/Coaching/Merged/Setup/P8-defer)
- Naming Rule에 Role Taxonomy + Dictionary 수정정책(P4 후 1회 리팩토링) 반영
- PST 카테고리 유지(LOCK)

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01AdDd8hWZsADEXdqNySEqXP
</commit_message>
<xml_diff>
--- a/DOH_P7.xlsx
+++ b/DOH_P7.xlsx
@@ -12,9 +12,10 @@
     <sheet name="Observation_Dictionary" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="Naming Rule" sheetId="4" state="visible" r:id="rId4"/>
     <sheet name="Evidence Layer" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="DOH Coaching Knowledge" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="Derived Parameters" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="Todo" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="DOH Candidate Concepts" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="DOH Coaching Knowledge" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="Derived Parameters" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="Todo" sheetId="9" state="visible" r:id="rId9"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -521,7 +522,7 @@
       <c r="D2" s="2" t="inlineStr"/>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>forward_hands</t>
+          <t>hand_direction_forward_p7</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
@@ -549,7 +550,7 @@
       <c r="D3" s="2" t="inlineStr"/>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>forward_hands</t>
+          <t>hand_direction_forward_p7</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
@@ -577,7 +578,7 @@
       <c r="D4" s="2" t="inlineStr"/>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>forward_hands</t>
+          <t>hand_direction_forward_p7</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
@@ -605,7 +606,7 @@
       <c r="D5" s="2" t="inlineStr"/>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>forward_hands</t>
+          <t>hand_direction_forward_p7</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
@@ -633,7 +634,7 @@
       <c r="D6" s="2" t="inlineStr"/>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>club_face_closed_impact</t>
+          <t>club_face_closed_p7</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
@@ -661,7 +662,7 @@
       <c r="D7" s="2" t="inlineStr"/>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>club_face_open_impact</t>
+          <t>club_face_open_p7</t>
         </is>
       </c>
       <c r="F7" s="2" t="inlineStr">
@@ -689,7 +690,7 @@
       <c r="D8" s="2" t="inlineStr"/>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>club_face_open_impact</t>
+          <t>club_face_open_p7</t>
         </is>
       </c>
       <c r="F8" s="2" t="inlineStr">
@@ -717,7 +718,7 @@
       <c r="D9" s="2" t="inlineStr"/>
       <c r="E9" s="2" t="inlineStr">
         <is>
-          <t>club_face_closed_impact</t>
+          <t>club_face_closed_p7</t>
         </is>
       </c>
       <c r="F9" s="2" t="inlineStr">
@@ -749,7 +750,7 @@
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>club_face_open_impact</t>
+          <t>club_face_open_p7</t>
         </is>
       </c>
       <c r="F10" s="2" t="inlineStr">
@@ -781,7 +782,7 @@
       </c>
       <c r="E11" s="2" t="inlineStr">
         <is>
-          <t>club_face_closed_impact</t>
+          <t>club_face_closed_p7</t>
         </is>
       </c>
       <c r="F11" s="2" t="inlineStr">
@@ -809,7 +810,7 @@
       <c r="D12" s="2" t="inlineStr"/>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t>club_face_open_impact</t>
+          <t>club_face_open_p7</t>
         </is>
       </c>
       <c r="F12" s="2" t="inlineStr">
@@ -841,7 +842,7 @@
       </c>
       <c r="E13" s="2" t="inlineStr">
         <is>
-          <t>club_face_closed_impact</t>
+          <t>club_face_closed_p7</t>
         </is>
       </c>
       <c r="F13" s="2" t="inlineStr">
@@ -873,7 +874,7 @@
       </c>
       <c r="E14" s="2" t="inlineStr">
         <is>
-          <t>club_face_open_impact</t>
+          <t>club_face_open_p7</t>
         </is>
       </c>
       <c r="F14" s="2" t="inlineStr">
@@ -905,7 +906,7 @@
       </c>
       <c r="E15" s="2" t="inlineStr">
         <is>
-          <t>club_face_open_impact</t>
+          <t>club_face_open_p7</t>
         </is>
       </c>
       <c r="F15" s="2" t="inlineStr">
@@ -941,9 +942,9 @@
       </c>
       <c r="E16" s="2" t="inlineStr">
         <is>
-          <t>club_face_open_impact
-open_pelvis_impact
-open_thorax_impact</t>
+          <t>club_face_open_p7
+pelvis_open_p7
+thorax_open_p7</t>
         </is>
       </c>
       <c r="F16" s="2" t="inlineStr">
@@ -975,8 +976,8 @@
       </c>
       <c r="E17" s="2" t="inlineStr">
         <is>
-          <t>club_face_open_impact
-forward_hands</t>
+          <t>club_face_open_p7
+hand_direction_forward_p7</t>
         </is>
       </c>
       <c r="F17" s="2" t="inlineStr">
@@ -1004,7 +1005,7 @@
       <c r="D18" s="2" t="inlineStr"/>
       <c r="E18" s="2" t="inlineStr">
         <is>
-          <t>club_face_closed_impact</t>
+          <t>club_face_closed_p7</t>
         </is>
       </c>
       <c r="F18" s="2" t="inlineStr">
@@ -1036,8 +1037,8 @@
       </c>
       <c r="E19" s="2" t="inlineStr">
         <is>
-          <t>club_face_closed_impact
-closed_pelvis_impact</t>
+          <t>club_face_closed_p7
+pelvis_closed_p7</t>
         </is>
       </c>
       <c r="F19" s="2" t="inlineStr">
@@ -1070,7 +1071,7 @@
       </c>
       <c r="E20" s="2" t="inlineStr">
         <is>
-          <t>open_pelvis_impact</t>
+          <t>pelvis_open_p7</t>
         </is>
       </c>
       <c r="F20" s="2" t="inlineStr">
@@ -1102,7 +1103,7 @@
       </c>
       <c r="E21" s="2" t="inlineStr">
         <is>
-          <t>open_thorax_impact</t>
+          <t>thorax_open_p7</t>
         </is>
       </c>
       <c r="F21" s="2" t="inlineStr">
@@ -1130,7 +1131,7 @@
       <c r="D22" s="2" t="inlineStr"/>
       <c r="E22" s="2" t="inlineStr">
         <is>
-          <t>closed_thorax_impact</t>
+          <t>thorax_closed_p7</t>
         </is>
       </c>
       <c r="F22" s="2" t="inlineStr">
@@ -1162,7 +1163,7 @@
       </c>
       <c r="E23" s="2" t="inlineStr">
         <is>
-          <t>hands_too_close</t>
+          <t>hand_distance_close_p7</t>
         </is>
       </c>
       <c r="F23" s="2" t="inlineStr">
@@ -1190,7 +1191,7 @@
       <c r="D24" s="2" t="inlineStr"/>
       <c r="E24" s="2" t="inlineStr">
         <is>
-          <t>closed_thorax_impact</t>
+          <t>thorax_closed_p7</t>
         </is>
       </c>
       <c r="F24" s="2" t="inlineStr">
@@ -1223,7 +1224,7 @@
       </c>
       <c r="E25" s="2" t="inlineStr">
         <is>
-          <t>club_face_open_impact</t>
+          <t>club_face_open_p7</t>
         </is>
       </c>
       <c r="F25" s="2" t="inlineStr">
@@ -1256,8 +1257,8 @@
       </c>
       <c r="E26" s="2" t="inlineStr">
         <is>
-          <t>chicken_wing
-closed_pelvis_impact</t>
+          <t>chicken_wing_p7
+pelvis_closed_p7</t>
         </is>
       </c>
       <c r="F26" s="2" t="inlineStr">
@@ -1285,7 +1286,7 @@
       <c r="D27" s="2" t="inlineStr"/>
       <c r="E27" s="2" t="inlineStr">
         <is>
-          <t>forward_hands</t>
+          <t>hand_direction_forward_p7</t>
         </is>
       </c>
       <c r="F27" s="2" t="inlineStr">
@@ -1317,7 +1318,7 @@
       </c>
       <c r="E28" s="2" t="inlineStr">
         <is>
-          <t>forward_hands</t>
+          <t>hand_direction_forward_p7</t>
         </is>
       </c>
       <c r="F28" s="2" t="inlineStr">
@@ -1349,7 +1350,7 @@
       </c>
       <c r="E29" s="2" t="inlineStr">
         <is>
-          <t>open_pelvis_impact</t>
+          <t>pelvis_open_p7</t>
         </is>
       </c>
       <c r="F29" s="2" t="inlineStr">
@@ -1381,7 +1382,7 @@
       </c>
       <c r="E30" s="2" t="inlineStr">
         <is>
-          <t>open_pelvis_impact</t>
+          <t>pelvis_open_p7</t>
         </is>
       </c>
       <c r="F30" s="2" t="inlineStr">
@@ -1413,8 +1414,8 @@
       </c>
       <c r="E31" s="2" t="inlineStr">
         <is>
-          <t>open_pelvis_impact
-open_thorax_impact</t>
+          <t>pelvis_open_p7
+thorax_open_p7</t>
         </is>
       </c>
       <c r="F31" s="2" t="inlineStr">
@@ -1446,7 +1447,7 @@
       </c>
       <c r="E32" s="2" t="inlineStr">
         <is>
-          <t>open_thorax_impact</t>
+          <t>thorax_open_p7</t>
         </is>
       </c>
       <c r="F32" s="2" t="inlineStr">
@@ -1474,7 +1475,7 @@
       <c r="D33" s="2" t="inlineStr"/>
       <c r="E33" s="2" t="inlineStr">
         <is>
-          <t>open_thorax_impact</t>
+          <t>thorax_open_p7</t>
         </is>
       </c>
       <c r="F33" s="2" t="inlineStr">
@@ -1506,7 +1507,7 @@
       </c>
       <c r="E34" s="2" t="inlineStr">
         <is>
-          <t>open_thorax_impact</t>
+          <t>thorax_open_p7</t>
         </is>
       </c>
       <c r="F34" s="2" t="inlineStr">
@@ -1538,7 +1539,7 @@
       </c>
       <c r="E35" s="2" t="inlineStr">
         <is>
-          <t>closed_pelvis_impact</t>
+          <t>pelvis_closed_p7</t>
         </is>
       </c>
       <c r="F35" s="2" t="inlineStr">
@@ -1570,7 +1571,7 @@
       </c>
       <c r="E36" s="2" t="inlineStr">
         <is>
-          <t>closed_thorax_impact</t>
+          <t>thorax_closed_p7</t>
         </is>
       </c>
       <c r="F36" s="2" t="inlineStr">
@@ -1602,8 +1603,8 @@
       </c>
       <c r="E37" s="2" t="inlineStr">
         <is>
-          <t>closed_pelvis_impact
-closed_thorax_impact</t>
+          <t>pelvis_closed_p7
+thorax_closed_p7</t>
         </is>
       </c>
       <c r="F37" s="2" t="inlineStr">
@@ -1637,8 +1638,8 @@
       </c>
       <c r="E38" s="2" t="inlineStr">
         <is>
-          <t>open_pelvis_impact
-open_thorax_impact</t>
+          <t>pelvis_open_p7
+thorax_open_p7</t>
         </is>
       </c>
       <c r="F38" s="2" t="inlineStr">
@@ -1666,7 +1667,7 @@
       <c r="D39" s="2" t="inlineStr"/>
       <c r="E39" s="2" t="inlineStr">
         <is>
-          <t>closed_pelvis_impact</t>
+          <t>pelvis_closed_p7</t>
         </is>
       </c>
       <c r="F39" s="2" t="inlineStr">
@@ -1698,7 +1699,7 @@
       </c>
       <c r="E40" s="2" t="inlineStr">
         <is>
-          <t>closed_pelvis_impact</t>
+          <t>pelvis_closed_p7</t>
         </is>
       </c>
       <c r="F40" s="2" t="inlineStr">
@@ -1730,7 +1731,7 @@
       </c>
       <c r="E41" s="2" t="inlineStr">
         <is>
-          <t>lead_pressure_excessive_impact</t>
+          <t>lead_pressure_excessive_p7</t>
         </is>
       </c>
       <c r="F41" s="2" t="inlineStr">
@@ -1758,7 +1759,7 @@
       <c r="D42" s="2" t="inlineStr"/>
       <c r="E42" s="2" t="inlineStr">
         <is>
-          <t>forward_hands</t>
+          <t>hand_direction_forward_p7</t>
         </is>
       </c>
       <c r="F42" s="2" t="inlineStr">
@@ -1791,7 +1792,7 @@
       </c>
       <c r="E43" s="2" t="inlineStr">
         <is>
-          <t>lead_pressure_excessive_impact</t>
+          <t>lead_pressure_excessive_p7</t>
         </is>
       </c>
       <c r="F43" s="2" t="inlineStr">
@@ -1823,7 +1824,7 @@
       </c>
       <c r="E44" s="2" t="inlineStr">
         <is>
-          <t>lead_pressure_excessive_impact</t>
+          <t>lead_pressure_excessive_p7</t>
         </is>
       </c>
       <c r="F44" s="2" t="inlineStr">
@@ -1855,7 +1856,7 @@
       </c>
       <c r="E45" s="2" t="inlineStr">
         <is>
-          <t>lead_pressure_excessive_impact</t>
+          <t>lead_pressure_excessive_p7</t>
         </is>
       </c>
       <c r="F45" s="2" t="inlineStr">
@@ -1887,7 +1888,7 @@
       </c>
       <c r="E46" s="2" t="inlineStr">
         <is>
-          <t>lead_pressure_excessive_impact</t>
+          <t>lead_pressure_excessive_p7</t>
         </is>
       </c>
       <c r="F46" s="2" t="inlineStr">
@@ -1915,7 +1916,7 @@
       <c r="D47" s="2" t="inlineStr"/>
       <c r="E47" s="2" t="inlineStr">
         <is>
-          <t>closed_pelvis_impact</t>
+          <t>pelvis_closed_p7</t>
         </is>
       </c>
       <c r="F47" s="2" t="inlineStr">
@@ -1943,7 +1944,7 @@
       <c r="D48" s="2" t="inlineStr"/>
       <c r="E48" s="2" t="inlineStr">
         <is>
-          <t>lead_pressure_excessive_impact</t>
+          <t>lead_pressure_excessive_p7</t>
         </is>
       </c>
       <c r="F48" s="2" t="inlineStr">
@@ -1971,7 +1972,7 @@
       <c r="D49" s="2" t="inlineStr"/>
       <c r="E49" s="2" t="inlineStr">
         <is>
-          <t>lead_pressure_excessive_impact</t>
+          <t>lead_pressure_excessive_p7</t>
         </is>
       </c>
       <c r="F49" s="2" t="inlineStr">
@@ -2003,7 +2004,7 @@
       </c>
       <c r="E50" s="2" t="inlineStr">
         <is>
-          <t>open_pelvis_impact</t>
+          <t>pelvis_open_p7</t>
         </is>
       </c>
       <c r="F50" s="2" t="inlineStr">
@@ -2035,7 +2036,7 @@
       </c>
       <c r="E51" s="2" t="inlineStr">
         <is>
-          <t>hands_too_close</t>
+          <t>hand_distance_close_p7</t>
         </is>
       </c>
       <c r="F51" s="2" t="inlineStr">
@@ -2063,7 +2064,7 @@
       <c r="D52" s="2" t="inlineStr"/>
       <c r="E52" s="2" t="inlineStr">
         <is>
-          <t>hands_too_close</t>
+          <t>hand_distance_close_p7</t>
         </is>
       </c>
       <c r="F52" s="2" t="inlineStr">
@@ -2095,7 +2096,7 @@
       </c>
       <c r="E53" s="2" t="inlineStr">
         <is>
-          <t>hands_too_close</t>
+          <t>hand_distance_close_p7</t>
         </is>
       </c>
       <c r="F53" s="2" t="inlineStr">
@@ -2127,8 +2128,8 @@
       </c>
       <c r="E54" s="2" t="inlineStr">
         <is>
-          <t>hands_too_close
-chicken_wing</t>
+          <t>hand_distance_close_p7
+chicken_wing_p7</t>
         </is>
       </c>
       <c r="F54" s="2" t="inlineStr">
@@ -2160,7 +2161,7 @@
       </c>
       <c r="E55" s="2" t="inlineStr">
         <is>
-          <t>hands_too_close</t>
+          <t>hand_distance_close_p7</t>
         </is>
       </c>
       <c r="F55" s="2" t="inlineStr">
@@ -2192,7 +2193,7 @@
       </c>
       <c r="E56" s="2" t="inlineStr">
         <is>
-          <t>hands_too_close</t>
+          <t>hand_distance_close_p7</t>
         </is>
       </c>
       <c r="F56" s="2" t="inlineStr">
@@ -2224,7 +2225,7 @@
       </c>
       <c r="E57" s="2" t="inlineStr">
         <is>
-          <t>hands_too_far</t>
+          <t>hand_distance_far_p7</t>
         </is>
       </c>
       <c r="F57" s="2" t="inlineStr">
@@ -2252,7 +2253,7 @@
       <c r="D58" s="2" t="inlineStr"/>
       <c r="E58" s="2" t="inlineStr">
         <is>
-          <t>hands_too_far</t>
+          <t>hand_distance_far_p7</t>
         </is>
       </c>
       <c r="F58" s="2" t="inlineStr">
@@ -2284,7 +2285,7 @@
       </c>
       <c r="E59" s="2" t="inlineStr">
         <is>
-          <t>hands_too_far</t>
+          <t>hand_distance_far_p7</t>
         </is>
       </c>
       <c r="F59" s="2" t="inlineStr">
@@ -2312,7 +2313,7 @@
       <c r="D60" s="2" t="inlineStr"/>
       <c r="E60" s="2" t="inlineStr">
         <is>
-          <t>hands_too_far</t>
+          <t>hand_distance_far_p7</t>
         </is>
       </c>
       <c r="F60" s="2" t="inlineStr">
@@ -2344,7 +2345,7 @@
       </c>
       <c r="E61" s="2" t="inlineStr">
         <is>
-          <t>hands_too_far</t>
+          <t>hand_distance_far_p7</t>
         </is>
       </c>
       <c r="F61" s="2" t="inlineStr">
@@ -2372,7 +2373,7 @@
       <c r="D62" s="2" t="inlineStr"/>
       <c r="E62" s="2" t="inlineStr">
         <is>
-          <t>chicken_wing</t>
+          <t>chicken_wing_p7</t>
         </is>
       </c>
       <c r="F62" s="2" t="inlineStr">
@@ -2400,7 +2401,7 @@
       <c r="D63" s="2" t="inlineStr"/>
       <c r="E63" s="2" t="inlineStr">
         <is>
-          <t>standing_up</t>
+          <t>standing_up_p7</t>
         </is>
       </c>
       <c r="F63" s="2" t="inlineStr">
@@ -2428,7 +2429,7 @@
       <c r="D64" s="2" t="inlineStr"/>
       <c r="E64" s="2" t="inlineStr">
         <is>
-          <t>open_pelvis_impact</t>
+          <t>pelvis_open_p7</t>
         </is>
       </c>
       <c r="F64" s="2" t="inlineStr">
@@ -2456,7 +2457,7 @@
       <c r="D65" s="2" t="inlineStr"/>
       <c r="E65" s="2" t="inlineStr">
         <is>
-          <t>open_thorax_impact</t>
+          <t>thorax_open_p7</t>
         </is>
       </c>
       <c r="F65" s="2" t="inlineStr">
@@ -2484,7 +2485,7 @@
       <c r="D66" s="2" t="inlineStr"/>
       <c r="E66" s="2" t="inlineStr">
         <is>
-          <t>chicken_wing</t>
+          <t>chicken_wing_p7</t>
         </is>
       </c>
       <c r="F66" s="2" t="inlineStr">
@@ -2517,7 +2518,7 @@
       </c>
       <c r="E67" s="2" t="inlineStr">
         <is>
-          <t>chicken_wing</t>
+          <t>chicken_wing_p7</t>
         </is>
       </c>
       <c r="F67" s="2" t="inlineStr">
@@ -2545,7 +2546,7 @@
       <c r="D68" s="2" t="inlineStr"/>
       <c r="E68" s="2" t="inlineStr">
         <is>
-          <t>chicken_wing</t>
+          <t>chicken_wing_p7</t>
         </is>
       </c>
       <c r="F68" s="2" t="inlineStr">
@@ -2573,7 +2574,7 @@
       <c r="D69" s="2" t="inlineStr"/>
       <c r="E69" s="2" t="inlineStr">
         <is>
-          <t>chicken_wing</t>
+          <t>chicken_wing_p7</t>
         </is>
       </c>
       <c r="F69" s="2" t="inlineStr">
@@ -2605,7 +2606,7 @@
       </c>
       <c r="E70" s="2" t="inlineStr">
         <is>
-          <t>chicken_wing</t>
+          <t>chicken_wing_p7</t>
         </is>
       </c>
       <c r="F70" s="2" t="inlineStr">
@@ -2633,7 +2634,7 @@
       <c r="D71" s="2" t="inlineStr"/>
       <c r="E71" s="2" t="inlineStr">
         <is>
-          <t>chicken_wing</t>
+          <t>chicken_wing_p7</t>
         </is>
       </c>
       <c r="F71" s="2" t="inlineStr">
@@ -2661,7 +2662,7 @@
       <c r="D72" s="2" t="inlineStr"/>
       <c r="E72" s="2" t="inlineStr">
         <is>
-          <t>standing_up</t>
+          <t>standing_up_p7</t>
         </is>
       </c>
       <c r="F72" s="2" t="inlineStr">
@@ -2689,7 +2690,7 @@
       <c r="D73" s="2" t="inlineStr"/>
       <c r="E73" s="2" t="inlineStr">
         <is>
-          <t>standing_up</t>
+          <t>standing_up_p7</t>
         </is>
       </c>
       <c r="F73" s="2" t="inlineStr">
@@ -2721,7 +2722,7 @@
       </c>
       <c r="E74" s="2" t="inlineStr">
         <is>
-          <t>standing_up</t>
+          <t>standing_up_p7</t>
         </is>
       </c>
       <c r="F74" s="2" t="inlineStr">
@@ -2749,7 +2750,7 @@
       <c r="D75" s="2" t="inlineStr"/>
       <c r="E75" s="2" t="inlineStr">
         <is>
-          <t>standing_up</t>
+          <t>standing_up_p7</t>
         </is>
       </c>
       <c r="F75" s="2" t="inlineStr">
@@ -2777,7 +2778,7 @@
       <c r="D76" s="2" t="inlineStr"/>
       <c r="E76" s="2" t="inlineStr">
         <is>
-          <t>standing_up</t>
+          <t>standing_up_p7</t>
         </is>
       </c>
       <c r="F76" s="2" t="inlineStr">
@@ -2809,7 +2810,7 @@
       </c>
       <c r="E77" s="2" t="inlineStr">
         <is>
-          <t>standing_up</t>
+          <t>standing_up_p7</t>
         </is>
       </c>
       <c r="F77" s="2" t="inlineStr">
@@ -2841,7 +2842,7 @@
       </c>
       <c r="E78" s="2" t="inlineStr">
         <is>
-          <t>standing_up</t>
+          <t>standing_up_p7</t>
         </is>
       </c>
       <c r="F78" s="2" t="inlineStr">
@@ -2873,7 +2874,7 @@
       </c>
       <c r="E79" s="2" t="inlineStr">
         <is>
-          <t>standing_up</t>
+          <t>standing_up_p7</t>
         </is>
       </c>
       <c r="F79" s="2" t="inlineStr">
@@ -2901,7 +2902,7 @@
       <c r="D80" s="2" t="inlineStr"/>
       <c r="E80" s="2" t="inlineStr">
         <is>
-          <t>forward_bend_excessive</t>
+          <t>forward_bend_excessive_p7</t>
         </is>
       </c>
       <c r="F80" s="2" t="inlineStr">
@@ -2929,7 +2930,7 @@
       <c r="D81" s="2" t="inlineStr"/>
       <c r="E81" s="2" t="inlineStr">
         <is>
-          <t>forward_bend_excessive</t>
+          <t>forward_bend_excessive_p7</t>
         </is>
       </c>
       <c r="F81" s="2" t="inlineStr">
@@ -2961,7 +2962,7 @@
       </c>
       <c r="E82" s="2" t="inlineStr">
         <is>
-          <t>forward_bend_excessive</t>
+          <t>forward_bend_excessive_p7</t>
         </is>
       </c>
       <c r="F82" s="2" t="inlineStr">
@@ -2989,7 +2990,7 @@
       <c r="D83" s="2" t="inlineStr"/>
       <c r="E83" s="2" t="inlineStr">
         <is>
-          <t>forward_bend_excessive</t>
+          <t>forward_bend_excessive_p7</t>
         </is>
       </c>
       <c r="F83" s="2" t="inlineStr">
@@ -3022,7 +3023,7 @@
       </c>
       <c r="E84" s="2" t="inlineStr">
         <is>
-          <t>side_bend_excessive</t>
+          <t>side_bend_excessive_p7</t>
         </is>
       </c>
       <c r="F84" s="2" t="inlineStr">
@@ -3055,7 +3056,7 @@
       </c>
       <c r="E85" s="2" t="inlineStr">
         <is>
-          <t>side_bend_excessive</t>
+          <t>side_bend_excessive_p7</t>
         </is>
       </c>
       <c r="F85" s="2" t="inlineStr">
@@ -3088,7 +3089,7 @@
       </c>
       <c r="E86" s="2" t="inlineStr">
         <is>
-          <t>side_bend_excessive</t>
+          <t>side_bend_excessive_p7</t>
         </is>
       </c>
       <c r="F86" s="2" t="inlineStr">
@@ -3116,8 +3117,8 @@
       <c r="D87" s="2" t="inlineStr"/>
       <c r="E87" s="2" t="inlineStr">
         <is>
-          <t>open_pelvis_impact
-side_bend_excessive</t>
+          <t>pelvis_open_p7
+side_bend_excessive_p7</t>
         </is>
       </c>
       <c r="F87" s="2" t="inlineStr">
@@ -3149,7 +3150,7 @@
       </c>
       <c r="E88" s="2" t="inlineStr">
         <is>
-          <t>side_bend_excessive</t>
+          <t>side_bend_excessive_p7</t>
         </is>
       </c>
       <c r="F88" s="2" t="inlineStr">
@@ -3181,7 +3182,7 @@
       </c>
       <c r="E89" s="2" t="inlineStr">
         <is>
-          <t>side_bend_excessive</t>
+          <t>side_bend_excessive_p7</t>
         </is>
       </c>
       <c r="F89" s="2" t="inlineStr">
@@ -3213,7 +3214,7 @@
       </c>
       <c r="E90" s="2" t="inlineStr">
         <is>
-          <t>side_bend_excessive</t>
+          <t>side_bend_excessive_p7</t>
         </is>
       </c>
       <c r="F90" s="2" t="inlineStr">
@@ -3245,7 +3246,7 @@
       </c>
       <c r="E91" s="2" t="inlineStr">
         <is>
-          <t>open_thorax_impact</t>
+          <t>thorax_open_p7</t>
         </is>
       </c>
       <c r="F91" s="2" t="inlineStr">
@@ -3277,8 +3278,8 @@
       </c>
       <c r="E92" s="2" t="inlineStr">
         <is>
-          <t>open_pelvis_impact
-side_bend_excessive</t>
+          <t>pelvis_open_p7
+side_bend_excessive_p7</t>
         </is>
       </c>
       <c r="F92" s="2" t="inlineStr">
@@ -3310,7 +3311,7 @@
       </c>
       <c r="E93" s="2" t="inlineStr">
         <is>
-          <t>closed_pelvis_impact</t>
+          <t>pelvis_closed_p7</t>
         </is>
       </c>
       <c r="F93" s="2" t="inlineStr">
@@ -3343,8 +3344,8 @@
       </c>
       <c r="E94" s="2" t="inlineStr">
         <is>
-          <t>open_pelvis_impact
-open_thorax_impact</t>
+          <t>pelvis_open_p7
+thorax_open_p7</t>
         </is>
       </c>
       <c r="F94" s="2" t="inlineStr">
@@ -3376,7 +3377,7 @@
       </c>
       <c r="E95" s="2" t="inlineStr">
         <is>
-          <t>open_pelvis_impact</t>
+          <t>pelvis_open_p7</t>
         </is>
       </c>
       <c r="F95" s="2" t="inlineStr">
@@ -3408,7 +3409,7 @@
       </c>
       <c r="E96" s="2" t="inlineStr">
         <is>
-          <t>club_face_open_impact</t>
+          <t>club_face_open_p7</t>
         </is>
       </c>
       <c r="F96" s="2" t="inlineStr">
@@ -3441,8 +3442,8 @@
       </c>
       <c r="E97" s="2" t="inlineStr">
         <is>
-          <t>club_face_closed_impact
-closed_pelvis_impact</t>
+          <t>club_face_closed_p7
+pelvis_closed_p7</t>
         </is>
       </c>
       <c r="F97" s="2" t="inlineStr">
@@ -3474,7 +3475,7 @@
       </c>
       <c r="E98" s="2" t="inlineStr">
         <is>
-          <t>club_face_closed_impact</t>
+          <t>club_face_closed_p7</t>
         </is>
       </c>
       <c r="F98" s="2" t="inlineStr">
@@ -3506,7 +3507,7 @@
       </c>
       <c r="E99" s="2" t="inlineStr">
         <is>
-          <t>club_face_closed_impact</t>
+          <t>club_face_closed_p7</t>
         </is>
       </c>
       <c r="F99" s="2" t="inlineStr">
@@ -3538,7 +3539,7 @@
       </c>
       <c r="E100" s="2" t="inlineStr">
         <is>
-          <t>club_face_closed_impact</t>
+          <t>club_face_closed_p7</t>
         </is>
       </c>
       <c r="F100" s="2" t="inlineStr">
@@ -3570,7 +3571,7 @@
       </c>
       <c r="E101" s="2" t="inlineStr">
         <is>
-          <t>chicken_wing</t>
+          <t>chicken_wing_p7</t>
         </is>
       </c>
       <c r="F101" s="2" t="inlineStr">
@@ -3602,7 +3603,7 @@
       </c>
       <c r="E102" s="2" t="inlineStr">
         <is>
-          <t>hands_too_far</t>
+          <t>hand_distance_far_p7</t>
         </is>
       </c>
       <c r="F102" s="2" t="inlineStr">
@@ -3634,7 +3635,7 @@
       </c>
       <c r="E103" s="2" t="inlineStr">
         <is>
-          <t>standing_up</t>
+          <t>standing_up_p7</t>
         </is>
       </c>
       <c r="F103" s="2" t="inlineStr">
@@ -3666,7 +3667,7 @@
       </c>
       <c r="E104" s="2" t="inlineStr">
         <is>
-          <t>lead_pressure_excessive_impact</t>
+          <t>lead_pressure_excessive_p7</t>
         </is>
       </c>
       <c r="F104" s="2" t="inlineStr">
@@ -3698,7 +3699,7 @@
       </c>
       <c r="E105" s="2" t="inlineStr">
         <is>
-          <t>chicken_wing</t>
+          <t>chicken_wing_p7</t>
         </is>
       </c>
       <c r="F105" s="2" t="inlineStr">
@@ -3726,7 +3727,7 @@
       <c r="D106" s="2" t="inlineStr"/>
       <c r="E106" s="2" t="inlineStr">
         <is>
-          <t>forward_hands</t>
+          <t>hand_direction_forward_p7</t>
         </is>
       </c>
       <c r="F106" s="2" t="inlineStr">
@@ -3754,7 +3755,7 @@
       <c r="D107" s="2" t="inlineStr"/>
       <c r="E107" s="2" t="inlineStr">
         <is>
-          <t>forward_hands</t>
+          <t>hand_direction_forward_p7</t>
         </is>
       </c>
       <c r="F107" s="2" t="inlineStr">
@@ -3782,7 +3783,7 @@
       <c r="D108" s="2" t="inlineStr"/>
       <c r="E108" s="2" t="inlineStr">
         <is>
-          <t>closed_pelvis_impact</t>
+          <t>pelvis_closed_p7</t>
         </is>
       </c>
       <c r="F108" s="2" t="inlineStr">
@@ -3802,7 +3803,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G23"/>
+  <dimension ref="A1:G17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -3854,12 +3855,12 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>forward_hands</t>
+          <t>hand_direction_forward_p7</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Forward Hands</t>
+          <t>Hand Direction Forward (P7)</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
@@ -3891,12 +3892,12 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>club_face_open_impact</t>
+          <t>club_face_open_p7</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Club Face Open (Impact)</t>
+          <t>Club Face Open (P7)</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
@@ -3928,12 +3929,12 @@
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>club_face_closed_impact</t>
+          <t>club_face_closed_p7</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>Club Face Closed (Impact)</t>
+          <t>Club Face Closed (P7)</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
@@ -3965,12 +3966,12 @@
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>open_pelvis_impact</t>
+          <t>pelvis_open_p7</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>Open Pelvis At Impact</t>
+          <t>Pelvis Open (P7)</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
@@ -4002,12 +4003,12 @@
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>closed_pelvis_impact</t>
+          <t>pelvis_closed_p7</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>Closed Pelvis At Impact</t>
+          <t>Pelvis Closed (P7)</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
@@ -4017,7 +4018,7 @@
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>임팩트(P7) 순간 골반이 기준보다 목표 방향으로 충분히 회전하지 못한 상태. 골반 회전량만 관찰. Open Pelvis의 단순 반대가 아니라 독립 생성 메커니즘을 가진다. Closed는 Target Line 기준.</t>
+          <t>임팩트(P7) 순간 골반이 기준보다 목표 방향으로 충분히 회전하지 못한 상태. 골반 회전량만 관찰. Pelvis Open (P7)의 단순 반대가 아니라 독립 생성 메커니즘을 가진다. Closed는 Target Line 기준.</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr">
@@ -4039,12 +4040,12 @@
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>open_thorax_impact</t>
+          <t>thorax_open_p7</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>Open Thorax At Impact</t>
+          <t>Thorax Open (P7)</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
@@ -4076,12 +4077,12 @@
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>closed_thorax_impact</t>
+          <t>thorax_closed_p7</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>Closed Thorax At Impact</t>
+          <t>Thorax Closed (P7)</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
@@ -4113,12 +4114,12 @@
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>standing_up</t>
+          <t>standing_up_p7</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>Standing Up</t>
+          <t>Standing Up (P7)</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
@@ -4143,19 +4144,19 @@
       </c>
       <c r="G9" s="2" t="inlineStr">
         <is>
-          <t>임팩트 반경(Radius) 불안정 Hub. [Ref: 척추각/몸통 높이]</t>
+          <t>Pattern Feature(명칭 유지). 임팩트 반경(Radius) 불안정 Hub. [Ref: 척추각/몸통 높이]</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>forward_bend_excessive</t>
+          <t>forward_bend_excessive_p7</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>Excessive Forward Bend</t>
+          <t>Forward Bend Excessive (P7)</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
@@ -4187,12 +4188,12 @@
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>side_bend_excessive</t>
+          <t>side_bend_excessive_p7</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>Excessive Side Bend</t>
+          <t>Side Bend Excessive (P7)</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
@@ -4224,12 +4225,12 @@
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>lead_pressure_excessive_impact</t>
+          <t>lead_pressure_excessive_p7</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>Excessive Lead Pressure</t>
+          <t>Lead Pressure Excessive (P7)</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
@@ -4261,12 +4262,12 @@
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>hands_too_close</t>
+          <t>hand_distance_close_p7</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>Hands Too Close To Body</t>
+          <t>Hand Distance Close (P7)</t>
         </is>
       </c>
       <c r="C13" s="2" t="inlineStr">
@@ -4298,12 +4299,12 @@
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>hands_too_far</t>
+          <t>hand_distance_far_p7</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>Hands Too Far From Body</t>
+          <t>Hand Distance Far (P7)</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
@@ -4335,12 +4336,12 @@
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>chicken_wing</t>
+          <t>chicken_wing_p7</t>
         </is>
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>Chicken Wing</t>
+          <t>Chicken Wing (P7)</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
@@ -4365,19 +4366,19 @@
       </c>
       <c r="G15" s="2" t="inlineStr">
         <is>
-          <t>회전 부족·분절 시퀀스 이상의 대표 보상. Path+Face 동시 변화 Hub.</t>
+          <t>Pattern Feature(명칭 유지). 회전 부족·분절 시퀀스 이상의 대표 보상. Path+Face 동시 변화 Hub.</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>lead_wrist_flexion</t>
+          <t>lead_wrist_flexion_p7</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>Lead Wrist Flexion</t>
+          <t>Lead Wrist Flexion (P7)</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr">
@@ -4409,12 +4410,12 @@
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>lead_wrist_extension</t>
+          <t>lead_wrist_extension_p7</t>
         </is>
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>Lead Wrist Extension</t>
+          <t>Lead Wrist Extension (P7)</t>
         </is>
       </c>
       <c r="C17" s="2" t="inlineStr">
@@ -4440,228 +4441,6 @@
       <c r="G17" s="2" t="inlineStr">
         <is>
           <t>5-섹션 템플릿(원인/이후 없음). Context-dependent.</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="2" t="inlineStr">
-        <is>
-          <t>swing_path_out_to_in</t>
-        </is>
-      </c>
-      <c r="B18" s="2" t="inlineStr">
-        <is>
-          <t>Out-To-In Swing Path</t>
-        </is>
-      </c>
-      <c r="C18" s="2" t="inlineStr">
-        <is>
-          <t>아웃투인 스윙패스</t>
-        </is>
-      </c>
-      <c r="D18" s="2" t="inlineStr">
-        <is>
-          <t>클럽 헤드 경로가 목표선 기준 바깥→안쪽으로 진행되는 전달 방향. 임팩트 Path Observation.</t>
-        </is>
-      </c>
-      <c r="E18" s="2" t="inlineStr">
-        <is>
-          <t>Club Path</t>
-        </is>
-      </c>
-      <c r="F18" s="2" t="inlineStr">
-        <is>
-          <t>Candidate Observation</t>
-        </is>
-      </c>
-      <c r="G18" s="2" t="inlineStr">
-        <is>
-          <t>P7 Core 미포함. 원인↔결과 연결 중간 Observation. P1~P8 완료 후 승격/Layer 결정.</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="2" t="inlineStr">
-        <is>
-          <t>swing_path_in_to_out</t>
-        </is>
-      </c>
-      <c r="B19" s="2" t="inlineStr">
-        <is>
-          <t>In-To-Out Swing Path</t>
-        </is>
-      </c>
-      <c r="C19" s="2" t="inlineStr">
-        <is>
-          <t>인투아웃 스윙패스</t>
-        </is>
-      </c>
-      <c r="D19" s="2" t="inlineStr">
-        <is>
-          <t>클럽 헤드 경로가 목표선 기준 안쪽→바깥쪽으로 진행되는 전달 방향. 임팩트 Path Observation.</t>
-        </is>
-      </c>
-      <c r="E19" s="2" t="inlineStr">
-        <is>
-          <t>Club Path</t>
-        </is>
-      </c>
-      <c r="F19" s="2" t="inlineStr">
-        <is>
-          <t>Candidate Observation</t>
-        </is>
-      </c>
-      <c r="G19" s="2" t="inlineStr">
-        <is>
-          <t>P7 Core 미포함. Excessive In-To-Out 포함. 중간 Observation.</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="2" t="inlineStr">
-        <is>
-          <t>late_face_closure</t>
-        </is>
-      </c>
-      <c r="B20" s="2" t="inlineStr">
-        <is>
-          <t>Late Face Closure</t>
-        </is>
-      </c>
-      <c r="C20" s="2" t="inlineStr">
-        <is>
-          <t>늦은 페이스 클로징</t>
-        </is>
-      </c>
-      <c r="D20" s="2" t="inlineStr">
-        <is>
-          <t>임팩트 직전 손 사용을 급격히 증가시켜 페이스를 닫으려는 늦은 보상 동작.</t>
-        </is>
-      </c>
-      <c r="E20" s="2" t="inlineStr">
-        <is>
-          <t>Club</t>
-        </is>
-      </c>
-      <c r="F20" s="2" t="inlineStr">
-        <is>
-          <t>Candidate Feature</t>
-        </is>
-      </c>
-      <c r="G20" s="2" t="inlineStr">
-        <is>
-          <t>향후 독립 Feature 발전 가능. 현재 Chain 참조 노드.</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="2" t="inlineStr">
-        <is>
-          <t>trail_elbow_out</t>
-        </is>
-      </c>
-      <c r="B21" s="2" t="inlineStr">
-        <is>
-          <t>Trail Elbow Out</t>
-        </is>
-      </c>
-      <c r="C21" s="2" t="inlineStr">
-        <is>
-          <t>트레일 팔꿈치 벌어짐</t>
-        </is>
-      </c>
-      <c r="D21" s="2" t="inlineStr">
-        <is>
-          <t>임팩트 구간에서 트레일 팔꿈치가 몸통에서 과도하게 벌어지는 현상.</t>
-        </is>
-      </c>
-      <c r="E21" s="2" t="inlineStr">
-        <is>
-          <t>Trail Elbow</t>
-        </is>
-      </c>
-      <c r="F21" s="2" t="inlineStr">
-        <is>
-          <t>Candidate Feature</t>
-        </is>
-      </c>
-      <c r="G21" s="2" t="inlineStr">
-        <is>
-          <t>향후 독립 Feature 발전 가능. Open Pelvis 결과 Chain에서 관찰.</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="2" t="inlineStr">
-        <is>
-          <t>lead_arm_against_chest</t>
-        </is>
-      </c>
-      <c r="B22" s="2" t="inlineStr">
-        <is>
-          <t>Lead Arm Against Chest</t>
-        </is>
-      </c>
-      <c r="C22" s="2" t="inlineStr">
-        <is>
-          <t>리드암 가슴 밀착</t>
-        </is>
-      </c>
-      <c r="D22" s="2" t="inlineStr">
-        <is>
-          <t>(통합됨) 리드암이 가슴에 밀착되어 신전되지 못하는 현상.</t>
-        </is>
-      </c>
-      <c r="E22" s="2" t="inlineStr">
-        <is>
-          <t>Arm</t>
-        </is>
-      </c>
-      <c r="F22" s="2" t="inlineStr">
-        <is>
-          <t>Merged→chicken_wing</t>
-        </is>
-      </c>
-      <c r="G22" s="2" t="inlineStr">
-        <is>
-          <t>원칙 ⑨: 독립 Information Gain 없음 → Chicken Wing에 통합.</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" s="2" t="inlineStr">
-        <is>
-          <t>arm_dominant_pattern</t>
-        </is>
-      </c>
-      <c r="B23" s="2" t="inlineStr">
-        <is>
-          <t>Arm Dominant Pattern</t>
-        </is>
-      </c>
-      <c r="C23" s="2" t="inlineStr">
-        <is>
-          <t>팔 주도 패턴</t>
-        </is>
-      </c>
-      <c r="D23" s="2" t="inlineStr">
-        <is>
-          <t>(해석 개념) 몸 회전 대비 팔이 독립적으로 클럽 전달을 주도하는 종합 해석.</t>
-        </is>
-      </c>
-      <c r="E23" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F23" s="2" t="inlineStr">
-        <is>
-          <t>Coaching Knowledge</t>
-        </is>
-      </c>
-      <c r="G23" s="2" t="inlineStr">
-        <is>
-          <t>여러 Feature 종합 해석 → Feature 아님. Coaching Knowledge 시트로 관리.</t>
         </is>
       </c>
     </row>
@@ -4716,7 +4495,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>forward_hands</t>
+          <t>hand_direction_forward_p7</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
@@ -4743,7 +4522,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>club_face_open_impact</t>
+          <t>club_face_open_p7</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
@@ -4770,7 +4549,7 @@
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>club_face_closed_impact</t>
+          <t>club_face_closed_p7</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
@@ -4797,7 +4576,7 @@
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>open_pelvis_impact</t>
+          <t>pelvis_open_p7</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
@@ -4824,7 +4603,7 @@
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>closed_pelvis_impact</t>
+          <t>pelvis_closed_p7</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
@@ -4851,7 +4630,7 @@
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>open_thorax_impact</t>
+          <t>thorax_open_p7</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
@@ -4878,7 +4657,7 @@
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>closed_thorax_impact</t>
+          <t>thorax_closed_p7</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
@@ -4905,7 +4684,7 @@
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>standing_up</t>
+          <t>standing_up_p7</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
@@ -4932,7 +4711,7 @@
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>forward_bend_excessive</t>
+          <t>forward_bend_excessive_p7</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
@@ -4959,7 +4738,7 @@
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>side_bend_excessive</t>
+          <t>side_bend_excessive_p7</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
@@ -4986,7 +4765,7 @@
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>lead_pressure_excessive_impact</t>
+          <t>lead_pressure_excessive_p7</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
@@ -5013,7 +4792,7 @@
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>hands_too_close</t>
+          <t>hand_distance_close_p7</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
@@ -5040,7 +4819,7 @@
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>hands_too_far</t>
+          <t>hand_distance_far_p7</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
@@ -5067,7 +4846,7 @@
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>chicken_wing</t>
+          <t>chicken_wing_p7</t>
         </is>
       </c>
       <c r="B15" s="2" t="inlineStr">
@@ -5094,7 +4873,7 @@
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>lead_wrist_flexion</t>
+          <t>lead_wrist_flexion_p7</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
@@ -5121,7 +4900,7 @@
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>lead_wrist_extension</t>
+          <t>lead_wrist_extension_p7</t>
         </is>
       </c>
       <c r="B17" s="2" t="inlineStr">
@@ -5156,7 +4935,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B32"/>
+  <dimension ref="A1:B47"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -5214,292 +4993,456 @@
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>② P7 명명 표기</t>
+          <t>② Feature Naming Rule (통일·LOCK)</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>P7은 Observation Timing이 정의의 일부이므로 P6의 [Object]+[Attribute] 어순을 강제하지 않는다. 초안 표기(예: Open Pelvis At Impact, Closed Thorax At Impact)를 표시명으로 유지한다. 단, 동일 의미는 항상 동일 표현을 사용하고, 새 표현이 필요하면 Dictionary에 먼저 등록한 뒤 전 문서에서 일관 재사용한다.</t>
+          <t>모든 Feature는 [Object] [Attribute] (Phase) 형식으로 명명한다. Phase 태그로 동일 관찰의 Phase 차이를 구분한다. 예) Pelvis Open (P7) · Pelvis Open (P4) · Thorax Open (P7) · Club Face Open (P7) · Lead Pressure Excessive (P7) · Club Path Out-To-In (P7) · Hand Depth Deep (P4) · Hand Distance Close (P7) · Hand Direction Forward (P7). Attribute는 같은 단어를 반복 사용하고 새 표현은 최소화한다. 동일 의미는 항상 동일 이름, 새 이름이 필요하면 Dictionary에 먼저 등록 후 전 문서 일관 재사용.</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>③ Coordinate System(절대 유지)</t>
+          <t>②-예외 Pattern Feature</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>모든 위치 표현은 DOH Coordinate System 기준을 명시한다. Forward→Ball/Target Line · Open/Closed→Target Line · Near(Close)/Far→Torso · Deep→Thorax · Height(High/Low)→척추각/몸통 높이. 기준이 불명확한 표현은 사용하지 않는다.</t>
+          <t>관용화된 패턴명(Standing Up, Chicken Wing)은 명칭을 유지하고 (Phase)만 붙인다. P6 선례: Spin-out · Early Extension · Casting.</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>④ Modifier Feature 구분</t>
+          <t>②-Hand Position Axes</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>Lead Wrist Flexion/Extension 등은 독립 Problem Feature가 아니라 다른 Feature를 해석하는 Modifier Feature다. 템플릿을 달리한다(정의/Modifier 특성/대표 해석 사례/관련 Feature/사고확장의 5-섹션, 원인·이후·Strong Co-occurrence 없음).</t>
+          <t>손 위치 Feature는 축(Axis) 단어를 포함한다. Depth(Deep/Shallow)→Thorax · Height(High/Low) · Distance(Close/Far)→Torso · Direction(Forward/Backward)→Ball/Target Line. 예) Hand Depth Deep · Hand Distance Close · Hand Direction Forward.</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>⑤ Coaching Knowledge 분리</t>
+          <t>③ Coordinate System(절대 유지)</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>레슨 경험·잘못된 움직임 이미지·그립별 손목 해석·조건부 해석은 Feature에 쓰지 않고 'DOH Coaching Knowledge' 시트에 기록한다.</t>
+          <t>모든 위치 표현은 DOH Coordinate System 기준을 명시한다. Forward→Ball/Target Line · Open/Closed→Target Line · Near(Close)/Far→Torso · Deep→Thorax · Height(High/Low)→척추각/몸통 높이. 기준이 불명확한 표현은 사용하지 않는다.</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>⑥ Evidence Layer 분리</t>
+          <t>④ Modifier Feature 구분</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>Ball Flight·Impact Strike·Ground Contact는 Feature도 Outcome도 아닌 Evidence Layer다. 회원이 인지·입력하는 정보로, AI가 Feature를 역추론하는 근거다. 'Evidence Layer' 참조 시트로 관리하고, 각 Feature 우측 Evidence Matrix로 연결한다(별점은 후속 작업).</t>
+          <t>Lead Wrist Flexion/Extension 등은 독립 Problem Feature가 아니라 다른 Feature를 해석하는 Modifier Feature다. 템플릿을 달리한다(정의/Modifier 특성/대표 해석 사례/관련 Feature/사고확장의 5-섹션, 원인·이후·Strong Co-occurrence 없음).</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>⑦ Branch Chain</t>
+          <t>⑤ Coaching Knowledge 분리</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>동일 Feature라도 보상 전략에 따라 이후 Chain이 분기하면 단일 결과로 단정하지 않고 Branch Chain으로 작성한다.</t>
+          <t>레슨 경험·잘못된 움직임 이미지·그립별 손목 해석·조건부 해석은 Feature에 쓰지 않고 'DOH Coaching Knowledge' 시트에 기록한다.</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>⑧ Confidence 등급</t>
+          <t>⑥ Evidence Layer 분리</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>[High Confidence]=생체역학적으로 확실 · [Medium Confidence]=레슨상 자주 · [Low Confidence / Pattern Dependent] 또는 ※추론=특정 유형. 원인/이후 Chain에 등급을 명시한다.</t>
+          <t>Ball Flight·Impact Strike·Ground Contact는 Feature도 Outcome도 아닌 Evidence Layer다. 회원이 인지·입력하는 정보로, AI가 Feature를 역추론하는 근거다. 'Evidence Layer' 참조 시트로 관리하고, 각 Feature 우측 Evidence Matrix로 연결한다(별점은 후속 작업).</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>⑨ Feature 신설 3원칙</t>
+          <t>⑦ Branch Chain</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>새 Feature는 ①Observation이 다른가 ②새 Chain을 생성하는가 ③새 추론 정보(Information Gain)를 주는가 를 모두 만족할 때만 만든다. 아니면 기존 Feature 통합을 우선한다. 애매하면 임의 결정 없이 질문 후 진행한다.</t>
+          <t>동일 Feature라도 보상 전략에 따라 이후 Chain이 분기하면 단일 결과로 단정하지 않고 Branch Chain으로 작성한다.</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="2" t="inlineStr"/>
-      <c r="B14" s="2" t="inlineStr"/>
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>⑧ Confidence 등급</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>[High Confidence]=생체역학적으로 확실 · [Medium Confidence]=레슨상 자주 · [Low Confidence / Pattern Dependent] 또는 ※추론=특정 유형. 원인/이후 Chain에 등급을 명시한다.</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>Coordinate Reference Vocabulary</t>
-        </is>
-      </c>
-      <c r="B15" s="2" t="inlineStr"/>
+          <t>⑨ Feature 신설 3원칙</t>
+        </is>
+      </c>
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t>새 Feature는 ①Observation이 다른가 ②새 Chain을 생성하는가 ③새 추론 정보(Information Gain)를 주는가 를 모두 만족할 때만 만든다. 아니면 기존 Feature 통합을 우선한다. 애매하면 임의 결정 없이 질문 후 진행한다.</t>
+        </is>
+      </c>
     </row>
     <row r="16">
-      <c r="A16" s="2" t="inlineStr">
-        <is>
-          <t>Forward / Backward</t>
-        </is>
-      </c>
-      <c r="B16" s="2" t="inlineStr">
-        <is>
-          <t>Ball / Target Line 기준</t>
-        </is>
-      </c>
+      <c r="A16" s="2" t="inlineStr"/>
+      <c r="B16" s="2" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>Open / Closed</t>
-        </is>
-      </c>
-      <c r="B17" s="2" t="inlineStr">
-        <is>
-          <t>Target Line 기준</t>
-        </is>
-      </c>
+          <t>Coordinate Reference Vocabulary</t>
+        </is>
+      </c>
+      <c r="B17" s="2" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>Near(Close) / Far</t>
+          <t>Forward / Backward</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>Torso 기준</t>
+          <t>Ball / Target Line 기준</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>Deep / Shallow</t>
+          <t>Open / Closed</t>
         </is>
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>Thorax 기준</t>
+          <t>Target Line 기준</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>High / Low (Height)</t>
+          <t>Near(Close) / Far</t>
         </is>
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>척추각 / 몸통 높이 기준</t>
+          <t>Torso 기준</t>
         </is>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="2" t="inlineStr"/>
-      <c r="B21" s="2" t="inlineStr"/>
+      <c r="A21" s="2" t="inlineStr">
+        <is>
+          <t>Deep / Shallow</t>
+        </is>
+      </c>
+      <c r="B21" s="2" t="inlineStr">
+        <is>
+          <t>Thorax 기준</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>Mechanism Categories (P7)</t>
-        </is>
-      </c>
-      <c r="B22" s="2" t="inlineStr"/>
+          <t>High / Low (Height)</t>
+        </is>
+      </c>
+      <c r="B22" s="2" t="inlineStr">
+        <is>
+          <t>척추각 / 몸통 높이 기준</t>
+        </is>
+      </c>
     </row>
     <row r="23">
-      <c r="A23" s="2" t="inlineStr">
-        <is>
-          <t>ROT</t>
-        </is>
-      </c>
-      <c r="B23" s="2" t="inlineStr">
-        <is>
-          <t>Rotation — 골반/흉곽 회전(Amount·Timing·Velocity·Axis)</t>
-        </is>
-      </c>
+      <c r="A23" s="2" t="inlineStr"/>
+      <c r="B23" s="2" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>PRS</t>
-        </is>
-      </c>
-      <c r="B24" s="2" t="inlineStr">
-        <is>
-          <t>Pressure — 리드/트레일 하중 및 압력 분포</t>
-        </is>
-      </c>
+          <t>Mechanism Categories (P7)</t>
+        </is>
+      </c>
+      <c r="B24" s="2" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>ARM</t>
+          <t>ROT</t>
         </is>
       </c>
       <c r="B25" s="2" t="inlineStr">
         <is>
-          <t>Arm Delivery — 팔·손·팔꿈치의 전달과 신전</t>
+          <t>Rotation — 골반/흉곽 회전(Amount·Timing·Velocity·Axis)</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>CLB</t>
+          <t>PRS</t>
         </is>
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t>Club Delivery — 페이스 방향·경로(Path)·릴리즈·로프트</t>
+          <t>Pressure — 리드/트레일 하중 및 압력 분포</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t>SPC</t>
+          <t>ARM</t>
         </is>
       </c>
       <c r="B27" s="2" t="inlineStr">
         <is>
-          <t>Space — 몸-팔 전달 공간 및 스윙 반경(Radius)</t>
+          <t>Arm Delivery — 팔·손·팔꿈치의 전달과 신전</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>LOD</t>
+          <t>CLB</t>
         </is>
       </c>
       <c r="B28" s="2" t="inlineStr">
         <is>
-          <t>Loading — 리드/트레일측 하중 수용과 안정</t>
+          <t>Club Delivery — 페이스 방향·경로(Path)·릴리즈·로프트</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
         <is>
-          <t>CMP</t>
+          <t>SPC</t>
         </is>
       </c>
       <c r="B29" s="2" t="inlineStr">
         <is>
-          <t>Compensation — 페이스·회전·손·몸의 보상 동작</t>
+          <t>Space — 몸-팔 전달 공간 및 스윙 반경(Radius)</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>PST</t>
+          <t>LOD</t>
         </is>
       </c>
       <c r="B30" s="2" t="inlineStr">
         <is>
-          <t>Posture / Axis — 척추각·측굴·전경·몸통 높이(신규, P7에서 신설)</t>
+          <t>Loading — 리드/트레일측 하중 수용과 안정</t>
         </is>
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="2" t="inlineStr"/>
-      <c r="B31" s="2" t="inlineStr"/>
+      <c r="A31" s="2" t="inlineStr">
+        <is>
+          <t>CMP</t>
+        </is>
+      </c>
+      <c r="B31" s="2" t="inlineStr">
+        <is>
+          <t>Compensation — 페이스·회전·손·몸의 보상 동작</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
+          <t>PST</t>
+        </is>
+      </c>
+      <c r="B32" s="2" t="inlineStr">
+        <is>
+          <t>Posture / Axis — 척추각·측굴·전경·몸통 높이(신규, P7에서 신설)</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="2" t="inlineStr"/>
+      <c r="B33" s="2" t="inlineStr"/>
+    </row>
+    <row r="34">
+      <c r="A34" s="2" t="inlineStr">
+        <is>
           <t>Player Type 태그(신규)</t>
         </is>
       </c>
-      <c r="B32" s="2" t="inlineStr">
-        <is>
-          <t>같은 Feature라도 생성 메커니즘이 선수/아마추어에서 다를 때 [Player Type: Amateur/Elite] 태그로 해석 맥락(Context)을 부여한다. Feature 자체는 바꾸지 않는다. (예: Excessive Side Bend)</t>
+      <c r="B34" s="2" t="inlineStr">
+        <is>
+          <t>같은 Feature라도 생성 메커니즘이 선수/아마추어에서 다를 때 [Player Type: Amateur/Elite] 태그로 해석 맥락(Context)을 부여한다. Feature 자체는 바꾸지 않는다. (예: Side Bend Excessive (P7))</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="2" t="inlineStr"/>
+      <c r="B35" s="2" t="inlineStr"/>
+    </row>
+    <row r="36">
+      <c r="A36" s="2" t="inlineStr">
+        <is>
+          <t>Role Taxonomy (DOH Object Roles)</t>
+        </is>
+      </c>
+      <c r="B36" s="2" t="inlineStr">
+        <is>
+          <t>역할을 명확히 분리한다. 규모가 커질수록 합치지 말고 유지한다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="2" t="inlineStr">
+        <is>
+          <t>Core Feature</t>
+        </is>
+      </c>
+      <c r="B37" s="2" t="inlineStr">
+        <is>
+          <t>독립적으로 관찰되는 문제/현상 Feature. 6-섹션 템플릿.</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="2" t="inlineStr">
+        <is>
+          <t>Modifier Feature</t>
+        </is>
+      </c>
+      <c r="B38" s="2" t="inlineStr">
+        <is>
+          <t>다른 Feature의 해석을 바꾸는 보조 Feature. 5-섹션 템플릿(원인/이후/Strong Co-occurrence 없음).</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="2" t="inlineStr">
+        <is>
+          <t>Setup Influence</t>
+        </is>
+      </c>
+      <c r="B39" s="2" t="inlineStr">
+        <is>
+          <t>P1 Setup에서 기원하는 영향 요인(예: Grip Strong/Weak). 후속 Phase에서 새로 만들지 않고 참조한다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="2" t="inlineStr">
+        <is>
+          <t>Coaching Knowledge</t>
+        </is>
+      </c>
+      <c r="B40" s="2" t="inlineStr">
+        <is>
+          <t>여러 Feature 종합 해석·레슨 이미지·조건부 지식(예: Arm Dominant Pattern). 별도 시트.</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="2" t="inlineStr">
+        <is>
+          <t>Candidate Concepts</t>
+        </is>
+      </c>
+      <c r="B41" s="2" t="inlineStr">
+        <is>
+          <t>Feature화가 애매한 개념. 'DOH Candidate Concepts' 시트에 선등록(Repeated 공백).</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="2" t="inlineStr">
+        <is>
+          <t>Biomechanical Concepts</t>
+        </is>
+      </c>
+      <c r="B42" s="2" t="inlineStr">
+        <is>
+          <t>생체역학 개념·Injury Risk 등(예: Lumbar Stress). Mechanism/Note로 관리.</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="2" t="inlineStr">
+        <is>
+          <t>Derived Parameters</t>
+        </is>
+      </c>
+      <c r="B43" s="2" t="inlineStr">
+        <is>
+          <t>계산·조합으로 산출되는 값(예: Dynamic Loft). 별도 시트.</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="2" t="inlineStr">
+        <is>
+          <t>PST</t>
+        </is>
+      </c>
+      <c r="B44" s="2" t="inlineStr">
+        <is>
+          <t>Posture/Axis Mechanism 카테고리(척추각·측굴·전경·몸통 높이). CMP와 합치지 않고 유지(LOCK).</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="2" t="inlineStr"/>
+      <c r="B45" s="2" t="inlineStr"/>
+    </row>
+    <row r="46">
+      <c r="A46" s="2" t="inlineStr">
+        <is>
+          <t>⑩ Candidate 우선 원칙</t>
+        </is>
+      </c>
+      <c r="B46" s="2" t="inlineStr">
+        <is>
+          <t>Stage 2 등 이후 작업에서 새 개념/Mechanism 구조/Knowledge Structure가 나오면 억지로 Feature를 만들지 말고 Candidate Concepts 시트에 먼저 등록한다. Definition·First Found·Status·Example만 작성하고 Repeated는 비워둔다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="2" t="inlineStr">
+        <is>
+          <t>⑪ Dictionary 수정 정책(LOCK)</t>
+        </is>
+      </c>
+      <c r="B47" s="2" t="inlineStr">
+        <is>
+          <t>현재 Dictionary는 유지. P1~P4 진행 중에는 '추가'만 하고 수정은 최소화한다. P4 완료 후 Dictionary Refactoring을 1회 일괄 수행한다.</t>
         </is>
       </c>
     </row>
@@ -5987,6 +5930,266 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:F17"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="26" customWidth="1" min="1" max="1"/>
+    <col width="52" customWidth="1" min="2" max="2"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
+    <col width="20" customWidth="1" min="4" max="4"/>
+    <col width="40" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Concept</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Definition</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>First Found</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Example</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Repeated</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Club Path Out-To-In (P7)</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>클럽 헤드 경로가 목표선 기준 바깥→안쪽으로 진행되는 전달 방향(Path Observation).</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>P7 (2026-07-08)</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>candidate-observation</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>Pelvis Open (P7) → Club Path Out-To-In (P7)</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr"/>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>Club Path In-To-Out (P7)</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>클럽 헤드 경로가 안쪽→바깥으로 진행되는 전달 방향. Excessive In-To-Out 포함.</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>P7 (2026-07-08)</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>candidate-observation</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>Thorax Closed (P7) → Club Path In-To-Out (P7)</t>
+        </is>
+      </c>
+      <c r="F3" s="2" t="inlineStr"/>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>Face Closure Late (P7)</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>임팩트 직전 손 사용을 급격히 증가시켜 페이스를 닫으려는 늦은 보상 동작.</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>P7 (2026-07-08)</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>candidate-feature</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>Club Face Open (P7) → Face Closure Late (P7)</t>
+        </is>
+      </c>
+      <c r="F4" s="2" t="inlineStr"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>Trail Elbow Out (P7)</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>임팩트 구간에서 트레일 팔꿈치가 몸통에서 과도하게 벌어지는 현상.</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>P7 (2026-07-08)</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>candidate-feature</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>Pelvis Open (P7) → Trail Elbow Out (P7)</t>
+        </is>
+      </c>
+      <c r="F5" s="2" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>Forward COM (P7)</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>임팩트에서 신체 무게중심(COM)이 전방(타깃 방향)으로 과도하게 이동한 상태.</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>P7 (2026-07-08)</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>candidate-feature</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>Forward COM (P7) → Hand Direction Forward (P7)</t>
+        </is>
+      </c>
+      <c r="F6" s="2" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="3" t="inlineStr">
+        <is>
+          <t>── DOH Candidate Concepts 운영 규칙 ──</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>Stage 2 작업 중 새로운 Feature를 만들기 애매한 개념 / 새로운 Mechanism 구조 / 새로운 Knowledge Structure가 발견되면, 억지로 Feature를 만들지 말고 이 시트에 먼저 등록한다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="4" t="inlineStr">
+        <is>
+          <t>Candidate는 Definition · First Found · Status · Example 만 작성하고 Repeated는 비워둔다. (반복 관찰이 누적되면 Repeated를 채우고 승격 검토)</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="4" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="3" t="inlineStr">
+        <is>
+          <t>── 후보 노드 재분류 로그 (원칙3: 계층별 분류) ──</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="4" t="inlineStr">
+        <is>
+          <t>Dynamic Loft Low / High → Derived Parameters 시트 (계산·조합값).</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="4" t="inlineStr">
+        <is>
+          <t>Arm Dominant Pattern → DOH Coaching Knowledge 시트 (여러 Feature 종합 해석).</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="4" t="inlineStr">
+        <is>
+          <t>Lead Arm Against Chest → Chicken Wing (P7)에 통합 (원칙 ⑨: 독립 Information Gain 없음).</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="4" t="inlineStr">
+        <is>
+          <t>Grip Strong / Weak → P1 Setup Influence 참조 (P7 신규 Feature 아님).</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="4" t="inlineStr">
+        <is>
+          <t>Trail Wrist / Forearm 계열 → P8 Release 단계에서 재검토 (현재 독립 Feature 아님).</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:F14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -6451,7 +6654,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -6681,13 +6884,13 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D17"/>
+  <dimension ref="A1:D19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -6872,59 +7075,63 @@
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>LOCK 검토 (프로 승인)</t>
+          <t>Feature Naming Rule 통일 적용 [Object][Attribute](Phase)</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>todo</t>
+          <t>done</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>← 현재 단계. 승인 후 Stage 2 착수.</t>
+          <t>LOCK. Pattern Feature 예외 + Hand Axes 명시.</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>p7 메인 시트: Core 14 Feature 6-섹션 표준화</t>
+          <t>Candidate Concepts 시트 신설 + 재분류 로그</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>todo</t>
+          <t>done</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>Dictionary 기준 문장만 사용.</t>
+          <t>Repeated 공백. Stage 2 선등록 운영.</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>p7 메인 시트: Modifier 2 Feature 5-섹션</t>
+          <t>LOCK 검토 (프로 승인)</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>todo</t>
-        </is>
-      </c>
-      <c r="D11" s="2" t="inlineStr"/>
+          <t>done</t>
+        </is>
+      </c>
+      <c r="D11" s="2" t="inlineStr">
+        <is>
+          <t>PST/Naming/Dictionary 정책 LOCK 완료.</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
@@ -6934,7 +7141,7 @@
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>각 Feature 우측 Evidence Matrix 컬럼 구조(별점 제외)</t>
+          <t>p7 메인 시트: Core 14 Feature 6-섹션 표준화</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
@@ -6942,17 +7149,21 @@
           <t>todo</t>
         </is>
       </c>
-      <c r="D12" s="2" t="inlineStr"/>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
+          <t>Dictionary 기준 문장만 사용.</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>Evidence Matrix 별점 일괄 부여</t>
+          <t>p7 메인 시트: Modifier 2 Feature 5-섹션</t>
         </is>
       </c>
       <c r="C13" s="2" t="inlineStr">
@@ -6960,71 +7171,107 @@
           <t>todo</t>
         </is>
       </c>
-      <c r="D13" s="2" t="inlineStr">
-        <is>
-          <t>P1~P8 설계 완료 후 별도 세션.</t>
-        </is>
-      </c>
+      <c r="D13" s="2" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>각 Feature 우측 Evidence Matrix 컬럼 구조(별점 제외)</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t>todo</t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="inlineStr"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="inlineStr">
+        <is>
           <t>3</t>
         </is>
       </c>
-      <c r="B14" s="2" t="inlineStr">
-        <is>
-          <t>HTML/JSON 변환</t>
-        </is>
-      </c>
-      <c r="C14" s="2" t="inlineStr">
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t>Evidence Matrix 별점 일괄 부여</t>
+        </is>
+      </c>
+      <c r="C15" s="2" t="inlineStr">
         <is>
           <t>todo</t>
         </is>
       </c>
-      <c r="D14" s="2" t="inlineStr">
-        <is>
-          <t>P1~P8 LOCK 후 일괄.</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="2" t="inlineStr"/>
-      <c r="B15" s="2" t="inlineStr"/>
-      <c r="C15" s="2" t="inlineStr"/>
       <c r="D15" s="2" t="inlineStr">
         <is>
-          <t> </t>
+          <t>P1~P8 설계 완료 후 별도 세션.</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>HTML/JSON 변환</t>
+        </is>
+      </c>
+      <c r="C16" s="2" t="inlineStr">
+        <is>
+          <t>todo</t>
+        </is>
+      </c>
+      <c r="D16" s="2" t="inlineStr">
+        <is>
+          <t>P1~P8 LOCK 후 일괄.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="inlineStr"/>
+      <c r="B17" s="2" t="inlineStr"/>
+      <c r="C17" s="2" t="inlineStr"/>
+      <c r="D17" s="2" t="inlineStr">
+        <is>
+          <t> </t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
           <t>참고</t>
         </is>
       </c>
-      <c r="B16" s="2" t="inlineStr">
+      <c r="B18" s="2" t="inlineStr">
         <is>
           <t>작업 순서: Dictionary LOCK → Feature 6-섹션 → Evidence Matrix 별점 → HTML/JSON</t>
         </is>
       </c>
-      <c r="C16" s="2" t="inlineStr"/>
-      <c r="D16" s="2" t="inlineStr"/>
-    </row>
-    <row r="17">
-      <c r="A17" s="2" t="inlineStr">
+      <c r="C18" s="2" t="inlineStr"/>
+      <c r="D18" s="2" t="inlineStr"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="inlineStr">
         <is>
           <t>참고</t>
         </is>
       </c>
-      <c r="B17" s="2" t="inlineStr">
+      <c r="B19" s="2" t="inlineStr">
         <is>
           <t>동일 의미=동일 문장, 동일 Mechanism=동일 문장, 동일 Feature=동일 이름</t>
         </is>
       </c>
-      <c r="C17" s="2" t="inlineStr"/>
-      <c r="D17" s="2" t="inlineStr"/>
+      <c r="C19" s="2" t="inlineStr"/>
+      <c r="D19" s="2" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
feat(P7): Naming Rule을 Object+Axis+Attribute로 확정
- 'Position' 폐기(축 정보 소실 방지), Axis 필수 포함
- Hand Distance Close/Far → Close To Body / Far From Body (기준점 포함)
- Axis 재사용 표준(Direction/Height/Distance/Lateral/Depth) 명문화
  → Hand뿐 아니라 Club/Shaft/Pelvis/Thorax에 동일 축 체계 재사용
- Coordinate Reference Vocabulary를 Axis 기준으로 정리

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01AdDd8hWZsADEXdqNySEqXP
</commit_message>
<xml_diff>
--- a/DOH_P7.xlsx
+++ b/DOH_P7.xlsx
@@ -4267,7 +4267,7 @@
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>Hand Distance Close (P7)</t>
+          <t>Hand Distance Close To Body (P7)</t>
         </is>
       </c>
       <c r="C13" s="2" t="inlineStr">
@@ -4304,7 +4304,7 @@
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>Hand Distance Far (P7)</t>
+          <t>Hand Distance Far From Body (P7)</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
@@ -4935,7 +4935,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B47"/>
+  <dimension ref="A1:B49"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -4998,311 +4998,319 @@
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>모든 Feature는 [Object] [Attribute] (Phase) 형식으로 명명한다. Phase 태그로 동일 관찰의 Phase 차이를 구분한다. 예) Pelvis Open (P7) · Pelvis Open (P4) · Thorax Open (P7) · Club Face Open (P7) · Lead Pressure Excessive (P7) · Club Path Out-To-In (P7) · Hand Depth Deep (P4) · Hand Distance Close (P7) · Hand Direction Forward (P7). Attribute는 같은 단어를 반복 사용하고 새 표현은 최소화한다. 동일 의미는 항상 동일 이름, 새 이름이 필요하면 Dictionary에 먼저 등록 후 전 문서 일관 재사용.</t>
+          <t>모든 Feature는 [Object] [Axis] [Attribute] (Phase) 형식으로 명명한다. Axis(좌표축)를 반드시 포함해 AI가 축을 잃지 않게 한다. 'Position'은 축 정보가 사라지므로 사용하지 않는다. Phase 태그로 동일 관찰의 Phase 차이를 구분한다. 예) Hand Direction Forward (P7) · Hand Height High (P6) · Hand Depth Deep (P4) · Hand Distance Far From Body (P7) · Hand Lateral Out (P7). Attribute는 같은 단어를 반복 사용하고 새 표현은 최소화한다. 동일 의미는 항상 동일 이름, 새 이름은 Dictionary 등록 후 전 문서 일관 재사용.</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>②-예외 Pattern Feature</t>
+          <t>②-회전/상태 Feature</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>관용화된 패턴명(Standing Up, Chicken Wing)은 명칭을 유지하고 (Phase)만 붙인다. P6 선례: Spin-out · Early Extension · Casting.</t>
+          <t>회전·상태처럼 Axis가 자명한 경우 Object+Attribute로 축약한다. 예) Pelvis Open (P7) · Thorax Closed (P7) · Club Face Open (P7) · Lead Pressure Excessive (P7) · Club Path Out-To-In (P7).</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>②-Hand Position Axes</t>
+          <t>②-예외 Pattern Feature</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>손 위치 Feature는 축(Axis) 단어를 포함한다. Depth(Deep/Shallow)→Thorax · Height(High/Low) · Distance(Close/Far)→Torso · Direction(Forward/Backward)→Ball/Target Line. 예) Hand Depth Deep · Hand Distance Close · Hand Direction Forward.</t>
+          <t>관용화된 패턴명(Standing Up, Chicken Wing)은 명칭을 유지하고 (Phase)만 붙인다. P6 선례: Spin-out · Early Extension · Casting.</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>③ Coordinate System(절대 유지)</t>
+          <t>②-Axis 체계 (재사용 표준)</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>모든 위치 표현은 DOH Coordinate System 기준을 명시한다. Forward→Ball/Target Line · Open/Closed→Target Line · Near(Close)/Far→Torso · Deep→Thorax · Height(High/Low)→척추각/몸통 높이. 기준이 불명확한 표현은 사용하지 않는다.</t>
+          <t>Direction: Forward/Backward (Ball/Target Line 기준) · Height: High/Low · Distance: Close To Body/Far From Body (몸과의 거리, 기준점 포함) · Lateral: In/Out (Target Line 기준) · Depth: Deep/Shallow (몸 회전 기준). 이 Axis 체계는 Hand뿐 아니라 Club·Shaft·Pelvis·Thorax 등 모든 Object에 그대로 재사용한다.</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>④ Modifier Feature 구분</t>
+          <t>③ Coordinate System(절대 유지)</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>Lead Wrist Flexion/Extension 등은 독립 Problem Feature가 아니라 다른 Feature를 해석하는 Modifier Feature다. 템플릿을 달리한다(정의/Modifier 특성/대표 해석 사례/관련 Feature/사고확장의 5-섹션, 원인·이후·Strong Co-occurrence 없음).</t>
+          <t>모든 위치 표현은 DOH Coordinate System 기준을 명시한다. Forward→Ball/Target Line · Open/Closed→Target Line · Near(Close)/Far→Torso · Deep→Thorax · Height(High/Low)→척추각/몸통 높이. 기준이 불명확한 표현은 사용하지 않는다.</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>⑤ Coaching Knowledge 분리</t>
+          <t>④ Modifier Feature 구분</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>레슨 경험·잘못된 움직임 이미지·그립별 손목 해석·조건부 해석은 Feature에 쓰지 않고 'DOH Coaching Knowledge' 시트에 기록한다.</t>
+          <t>Lead Wrist Flexion/Extension 등은 독립 Problem Feature가 아니라 다른 Feature를 해석하는 Modifier Feature다. 템플릿을 달리한다(정의/Modifier 특성/대표 해석 사례/관련 Feature/사고확장의 5-섹션, 원인·이후·Strong Co-occurrence 없음).</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>⑥ Evidence Layer 분리</t>
+          <t>⑤ Coaching Knowledge 분리</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>Ball Flight·Impact Strike·Ground Contact는 Feature도 Outcome도 아닌 Evidence Layer다. 회원이 인지·입력하는 정보로, AI가 Feature를 역추론하는 근거다. 'Evidence Layer' 참조 시트로 관리하고, 각 Feature 우측 Evidence Matrix로 연결한다(별점은 후속 작업).</t>
+          <t>레슨 경험·잘못된 움직임 이미지·그립별 손목 해석·조건부 해석은 Feature에 쓰지 않고 'DOH Coaching Knowledge' 시트에 기록한다.</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>⑦ Branch Chain</t>
+          <t>⑥ Evidence Layer 분리</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>동일 Feature라도 보상 전략에 따라 이후 Chain이 분기하면 단일 결과로 단정하지 않고 Branch Chain으로 작성한다.</t>
+          <t>Ball Flight·Impact Strike·Ground Contact는 Feature도 Outcome도 아닌 Evidence Layer다. 회원이 인지·입력하는 정보로, AI가 Feature를 역추론하는 근거다. 'Evidence Layer' 참조 시트로 관리하고, 각 Feature 우측 Evidence Matrix로 연결한다(별점은 후속 작업).</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>⑧ Confidence 등급</t>
+          <t>⑦ Branch Chain</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>[High Confidence]=생체역학적으로 확실 · [Medium Confidence]=레슨상 자주 · [Low Confidence / Pattern Dependent] 또는 ※추론=특정 유형. 원인/이후 Chain에 등급을 명시한다.</t>
+          <t>동일 Feature라도 보상 전략에 따라 이후 Chain이 분기하면 단일 결과로 단정하지 않고 Branch Chain으로 작성한다.</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
+          <t>⑧ Confidence 등급</t>
+        </is>
+      </c>
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t>[High Confidence]=생체역학적으로 확실 · [Medium Confidence]=레슨상 자주 · [Low Confidence / Pattern Dependent] 또는 ※추론=특정 유형. 원인/이후 Chain에 등급을 명시한다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
           <t>⑨ Feature 신설 3원칙</t>
         </is>
       </c>
-      <c r="B15" s="2" t="inlineStr">
+      <c r="B16" s="2" t="inlineStr">
         <is>
           <t>새 Feature는 ①Observation이 다른가 ②새 Chain을 생성하는가 ③새 추론 정보(Information Gain)를 주는가 를 모두 만족할 때만 만든다. 아니면 기존 Feature 통합을 우선한다. 애매하면 임의 결정 없이 질문 후 진행한다.</t>
         </is>
       </c>
     </row>
-    <row r="16">
-      <c r="A16" s="2" t="inlineStr"/>
-      <c r="B16" s="2" t="inlineStr"/>
-    </row>
     <row r="17">
-      <c r="A17" s="2" t="inlineStr">
-        <is>
-          <t>Coordinate Reference Vocabulary</t>
-        </is>
-      </c>
+      <c r="A17" s="2" t="inlineStr"/>
       <c r="B17" s="2" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>Forward / Backward</t>
-        </is>
-      </c>
-      <c r="B18" s="2" t="inlineStr">
-        <is>
-          <t>Ball / Target Line 기준</t>
-        </is>
-      </c>
+          <t>Coordinate Reference Vocabulary (Axis 기준점)</t>
+        </is>
+      </c>
+      <c r="B18" s="2" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>Open / Closed</t>
+          <t>Direction (Forward / Backward)</t>
         </is>
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>Target Line 기준</t>
+          <t>Ball / Target Line 기준</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>Near(Close) / Far</t>
+          <t>Lateral (In / Out)</t>
         </is>
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>Torso 기준</t>
+          <t>Target Line 기준</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>Deep / Shallow</t>
+          <t>Rotation (Open / Closed)</t>
         </is>
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>Thorax 기준</t>
+          <t>Target Line 기준</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>High / Low (Height)</t>
+          <t>Distance (Close To Body / Far From Body)</t>
         </is>
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>척추각 / 몸통 높이 기준</t>
+          <t>Torso(몸) 기준</t>
         </is>
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="2" t="inlineStr"/>
-      <c r="B23" s="2" t="inlineStr"/>
+      <c r="A23" s="2" t="inlineStr">
+        <is>
+          <t>Depth (Deep / Shallow)</t>
+        </is>
+      </c>
+      <c r="B23" s="2" t="inlineStr">
+        <is>
+          <t>Thorax(몸 회전) 기준</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>Mechanism Categories (P7)</t>
-        </is>
-      </c>
-      <c r="B24" s="2" t="inlineStr"/>
+          <t>Height (High / Low)</t>
+        </is>
+      </c>
+      <c r="B24" s="2" t="inlineStr">
+        <is>
+          <t>척추각 / 몸통 높이 기준</t>
+        </is>
+      </c>
     </row>
     <row r="25">
-      <c r="A25" s="2" t="inlineStr">
-        <is>
-          <t>ROT</t>
-        </is>
-      </c>
-      <c r="B25" s="2" t="inlineStr">
-        <is>
-          <t>Rotation — 골반/흉곽 회전(Amount·Timing·Velocity·Axis)</t>
-        </is>
-      </c>
+      <c r="A25" s="2" t="inlineStr"/>
+      <c r="B25" s="2" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>PRS</t>
-        </is>
-      </c>
-      <c r="B26" s="2" t="inlineStr">
-        <is>
-          <t>Pressure — 리드/트레일 하중 및 압력 분포</t>
-        </is>
-      </c>
+          <t>Mechanism Categories (P7)</t>
+        </is>
+      </c>
+      <c r="B26" s="2" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t>ARM</t>
+          <t>ROT</t>
         </is>
       </c>
       <c r="B27" s="2" t="inlineStr">
         <is>
-          <t>Arm Delivery — 팔·손·팔꿈치의 전달과 신전</t>
+          <t>Rotation — 골반/흉곽 회전(Amount·Timing·Velocity·Axis)</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>CLB</t>
+          <t>PRS</t>
         </is>
       </c>
       <c r="B28" s="2" t="inlineStr">
         <is>
-          <t>Club Delivery — 페이스 방향·경로(Path)·릴리즈·로프트</t>
+          <t>Pressure — 리드/트레일 하중 및 압력 분포</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
         <is>
-          <t>SPC</t>
+          <t>ARM</t>
         </is>
       </c>
       <c r="B29" s="2" t="inlineStr">
         <is>
-          <t>Space — 몸-팔 전달 공간 및 스윙 반경(Radius)</t>
+          <t>Arm Delivery — 팔·손·팔꿈치의 전달과 신전</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>LOD</t>
+          <t>CLB</t>
         </is>
       </c>
       <c r="B30" s="2" t="inlineStr">
         <is>
-          <t>Loading — 리드/트레일측 하중 수용과 안정</t>
+          <t>Club Delivery — 페이스 방향·경로(Path)·릴리즈·로프트</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
         <is>
-          <t>CMP</t>
+          <t>SPC</t>
         </is>
       </c>
       <c r="B31" s="2" t="inlineStr">
         <is>
-          <t>Compensation — 페이스·회전·손·몸의 보상 동작</t>
+          <t>Space — 몸-팔 전달 공간 및 스윙 반경(Radius)</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>PST</t>
+          <t>LOD</t>
         </is>
       </c>
       <c r="B32" s="2" t="inlineStr">
         <is>
-          <t>Posture / Axis — 척추각·측굴·전경·몸통 높이(신규, P7에서 신설)</t>
+          <t>Loading — 리드/트레일측 하중 수용과 안정</t>
         </is>
       </c>
     </row>
     <row r="33">
-      <c r="A33" s="2" t="inlineStr"/>
-      <c r="B33" s="2" t="inlineStr"/>
+      <c r="A33" s="2" t="inlineStr">
+        <is>
+          <t>CMP</t>
+        </is>
+      </c>
+      <c r="B33" s="2" t="inlineStr">
+        <is>
+          <t>Compensation — 페이스·회전·손·몸의 보상 동작</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>Player Type 태그(신규)</t>
+          <t>PST</t>
         </is>
       </c>
       <c r="B34" s="2" t="inlineStr">
         <is>
-          <t>같은 Feature라도 생성 메커니즘이 선수/아마추어에서 다를 때 [Player Type: Amateur/Elite] 태그로 해석 맥락(Context)을 부여한다. Feature 자체는 바꾸지 않는다. (예: Side Bend Excessive (P7))</t>
+          <t>Posture / Axis — 척추각·측굴·전경·몸통 높이(신규, P7에서 신설)</t>
         </is>
       </c>
     </row>
@@ -5313,134 +5321,150 @@
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>Role Taxonomy (DOH Object Roles)</t>
+          <t>Player Type 태그(신규)</t>
         </is>
       </c>
       <c r="B36" s="2" t="inlineStr">
         <is>
-          <t>역할을 명확히 분리한다. 규모가 커질수록 합치지 말고 유지한다.</t>
+          <t>같은 Feature라도 생성 메커니즘이 선수/아마추어에서 다를 때 [Player Type: Amateur/Elite] 태그로 해석 맥락(Context)을 부여한다. Feature 자체는 바꾸지 않는다. (예: Side Bend Excessive (P7))</t>
         </is>
       </c>
     </row>
     <row r="37">
-      <c r="A37" s="2" t="inlineStr">
-        <is>
-          <t>Core Feature</t>
-        </is>
-      </c>
-      <c r="B37" s="2" t="inlineStr">
-        <is>
-          <t>독립적으로 관찰되는 문제/현상 Feature. 6-섹션 템플릿.</t>
-        </is>
-      </c>
+      <c r="A37" s="2" t="inlineStr"/>
+      <c r="B37" s="2" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>Modifier Feature</t>
+          <t>Role Taxonomy (DOH Object Roles)</t>
         </is>
       </c>
       <c r="B38" s="2" t="inlineStr">
         <is>
-          <t>다른 Feature의 해석을 바꾸는 보조 Feature. 5-섹션 템플릿(원인/이후/Strong Co-occurrence 없음).</t>
+          <t>역할을 명확히 분리한다. 규모가 커질수록 합치지 말고 유지한다.</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
         <is>
-          <t>Setup Influence</t>
+          <t>Core Feature</t>
         </is>
       </c>
       <c r="B39" s="2" t="inlineStr">
         <is>
-          <t>P1 Setup에서 기원하는 영향 요인(예: Grip Strong/Weak). 후속 Phase에서 새로 만들지 않고 참조한다.</t>
+          <t>독립적으로 관찰되는 문제/현상 Feature. 6-섹션 템플릿.</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>Coaching Knowledge</t>
+          <t>Modifier Feature</t>
         </is>
       </c>
       <c r="B40" s="2" t="inlineStr">
         <is>
-          <t>여러 Feature 종합 해석·레슨 이미지·조건부 지식(예: Arm Dominant Pattern). 별도 시트.</t>
+          <t>다른 Feature의 해석을 바꾸는 보조 Feature. 5-섹션 템플릿(원인/이후/Strong Co-occurrence 없음).</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
         <is>
-          <t>Candidate Concepts</t>
+          <t>Setup Influence</t>
         </is>
       </c>
       <c r="B41" s="2" t="inlineStr">
         <is>
-          <t>Feature화가 애매한 개념. 'DOH Candidate Concepts' 시트에 선등록(Repeated 공백).</t>
+          <t>P1 Setup에서 기원하는 영향 요인(예: Grip Strong/Weak). 후속 Phase에서 새로 만들지 않고 참조한다.</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>Biomechanical Concepts</t>
+          <t>Coaching Knowledge</t>
         </is>
       </c>
       <c r="B42" s="2" t="inlineStr">
         <is>
-          <t>생체역학 개념·Injury Risk 등(예: Lumbar Stress). Mechanism/Note로 관리.</t>
+          <t>여러 Feature 종합 해석·레슨 이미지·조건부 지식(예: Arm Dominant Pattern). 별도 시트.</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
         <is>
-          <t>Derived Parameters</t>
+          <t>Candidate Concepts</t>
         </is>
       </c>
       <c r="B43" s="2" t="inlineStr">
         <is>
-          <t>계산·조합으로 산출되는 값(예: Dynamic Loft). 별도 시트.</t>
+          <t>Feature화가 애매한 개념. 'DOH Candidate Concepts' 시트에 선등록(Repeated 공백).</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
         <is>
-          <t>PST</t>
+          <t>Biomechanical Concepts</t>
         </is>
       </c>
       <c r="B44" s="2" t="inlineStr">
         <is>
-          <t>Posture/Axis Mechanism 카테고리(척추각·측굴·전경·몸통 높이). CMP와 합치지 않고 유지(LOCK).</t>
+          <t>생체역학 개념·Injury Risk 등(예: Lumbar Stress). Mechanism/Note로 관리.</t>
         </is>
       </c>
     </row>
     <row r="45">
-      <c r="A45" s="2" t="inlineStr"/>
-      <c r="B45" s="2" t="inlineStr"/>
+      <c r="A45" s="2" t="inlineStr">
+        <is>
+          <t>Derived Parameters</t>
+        </is>
+      </c>
+      <c r="B45" s="2" t="inlineStr">
+        <is>
+          <t>계산·조합으로 산출되는 값(예: Dynamic Loft). 별도 시트.</t>
+        </is>
+      </c>
     </row>
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
         <is>
+          <t>PST</t>
+        </is>
+      </c>
+      <c r="B46" s="2" t="inlineStr">
+        <is>
+          <t>Posture/Axis Mechanism 카테고리(척추각·측굴·전경·몸통 높이). CMP와 합치지 않고 유지(LOCK).</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="2" t="inlineStr"/>
+      <c r="B47" s="2" t="inlineStr"/>
+    </row>
+    <row r="48">
+      <c r="A48" s="2" t="inlineStr">
+        <is>
           <t>⑩ Candidate 우선 원칙</t>
         </is>
       </c>
-      <c r="B46" s="2" t="inlineStr">
+      <c r="B48" s="2" t="inlineStr">
         <is>
           <t>Stage 2 등 이후 작업에서 새 개념/Mechanism 구조/Knowledge Structure가 나오면 억지로 Feature를 만들지 말고 Candidate Concepts 시트에 먼저 등록한다. Definition·First Found·Status·Example만 작성하고 Repeated는 비워둔다.</t>
         </is>
       </c>
     </row>
-    <row r="47">
-      <c r="A47" s="2" t="inlineStr">
+    <row r="49">
+      <c r="A49" s="2" t="inlineStr">
         <is>
           <t>⑪ Dictionary 수정 정책(LOCK)</t>
         </is>
       </c>
-      <c r="B47" s="2" t="inlineStr">
+      <c r="B49" s="2" t="inlineStr">
         <is>
           <t>현재 Dictionary는 유지. P1~P4 진행 중에는 '추가'만 하고 수정은 최소화한다. P4 완료 후 Dictionary Refactoring을 1회 일괄 수행한다.</t>
         </is>

</xml_diff>

<commit_message>
feat(P7): Stage 2 전체 — Core 14 (6-섹션) + Modifier 2 (5-섹션)
p7 메인 시트 완성. 프로토타입 5개 피드백 전량 반영:
- Ball Flight/Contact를 Feature Chain에서 제거 → 체인은 Feature에서 종료,
  Ball Flight·Impact Strike·Ground Contact는 Evidence Matrix에서만 관리
- Branch Chain에 분기 원인 Mechanism 한 줄 삽입(표준문장)
- Confidence 3단계(High / Pattern Dependent / Low)
- Feature Header에 Family 필드 추가(Object 분류)
- Evidence Matrix 별도 시트 유지(16 Feature × 14 Outcome, 별점 보류)
- 체인 문장은 Mechanism_Dictionary 표준문장만 사용(무결성 검증 통과)
- Stage2에서 필요한 Mechanism 12개 사전에 추가(수정 없이 추가만) → 총 120

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01AdDd8hWZsADEXdqNySEqXP
</commit_message>
<xml_diff>
--- a/DOH_P7.xlsx
+++ b/DOH_P7.xlsx
@@ -57,7 +57,7 @@
       <color rgb="00FFFFFF"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="6">
     <fill>
       <patternFill/>
     </fill>
@@ -77,6 +77,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00EEF2FA"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00548235"/>
       </patternFill>
     </fill>
   </fills>
@@ -120,7 +125,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
@@ -144,6 +149,9 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="2" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -514,11 +522,11 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B26"/>
+  <dimension ref="A1:B131"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="24" customWidth="1" min="1" max="1"/>
-    <col width="108" customWidth="1" min="2" max="2"/>
+    <col width="26" customWidth="1" min="1" max="1"/>
+    <col width="112" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -529,7 +537,7 @@
       </c>
       <c r="B1" s="5" t="inlineStr">
         <is>
-          <t>DOH Impact (P7) — Feature 표준화 시트 · Stage 2 (PROTOTYPE: ① Impact Geometry)</t>
+          <t>DOH Impact (P7) — Feature 표준화 시트 · Stage 2 (Core 14 + Modifier 2)</t>
         </is>
       </c>
     </row>
@@ -549,7 +557,7 @@
       </c>
       <c r="B3" s="6" t="inlineStr">
         <is>
-          <t>Hand Direction Forward (P7)  ·  손 앞섬  ·  Hands / Direction · Forward</t>
+          <t>Hand Direction Forward (P7)  ·  손 앞섬  ·  Family: Hand Position Family  ·  Hands / Direction · Forward</t>
         </is>
       </c>
     </row>
@@ -561,7 +569,7 @@
       </c>
       <c r="B4" s="8" t="inlineStr">
         <is>
-          <t>임팩트(P7) 순간 그립 핸들(손)이 기준 위치보다 타깃 방향(Forward)에 위치하는 현상. 관찰 대상은 손(그립 핸들)이며 Forward는 Ball / Target Line 기준. 손의 위치를 관찰하는 Feature이며 샤프트 기울기(Forward Shaft Lean)와는 구분한다.</t>
+          <t>임팩트(P7) 순간 그립 핸들(손)이 기준 위치보다 타깃 방향(Forward)에 위치하는 현상. 관찰 대상은 손(그립 핸들)이며 Forward는 Ball / Target Line 기준. 손의 위치를 관찰하며 샤프트 기울기(Forward Shaft Lean)와 구분한다.</t>
         </is>
       </c>
     </row>
@@ -593,7 +601,7 @@
  ↓
 Hand Direction Forward (P7)
 ※ Modifier 해석
-[Medium Confidence]
+[Pattern Dependent]
 Thorax Open (P7) (임팩트 시 흉곽 과오픈)
  ↓
 Earlier Thorax Rotation Transports The Handle Further Forward Before Impact.
@@ -606,22 +614,20 @@
 (손목 각도를 오래 유지하면 클럽헤드보다 핸들이 계속 앞선다.)
  ↓
 Hand Direction Forward (P7)
-※ 추론
 Forward COM (P7) [Candidate]
  ↓
 Forward Body Motion Moves The Entire Delivery System Closer To The Target.
 (신체 전체가 전방으로 이동하면서 핸들 위치도 함께 전진한다.)
  ↓
 Hand Direction Forward (P7)
-※ 추론
-[Low Confidence / Pattern Dependent]
+[Low Confidence]
 Early Extension (P6, 얼리 익스텐션)
  ↓
 Some Golfers Push The Handle Forward While Losing Hip Depth.
 (골반 깊이를 잃는 과정에서 손을 앞으로 밀어내는 보상이 나타날 수 있다.)
  ↓
 Hand Direction Forward (P7)
-※ 특정 패턴에서만 관찰</t>
+※ 특정 패턴</t>
         </is>
       </c>
     </row>
@@ -639,27 +645,21 @@
 The Handle Arrives Ahead Of The Clubhead At Impact.
 (핸들이 클럽헤드보다 앞선 상태로 임팩트를 형성한다.)
  ↓
-Forward Shaft Lean (샤프트 전경)
+Forward Shaft Lean (P7) [Candidate]
 Hand Direction Forward (P7)
  ↓
 Handle Lead Reduces Dynamic Loft At Impact.
 (핸들의 선행은 임팩트 시 동적 로프트를 감소시킨다.)
  ↓
-Dynamic Loft Low (동적 로프트 부족) ※ Derived Parameter
-[Medium Confidence]
+Dynamic Loft Low  ※ Derived Parameter
+[Pattern Dependent]
 Hand Direction Forward (P7)
  ↓
 Excessive Handle Lead Can Delay Clubface Closure.
 (과도한 핸들 선행은 페이스 닫힘을 늦출 수 있다.)
  ↓
 Club Face Open (P7)
-※ 패턴 의존
-Hand Direction Forward (P7)
- ↓
-The Club Strikes The Ball Before The Turf.
-(볼을 먼저 맞힌다.)
- ↓
-Ball-Then-Turf Contact  ※ Evidence Layer (Impact Condition)</t>
+※ 패턴 의존</t>
         </is>
       </c>
     </row>
@@ -671,12 +671,12 @@
       </c>
       <c r="B7" s="8" t="inlineStr">
         <is>
-          <t>★★★★★  Forward Shaft Lean (샤프트 전경)
+          <t>★★★★★  Forward Shaft Lean (P7)
 ★★★★★  Lead Pressure (리드측 압력)
-★★★★☆  Pelvis Open (P7) (임팩트 시 골반 과오픈)
-★★★★☆  Lead Wrist Flexion (P7) (리드 손목 굴곡)
-★★★☆☆  Late Release (릴리즈 지연)
-★★★☆☆  Thorax Open (P7) (임팩트 시 흉곽 과오픈)</t>
+★★★★☆  Pelvis Open (P7)
+★★★★☆  Lead Wrist Flexion (P7)
+★★★☆☆  Late Release (P6)
+★★★☆☆  Thorax Open (P7)</t>
         </is>
       </c>
     </row>
@@ -692,8 +692,8 @@
 - 손의 위치(Direction)와 샤프트 기울기(Geometry)를 혼동하고 있지 않은가?
 - 리드측 압력이 실제로 확보된 상태인가?
 - 골반 회전에 의해 형성된 것인가, 손목 패턴에 의해 형성된 것인가?
-- 임팩트 직전(P6)부터 이미 Forward Hands가 형성되어 있었는가?
-- 과도한 Forward인지, 적절한 Compression을 위한 범위인지 구분 가능한가?</t>
+- 임팩트 직전(P6)부터 이미 Forward가 형성되어 있었는가?
+- 과도한 Forward인지, 적절한 Compression 범위인지 구분 가능한가?</t>
         </is>
       </c>
     </row>
@@ -705,10 +705,10 @@
       </c>
       <c r="B9" s="8" t="inlineStr">
         <is>
-          <t>- Hand Direction Forward는 P6 Delivery와 P7 Impact를 연결하는 대표 매개(Mediator) Feature일 가능성이 높다.
-- 동일 Forward라도 Pressure-driven / Rotation-driven / Wrist-driven / Release-driven으로 세분될 수 있다.
+          <t>- Hand Direction Forward는 P6 Delivery와 P7 Impact를 연결하는 대표 매개(Mediator) Feature.
+- 동일 Forward라도 Pressure-driven / Rotation-driven / Wrist-driven / Release-driven으로 세분 가능.
 - Forward Shaft Lean · Dynamic Loft · Compression · Strike Quality를 연결하는 Hub Feature.
-- 향후 'Hand Position Family'(Direction/Height/Depth/Distance/Lateral)의 중심 Feature로 발전 가능.</t>
+- 향후 Hand Position Family(Direction/Height/Depth/Distance/Lateral)의 중심 Feature로 발전 가능.</t>
         </is>
       </c>
     </row>
@@ -724,7 +724,7 @@
       </c>
       <c r="B11" s="6" t="inlineStr">
         <is>
-          <t>Club Face Open (P7)  ·  임팩트 시 클럽페이스 오픈  ·  Club / Rotation · Open</t>
+          <t>Club Face Open (P7)  ·  임팩트 시 클럽페이스 오픈  ·  Family: Club Face Family  ·  Club / Rotation · Open</t>
         </is>
       </c>
     </row>
@@ -775,35 +775,33 @@
  ↓
 Club Face Open (P7)
 ※ Setup Influence
-[Medium Confidence]
+[Pattern Dependent]
 Thorax Open (P7) (임팩트 시 흉곽 과오픈)
  ↓
 Body Rotation Outpaces Clubface Rotation, Leaving The Face Open.
 (몸 회전이 페이스 회전보다 빨라 페이스가 열린 채 남는다.)
  ↓
 Club Face Open (P7)
-※ 추론
 Steep Shaft (P6, 가파른 샤프트)
  ↓
 A Steeper Delivery Requires More Face Rotation To Square The Club.
 (가파른 전달에서는 스퀘어를 위한 페이스 회전량이 증가한다.)
  ↓
 Club Face Open (P7)
-※ 추론
 Late Arm (P6, 팔 하강 지연)
  ↓
 Delayed Arm Delivery Leaves The Clubface Open Into Impact.
 (팔 전달이 늦어지면 페이스가 열린 상태로 임팩트에 도달한다.)
  ↓
 Club Face Open (P7)
-[Low Confidence / Pattern Dependent]
+[Low Confidence]
 Pelvis Open (P7) (임팩트 시 골반 과오픈)
  ↓
 Body Rotation Outpaces Clubface Rotation, Leaving The Face Open.
 (몸 회전이 페이스 회전보다 빨라 페이스가 열린 채 남는다.)
  ↓
 Club Face Open (P7)
-※ 특정 패턴 (몸 회전 대비 팔·페이스 회전 부족)</t>
+※ 특정 패턴</t>
         </is>
       </c>
     </row>
@@ -815,47 +813,39 @@
       </c>
       <c r="B14" s="8" t="inlineStr">
         <is>
-          <t>[High Confidence]
-Club Face Open (P7)
- ↓
-An Open Clubface Starts The Ball Right Of The Target.
-(열린 페이스는 볼을 목표 우측으로 출발시킨다.)
- ↓
-Push / Push-Slice  ※ Evidence Layer (Ball Flight)
-Club Face Open (P7)
- ↓
-An Open Face Relative To Swing Path Produces Fade Or Slice Spin.
-(스윙패스 대비 열린 페이스는 페이드/슬라이스 회전을 만든다.)
- ↓
-Fade / Slice  ※ Evidence Layer (Ball Flight)
+          <t>── Branch (분기) ──
+The Chosen Compensation Strategy Determines The Subsequent Chain.
+(선택된 보상 전략이 이후 Chain을 결정한다.)
+[High Confidence]
 Club Face Open (P7)
  ↓
 The Player Rotates The Body More Aggressively To Help Square The Clubface.
 (열린 페이스를 맞추기 위해 몸 회전을 더 적극적으로 사용한다.)
  ↓
 Pelvis Open (P7) / Thorax Open (P7)
-※ Rotation Compensation
+※ ① Rotation Compensation
 Club Face Open (P7)
  ↓
 Excessive Body Rotation Shifts The Club Toward An Out-To-In Delivery.
 (과도한 몸 회전은 클럽을 아웃투인 궤도로 유도한다.)
  ↓
 Club Path Out-To-In (P7) [Candidate]
-※ 보상 결과 (직접 원인 아님)
-[Medium Confidence]
+※ Rotation Comp의 결과 (직접 원인 아님)
 Club Face Open (P7)
  ↓
 A Late Hand Rotation Attempts To Close The Clubface Just Before Impact.
 (임팩트 직전 손을 급하게 회전시켜 페이스를 닫으려 한다.)
  ↓
 Face Closure Late (P7) [Candidate]
-※ Hand Release Compensation
+※ ② Hand Release Compensation
+[Pattern Dependent]
 Club Face Open (P7)
  ↓
-Repeated Open-Face Contact Encourages Grip Or Release Compensation.
-(반복적인 오픈 페이스는 그립이나 릴리즈 보상을 유도한다.)
- ↓
-Compensation Pattern  ※ Coaching Knowledge</t>
+Players Increase Lead Wrist Flexion To Offset The Open Clubface.
+(열린 페이스를 보상하기 위해 리드 손목 굴곡을 더 사용한다.)
+ ↓
+Lead Wrist Flexion (P7)
+※ ② Hand Release (Modifier)</t>
         </is>
       </c>
     </row>
@@ -867,13 +857,13 @@
       </c>
       <c r="B15" s="8" t="inlineStr">
         <is>
-          <t>★★★★★  Late Release (릴리즈 지연)
+          <t>★★★★★  Late Release (P6)
 ★★★★★  Club Face Open (P6)
-★★★★★  Lead Wrist Extension (P7) (리드 손목 신전)
-★★★★☆  Weak Grip (위크 그립)
-★★★★☆  Late Arm (P6, 팔 하강 지연)
+★★★★★  Lead Wrist Extension (P7)
+★★★★☆  Weak Grip (P1 Setup)
+★★★★☆  Late Arm (P6)
 ★★★★☆  Club Path Out-To-In (P7)
-★★★★☆  Pelvis Open (P7)  ※ 보상 패턴으로 자주 동반</t>
+★★★★☆  Pelvis Open (P7)</t>
         </is>
       </c>
     </row>
@@ -887,10 +877,10 @@
         <is>
           <t>- P6에서 이미 페이스가 열린 상태였는가?
 - 리드 손목 조건(굴곡/신전)은 어떠한가?
-- 그립의 영향(Strong / Neutral / Weak)은 존재하는가? (Setup Influence)
-- 몸 회전을 과도하게 사용하여 페이스를 맞추려는 보상 패턴을 보이는가?
-- 손을 급하게 사용하여 페이스를 닫으려는 흔적이 있는가?
-- 보상 없이 그대로 임팩트하는 패턴인가, 보상을 통해 다른 구질을 만드는 패턴인가?</t>
+- 그립의 영향(Strong/Neutral/Weak)은 존재하는가? (Setup Influence)
+- 몸 회전을 과도하게 사용해 페이스를 맞추려는 보상인가?
+- 손을 급하게 사용해 페이스를 닫으려는 흔적이 있는가?
+- 보상 없이 그대로 임팩트하는가, 보상으로 다른 구질을 만드는가?</t>
         </is>
       </c>
     </row>
@@ -902,10 +892,10 @@
       </c>
       <c r="B17" s="8" t="inlineStr">
         <is>
-          <t>- Club Face Open은 단순히 슬라이스의 원인이 아니라, 이후 다양한 보상을 유발하는 Hub Feature.
+          <t>- Club Face Open은 슬라이스의 원인만이 아니라 다양한 보상을 유발하는 Hub Feature.
 - 보상 전략 3분기: ① Rotation Compensation ② Hand Release Compensation ③ No Compensation.
-- 이 세 분기는 이후 Swing Path·Release·Ball Flight를 크게 다르게 만드는 Archetype 기준이 된다.
-- [인과 정밀화] Open Face가 직접 Out-To-In을 만드는 것이 아니라, 골퍼의 보상 전략(몸을 더 돌려 맞추려는 의도)이 Out-To-In을 만든다.</t>
+- 이 3분기가 이후 Swing Path·Release·Ball Flight를 크게 다르게 만드는 Archetype 기준.
+- [인과 정밀화] Open Face가 직접 Out-To-In을 만드는 게 아니라, 골퍼의 보상 전략이 Out-To-In을 만든다.</t>
         </is>
       </c>
     </row>
@@ -921,7 +911,7 @@
       </c>
       <c r="B19" s="6" t="inlineStr">
         <is>
-          <t>Club Face Closed (P7)  ·  임팩트 시 클럽페이스 클로즈  ·  Club / Rotation · Closed</t>
+          <t>Club Face Closed (P7)  ·  임팩트 시 클럽페이스 클로즈  ·  Family: Club Face Family  ·  Club / Rotation · Closed</t>
         </is>
       </c>
     </row>
@@ -972,21 +962,19 @@
 (P6에서 닫힌 페이스가 임팩트까지 유지된다.)
  ↓
 Club Face Closed (P7)
-[Medium Confidence]
+[Pattern Dependent]
 Trail Forearm Rotation (P8 재검토 노드)
  ↓
 Earlier Forearm Rotation Accelerates Face Closure.
 (전완의 조기 회전은 페이스 닫힘을 빠르게 만든다.)
  ↓
 Club Face Closed (P7)
-※ 추론
 Pelvis Closed (P7) / Late Body Rotation
  ↓
 Reduced Body Rotation Allows The Hands To Overtake The Pivot.
 (몸 회전이 부족하면 손이 몸보다 먼저 작용한다.)
  ↓
-Club Face Closed (P7)
-※ 추론</t>
+Club Face Closed (P7)</t>
         </is>
       </c>
     </row>
@@ -1001,45 +989,37 @@
           <t>[High Confidence]
 Club Face Closed (P7)
  ↓
-A Closed Clubface Starts The Ball Left Of The Target.
-(닫힌 페이스는 볼을 목표 좌측으로 출발시킨다.)
- ↓
-Pull  ※ Evidence Layer (Ball Flight)
-Club Face Closed (P7)
- ↓
-A Closed Face Relative To Swing Path Produces Draw Or Hook Spin.
-(스윙패스 대비 닫힌 페이스는 드로우/훅 회전을 만든다.)
- ↓
-Draw / Hook  ※ Evidence Layer (Ball Flight)
-Club Face Closed (P7)
- ↓
 Players Shift The Swing Direction More In-To-Out To Offset The Closed Clubface.
 (닫힌 페이스를 보상하기 위해 스윙 방향을 더 인투아웃으로 만든다.)
  ↓
 Club Path In-To-Out (P7) [Candidate]
-※ Path Compensation (대표)
-[Medium Confidence]
+※ ① Path Compensation (대표)
+── Branch (분기) ──
+The Chosen Compensation Strategy Determines The Subsequent Chain.
+(선택된 보상 전략이 이후 Chain을 결정한다.)
+[High Confidence]
 Club Face Closed (P7)
  ↓
 Players Reduce Body Rotation To Prevent The Ball From Going Further Left.
 (볼이 더 왼쪽으로 가는 것을 막기 위해 몸 회전을 줄인다.)
  ↓
 Pelvis Closed (P7)
-※ 보상
+※ ① Path Comp 계열
+[Pattern Dependent]
 Club Face Closed (P7)
  ↓
 Players Combine A Closed Face With An Out-To-In Path To Suppress A Left Start.
 (닫힌 페이스와 아웃투인 궤도를 함께 사용하여 좌측 출발을 억제한다.)
  ↓
-Club Path Out-To-In (P7) [Candidate] → Fade / Pull Fade
-※ Counter Compensation · Evidence Layer(Ball Flight)
+Club Path Out-To-In (P7) [Candidate]
+※ ② Counter Compensation
 Club Face Closed (P7)
  ↓
 Players Hold The Face Open Longer During Delivery To Offset Early Closure.
 (조기 닫힘을 보상하기 위해 전달 구간에서 페이스를 더 오래 열어둔다.)
  ↓
 Club Face Open (P6)
-※ 보상</t>
+※ ② Counter Comp</t>
         </is>
       </c>
     </row>
@@ -1051,12 +1031,12 @@
       </c>
       <c r="B23" s="8" t="inlineStr">
         <is>
-          <t>★★★★★  Lead Wrist Flexion (P7) (리드 손목 굴곡)
-★★★★★  Strong Grip (스트롱 그립)
+          <t>★★★★★  Lead Wrist Flexion (P7)
+★★★★★  Strong Grip (P1 Setup)
 ★★★★★  Club Face Closed (P6)
-★★★★☆  Early Release (조기 릴리즈)
-★★★★☆  Club Path In-To-Out (P7)  ※ 가장 흔한 보상 패턴
-★★★☆☆  Club Path Out-To-In (P7)  ※ 의도적 보상 패턴</t>
+★★★★☆  Early Release (P6)
+★★★★☆  Club Path In-To-Out (P7)  ※ 가장 흔한 보상
+★★★☆☆  Club Path Out-To-In (P7)  ※ 의도적 보상</t>
         </is>
       </c>
     </row>
@@ -1069,11 +1049,11 @@
       <c r="B24" s="8" t="inlineStr">
         <is>
           <t>- P6에서 이미 페이스가 닫혀 있었는가?
-- 그립의 영향(Strong / Neutral / Weak)은 어떠한가? (Setup Influence)
+- 그립의 영향(Strong/Neutral/Weak)은 어떠한가? (Setup Influence)
 - 리드 손목 굴곡이 유지되고 있는가?
-- 닫힌 페이스를 보상하기 위해 In-To-Out 스윙을 형성하는가?
-- 반대로 Out-To-In을 이용하여 구질을 조절하는가?
-- 보상 없이 그대로 임팩트하여 Pull 계열 구질이 반복되는가?</t>
+- 닫힌 페이스를 보상하기 위해 In-To-Out을 형성하는가?
+- 반대로 Out-To-In을 이용해 구질을 조절하는가?
+- 보상 없이 그대로 임팩트하여 Pull 계열이 반복되는가?</t>
         </is>
       </c>
     </row>
@@ -1085,16 +1065,1957 @@
       </c>
       <c r="B25" s="8" t="inlineStr">
         <is>
-          <t>- Club Face Closed는 훅만의 원인이 아니라, 이후 다양한 보상 전략을 유도하는 Hub Feature.
-- 보상 전략 3분기: ① Path Compensation(In-To-Out) ② Counter Compensation(Out-To-In) ③ No Compensation(Pull/Pull Hook).
+          <t>- Club Face Closed는 훅만의 원인이 아니라 다양한 보상 전략을 유도하는 Hub Feature.
+- 보상 전략 3분기: ① Path Compensation(In-To-Out) ② Counter Compensation(Out-To-In) ③ No Compensation.
 - 같은 Closed Face라도 Swing Path에 따라 전혀 다른 Ball Flight가 나타난다.
-- Face Angle은 단독으로 Ball Flight를 결정하지 않으며 Swing Path와의 관계(Face-to-Path) 속에서 해석해야 한다.</t>
+- Face Angle은 단독으로 Ball Flight를 결정하지 않으며 Swing Path와의 관계(Face-to-Path)로 해석한다.</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="8" t="inlineStr"/>
       <c r="B26" s="8" t="inlineStr"/>
+    </row>
+    <row r="27">
+      <c r="A27" s="5" t="inlineStr">
+        <is>
+          <t>② Body Alignment (신체 정렬)</t>
+        </is>
+      </c>
+      <c r="B27" s="5" t="inlineStr"/>
+    </row>
+    <row r="28">
+      <c r="A28" s="6" t="inlineStr">
+        <is>
+          <t>●</t>
+        </is>
+      </c>
+      <c r="B28" s="6" t="inlineStr">
+        <is>
+          <t>Pelvis Open (P7)  ·  임팩트 시 골반 과오픈  ·  Family: Pelvis Rotation Family  ·  Pelvis / Rotation · Open</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="7" t="inlineStr">
+        <is>
+          <t>■ 정의</t>
+        </is>
+      </c>
+      <c r="B29" s="8" t="inlineStr">
+        <is>
+          <t>임팩트(P7) 순간 골반이 기준보다 목표 방향으로 과도하게 회전(Open)된 상태. 골반 회전량만 관찰하며 흉곽 회전·스윙패스와 독립적으로 판단한다. Open은 Target Line 기준.</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="7" t="inlineStr">
+        <is>
+          <t>■ 원인 추정</t>
+        </is>
+      </c>
+      <c r="B30" s="8" t="inlineStr">
+        <is>
+          <t>[High Confidence]
+Spin-out (P6, 스핀아웃)
+ ↓
+The Pelvis Rotates Faster Than The Thorax And Arms.
+(골반이 상체와 팔보다 먼저 과도하게 회전한다.)
+ ↓
+Pelvis Open (P7)
+Pelvis Open (P6)
+ ↓
+The Excessive Pelvic Rotation From P6 Is Maintained Into Impact.
+(P6의 과도한 골반 회전이 임팩트까지 유지된다.)
+ ↓
+Pelvis Open (P7)
+Club Face Open (P7) (임팩트 시 클럽페이스 오픈)
+ ↓
+The Player Rotates The Body More Aggressively To Help Square The Clubface.
+(열린 페이스를 맞추기 위해 몸 회전을 더 적극적으로 사용한다.)
+ ↓
+Pelvis Open (P7)
+※ 보상
+[Pattern Dependent]
+Lead Pressure (리드측 압력)
+ ↓
+Earlier Lead Side Loading Allows Continued Pelvic Rotation.
+(리드측 압력이 충분하면 골반 회전이 계속 진행될 수 있다.)
+ ↓
+Pelvis Open (P7)
+※ 정상 패턴에서도 흔함
+Thorax Open (P7) (임팩트 시 흉곽 과오픈)
+ ↓
+The Thorax And Pelvis Rotate Together Through Impact.
+(흉곽과 골반이 임팩트 구간에서 함께 회전한다.)
+ ↓
+Pelvis Open (P7)
+Late Arm (P6, 팔 하강 지연)
+ ↓
+Delayed Arm Delivery Allows The Pelvis To Continue Rotating.
+(팔 전달이 늦어지는 동안 골반 회전이 계속 진행된다.)
+ ↓
+Pelvis Open (P7)</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="7" t="inlineStr">
+        <is>
+          <t>■ 이후 나타날 가능성</t>
+        </is>
+      </c>
+      <c r="B31" s="8" t="inlineStr">
+        <is>
+          <t>[High Confidence]
+Pelvis Open (P7)
+ ↓
+Excessive Body Rotation Shifts The Club Toward An Out-To-In Delivery.
+(과도한 몸 회전은 클럽을 아웃투인 궤도로 유도한다.)
+ ↓
+Club Path Out-To-In (P7) [Candidate]
+Pelvis Open (P7)
+ ↓
+The Arms Cannot Keep Up With The Rotating Body.
+(몸 회전을 팔이 따라가지 못한다.)
+ ↓
+Late Arm (P6)
+Pelvis Open (P7)
+ ↓
+Body Rotation Outpaces Clubface Rotation, Leaving The Face Open.
+(몸 회전이 페이스 회전보다 빨라 페이스가 열린 채 남는다.)
+ ↓
+Club Face Open (P7)
+Pelvis Open (P7)
+ ↓
+The Thorax Rotates Ahead Of The Arms, Leaving The Lead Arm Trapped Across The Chest.
+(상체 회전이 팔 전달보다 앞서면서 리드암이 가슴 앞에 갇힌다.)
+ ↓
+Chicken Wing (P7)  +  Trail Elbow Out (P7) [Candidate]
+[Pattern Dependent]
+Pelvis Open (P7)
+ ↓
+Excessive Rotation Reduces Space For The Arms.
+(과도한 회전으로 팔 전달 공간이 감소한다.)
+ ↓
+Hand Distance Close To Body (P7)
+Pelvis Open (P7)
+ ↓
+Maintaining Spine Inclination Requires Greater Side Bend As Pelvic Rotation Increases.
+(골반 회전이 증가할수록 척추각을 유지하기 위해 더 많은 측굴이 요구된다.)
+ ↓
+Side Bend Excessive (P7)
+Pelvis Open (P7)
+ ↓
+Players Increase Lead Wrist Flexion To Offset The Open Clubface.
+(열린 페이스를 보상하기 위해 리드 손목 굴곡을 더 사용한다.)
+ ↓
+Lead Wrist Flexion (P7)
+※ 보상
+Pelvis Open (P7)
+ ↓
+Some Players Lose Pelvic Depth While Continuing To Rotate.
+(골반이 계속 회전하는 과정에서 깊이를 잃는 패턴이 나타날 수 있다.)
+ ↓
+Early Extension (P6)
+[Low Confidence]
+Pelvis Open (P7)
+ ↓
+Repeated Excessive Side Bend Increases Lumbar Loading.
+(과도한 측굴이 반복되면 요추의 부담을 증가시킨다.)
+ ↓
+Lumbar Stress  ※ Biomechanical Concept (Injury Risk)</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="7" t="inlineStr">
+        <is>
+          <t>■ Strong Co-occurrence</t>
+        </is>
+      </c>
+      <c r="B32" s="8" t="inlineStr">
+        <is>
+          <t>★★★★★  Spin-out (P6)
+★★★★★  Pelvis Open (P6)
+★★★★★  Club Path Out-To-In (P7)
+★★★★☆  Club Face Open (P7)
+★★★★☆  Late Arm (P6)
+★★★★☆  Thorax Open (P7)</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="7" t="inlineStr">
+        <is>
+          <t>■ 추가 검증 포인트</t>
+        </is>
+      </c>
+      <c r="B33" s="8" t="inlineStr">
+        <is>
+          <t>- P6부터 이미 골반이 과도하게 열려 있었는가?
+- 골반 회전이 자발적 움직임인가, 페이스를 맞추기 위한 보상인가?
+- 골반 회전에 비해 팔 전달이 늦어지고 있는가?
+- 골반 회전과 흉곽 회전이 함께 증가하는가?
+- Out-To-In 스윙패스가 동반되는가?</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="7" t="inlineStr">
+        <is>
+          <t>■ 사고확장</t>
+        </is>
+      </c>
+      <c r="B34" s="8" t="inlineStr">
+        <is>
+          <t>- Open Pelvis 자체보다 어떤 메커니즘으로 형성됐는지가 더 중요하다.
+- 정상 회전(Pivot-driven)과 Spin-out에 의한 회전은 전혀 다른 패턴으로 해석한다.
+- Open Pelvis는 Upper Body·Arm Delivery·Face Control을 연결하는 Hub Feature.
+- 골반 회전 증가 → 팔 전달 지연 → 페이스 오픈 → 리드 손목 굴곡의 Compensation Chain이 반복된다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="8" t="inlineStr"/>
+      <c r="B35" s="8" t="inlineStr"/>
+    </row>
+    <row r="36">
+      <c r="A36" s="6" t="inlineStr">
+        <is>
+          <t>●</t>
+        </is>
+      </c>
+      <c r="B36" s="6" t="inlineStr">
+        <is>
+          <t>Pelvis Closed (P7)  ·  임팩트 시 골반 부족회전  ·  Family: Pelvis Rotation Family  ·  Pelvis / Rotation · Closed</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="7" t="inlineStr">
+        <is>
+          <t>■ 정의</t>
+        </is>
+      </c>
+      <c r="B37" s="8" t="inlineStr">
+        <is>
+          <t>임팩트(P7) 순간 골반이 기준보다 목표 방향으로 충분히 회전하지 못한 상태. 골반 회전량만 관찰. Pelvis Open (P7)의 단순 반대가 아니라 독립 생성 메커니즘을 가진다. Closed는 Target Line 기준.</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="7" t="inlineStr">
+        <is>
+          <t>■ 원인 추정</t>
+        </is>
+      </c>
+      <c r="B38" s="8" t="inlineStr">
+        <is>
+          <t>[High Confidence]
+Trail Pressure (트레일측 압력)
+ ↓
+Pressure Remaining On The Trail Side Restricts Pelvic Rotation.
+(압력이 트레일측에 남아 골반 회전을 제한한다.)
+ ↓
+Pelvis Closed (P7)
+Slide (슬라이드)
+ ↓
+Excessive Lateral Motion Reduces Available Pelvic Rotation.
+(과도한 측면 이동은 골반 회전을 감소시킨다.)
+ ↓
+Pelvis Closed (P7)
+Pelvis Closed (P6)
+ ↓
+The Limited Pelvic Rotation From P6 Continues Into Impact.
+(P6의 부족한 골반 회전이 임팩트까지 이어진다.)
+ ↓
+Pelvis Closed (P7)
+[Pattern Dependent]
+Club Face Closed (P7) (임팩트 시 클럽페이스 클로즈)
+ ↓
+Players Reduce Body Rotation To Prevent The Ball From Going Further Left.
+(볼이 더 왼쪽으로 가는 것을 막기 위해 몸 회전을 줄인다.)
+ ↓
+Pelvis Closed (P7)
+※ 보상
+Lead Leg Flexed (리드 무릎 굴곡 유지)
+ ↓
+Insufficient Lead Side Stabilization Limits Pelvic Rotation.
+(리드측 지지가 부족하면 골반 회전이 충분히 이루어지지 않는다.)
+ ↓
+Pelvis Closed (P7)
+Thorax Closed (P7) (흉곽 회전 부족)
+ ↓
+Limited Thorax Rotation Accompanies Limited Pelvic Rotation.
+(흉곽 회전 부족은 골반 회전 부족과 함께 나타난다.)
+ ↓
+Pelvis Closed (P7)</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="7" t="inlineStr">
+        <is>
+          <t>■ 이후 나타날 가능성</t>
+        </is>
+      </c>
+      <c r="B39" s="8" t="inlineStr">
+        <is>
+          <t>[High Confidence]
+Pelvis Closed (P7)
+ ↓
+Reduced Pelvic Rotation Increases Arm Dominance Through Impact.
+(골반 회전이 부족하면 팔의 개입이 증가한다.)
+ ↓
+Arm Dominant Pattern  ※ Coaching Knowledge
+Pelvis Closed (P7)
+ ↓
+Reduced Body Rotation Allows The Hands To Overtake The Pivot.
+(몸 회전이 부족하면 손이 몸보다 먼저 작용한다.)
+ ↓
+Early Release (P6)
+Pelvis Closed (P7)
+ ↓
+Limited Pivot Encourages Hand Manipulation Of The Clubface.
+(몸 회전 부족으로 손을 이용한 페이스 조절이 증가한다.)
+ ↓
+Lead Wrist Flexion (P7) / Lead Wrist Extension (P7)
+※ 리드 손목 보상(Modifier)
+[Pattern Dependent]
+Pelvis Closed (P7)
+ ↓
+Limited Rotation Reduces Available Swing Direction To The Left.
+(회전 부족은 스윙 방향을 충분히 좌측으로 만들기 어렵게 한다.)
+ ↓
+Club Path In-To-Out (P7) [Candidate]
+Pelvis Closed (P7)
+ ↓
+Limited Pelvic Rotation Reduces Space For Lead Arm Extension.
+(골반 회전이 부족하면 리드암이 펴질 공간이 부족해진다.)
+ ↓
+Chicken Wing (P7)</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="7" t="inlineStr">
+        <is>
+          <t>■ Strong Co-occurrence</t>
+        </is>
+      </c>
+      <c r="B40" s="8" t="inlineStr">
+        <is>
+          <t>★★★★★  Trail Pressure (트레일측 압력)
+★★★★★  Slide (슬라이드)
+★★★★★  Early Release (P6)
+★★★★☆  Arm Dominant Pattern (Coaching)</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="7" t="inlineStr">
+        <is>
+          <t>■ 추가 검증 포인트</t>
+        </is>
+      </c>
+      <c r="B41" s="8" t="inlineStr">
+        <is>
+          <t>- P6부터 골반 회전이 부족했는가?
+- 압력이 트레일측에 남아 있는가?
+- 회전 부족이 Mobility 때문인가, 보상 전략 때문인가?
+- 손 사용이 증가하는 패턴이 나타나는가?
+- 릴리즈를 손으로 해결하려는 경향이 있는가?</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="7" t="inlineStr">
+        <is>
+          <t>■ 사고확장</t>
+        </is>
+      </c>
+      <c r="B42" s="8" t="inlineStr">
+        <is>
+          <t>- Closed Pelvis는 회전 능력 부족만이 아니라 의도적 보상 전략으로도 나타난다.
+- Pressure-driven / Slide-driven / Compensation-driven / Mobility-driven으로 구분된다.
+- 골반 회전 부족은 Arm Dominance → Hand Manipulation → Release Compensation Chain을 형성한다.
+- Open Pelvis와 Closed Pelvis는 단순 반대가 아니라 서로 다른 메커니즘과 보상 전략을 가진 독립 Feature.</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="8" t="inlineStr"/>
+      <c r="B43" s="8" t="inlineStr"/>
+    </row>
+    <row r="44">
+      <c r="A44" s="6" t="inlineStr">
+        <is>
+          <t>●</t>
+        </is>
+      </c>
+      <c r="B44" s="6" t="inlineStr">
+        <is>
+          <t>Thorax Open (P7)  ·  임팩트 시 흉곽 과오픈  ·  Family: Thorax Rotation Family  ·  Thorax / Rotation · Open</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="7" t="inlineStr">
+        <is>
+          <t>■ 정의</t>
+        </is>
+      </c>
+      <c r="B45" s="8" t="inlineStr">
+        <is>
+          <t>임팩트(P7) 순간 흉곽(상체)이 목표 방향으로 과도하게 먼저 열린 상태. 흉곽 회전만 관찰. 국내 레슨의 '상체 엎어짐/먼저 열림/덤빔' 대표 Feature. Open은 Target Line 기준.</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="7" t="inlineStr">
+        <is>
+          <t>■ 원인 추정</t>
+        </is>
+      </c>
+      <c r="B46" s="8" t="inlineStr">
+        <is>
+          <t>[High Confidence]
+Thorax Open (P6)
+ ↓
+Early Thorax Rotation From P6 Continues Into Impact.
+(이른 흉곽 회전이 임팩트까지 유지된다.)
+ ↓
+Thorax Open (P7)
+Pelvis Open (P7) (임팩트 시 골반 과오픈)
+ ↓
+Excessive Pelvic Rotation Pulls The Thorax Into Earlier Rotation.
+(골반이 과도하게 회전하면서 상체도 함께 먼저 열린다.)
+ ↓
+Thorax Open (P7)
+Club Face Open (P7) (임팩트 시 클럽페이스 오픈)
+ ↓
+The Player Rotates The Body More Aggressively To Help Square The Clubface.
+(열린 페이스를 맞추기 위해 몸 회전을 더 적극적으로 사용한다.)
+ ↓
+Thorax Open (P7)
+※ 보상
+Spin-out (P6, 스핀아웃)
+ ↓
+The Lower Body Spins Without Bracing And Pulls The Thorax Open.
+(하체가 지지 없이 스핀아웃되며 상체를 함께 연다.)
+ ↓
+Thorax Open (P7)
+[Pattern Dependent]
+Late Arm (P6, 팔 하강 지연)
+ ↓
+Delayed Arm Delivery Allows Continued Thorax Rotation.
+(팔 전달이 늦어지는 동안 상체 회전이 계속 진행된다.)
+ ↓
+Thorax Open (P7)</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="7" t="inlineStr">
+        <is>
+          <t>■ 이후 나타날 가능성</t>
+        </is>
+      </c>
+      <c r="B47" s="8" t="inlineStr">
+        <is>
+          <t>[High Confidence]
+Thorax Open (P7)
+ ↓
+The Arms Cannot Keep Up With The Rotating Body.
+(몸 회전을 팔이 따라가지 못한다.)
+ ↓
+Late Arm (P6)
+Thorax Open (P7)
+ ↓
+Body Rotation Outpaces Clubface Rotation, Leaving The Face Open.
+(몸 회전이 페이스 회전보다 빨라 페이스가 열린 채 남는다.)
+ ↓
+Club Face Open (P7)
+Thorax Open (P7)
+ ↓
+The Club Travels Across The Ball From Outside The Target Line.
+(클럽이 목표선 바깥에서 볼을 가로지른다.)
+ ↓
+Club Path Out-To-In (P7) [Candidate]
+Thorax Open (P7)
+ ↓
+The Thorax Rotates Ahead Of The Arms, Leaving The Lead Arm Trapped Across The Chest.
+(상체 회전이 팔 전달보다 앞서면서 리드암이 가슴 앞에 갇힌다.)
+ ↓
+Chicken Wing (P7)
+[Pattern Dependent]
+Thorax Open (P7)
+ ↓
+The Upper Body Loses Forward Inclination During Rotation.
+(상체가 회전하면서 척추 전경각을 유지하지 못한다.)
+ ↓
+Spine Angle Loss (P6)</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="7" t="inlineStr">
+        <is>
+          <t>■ Strong Co-occurrence</t>
+        </is>
+      </c>
+      <c r="B48" s="8" t="inlineStr">
+        <is>
+          <t>★★★★★  Steep Shaft (P6)
+★★★★★  Late Arm (P6)
+★★★★★  Club Face Open (P7)
+★★★★★  Club Path Out-To-In (P7)
+★★★★☆  Chicken Wing (P7)</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="7" t="inlineStr">
+        <is>
+          <t>■ 추가 검증 포인트</t>
+        </is>
+      </c>
+      <c r="B49" s="8" t="inlineStr">
+        <is>
+          <t>- P6부터 상체가 먼저 열리고 있었는가?
+- 골반 회전에 의해 상체가 끌려 열린 것인가?
+- 열린 페이스를 보상하기 위한 상체 회전인가?
+- 팔이 상체 회전을 따라오지 못하는가?
+- 임팩트 이후 치킨윙이 동반되는가?</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="7" t="inlineStr">
+        <is>
+          <t>■ 사고확장</t>
+        </is>
+      </c>
+      <c r="B50" s="8" t="inlineStr">
+        <is>
+          <t>- 국내 레슨의 '상체가 엎어진다/먼저 열린다/덤빈다'는 대부분 동일 패턴을 의미한다.
+- Open Thorax는 Arm Delivery·Face Control·Swing Path를 모두 바꾸는 Hub Feature.
+- 원인은 Rotation-driven / Compensation-driven / Spin-out-driven으로 구분된다.
+- 레슨 대표 Chain: Open Thorax → Steep Shaft → Late Arm → Club Face Open → Out-To-In → Chicken Wing.
+- [Strong Co-occurrence 원칙] Open Pelvis↔Open Thorax는 생체역학적으론 연결되나 레슨에서 하체주도/상체주도로 갈리면 Strong Co-occurrence에서 제외한다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="8" t="inlineStr"/>
+      <c r="B51" s="8" t="inlineStr"/>
+    </row>
+    <row r="52">
+      <c r="A52" s="6" t="inlineStr">
+        <is>
+          <t>●</t>
+        </is>
+      </c>
+      <c r="B52" s="6" t="inlineStr">
+        <is>
+          <t>Thorax Closed (P7)  ·  임팩트 시 흉곽 부족회전  ·  Family: Thorax Rotation Family  ·  Thorax / Rotation · Closed</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="7" t="inlineStr">
+        <is>
+          <t>■ 정의</t>
+        </is>
+      </c>
+      <c r="B53" s="8" t="inlineStr">
+        <is>
+          <t>임팩트(P7) 순간 흉곽 회전이 기준보다 부족한 상태. 흉곽 회전만 관찰. Physical Limitation(못 도는: 가동성·압력이동·시퀀스)과 Movement Intent(안 도는: 의도적 상체 참기)를 구분해 해석한다. Closed는 Target Line 기준.</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="7" t="inlineStr">
+        <is>
+          <t>■ 원인 추정</t>
+        </is>
+      </c>
+      <c r="B54" s="8" t="inlineStr">
+        <is>
+          <t>[High Confidence]
+Early Extension (P6, 얼리 익스텐션)
+ ↓
+Loss Of Pelvic Space Restricts Continued Thorax Rotation.
+(골반 공간을 잃으면서 상체 회전을 끝까지 이어가기 어려워진다.)
+ ↓
+Thorax Closed (P7)
+※ Physical Limitation
+Casting (P6, 캐스팅)
+ ↓
+Early Club Release Reduces The Need For Continued Thorax Rotation.
+(클럽을 일찍 풀면서 상체 회전을 지속할 필요성이 감소한다.)
+ ↓
+Thorax Closed (P7)
+Casting (P6) + Early Extension (P6)
+ ↓
+Early Release Combined With Loss Of Pelvic Space Greatly Limits Thorax Rotation Through Impact.
+(캐스팅과 얼리 익스텐션이 함께 나타나면 임팩트까지 상체 회전이 크게 제한된다.)
+ ↓
+Thorax Closed (P7)
+※ 복합(대표 Archetype)
+[Pattern Dependent]
+Slide (슬라이드)
+ ↓
+Excessive Lateral Motion Interrupts Rotational Motion.
+(과도한 슬라이드는 회전 동작을 방해할 수 있다.)
+ ↓
+Thorax Closed (P7)
+[High Confidence]
+Thorax Closed (P6)
+ ↓
+The Limited Thorax Rotation From P6 Continues Into Impact.
+(P6의 부족한 상체 회전이 임팩트까지 이어진다.)
+ ↓
+Thorax Closed (P7)
+※ Physical Limitation
+[Pattern Dependent]
+Fear Of Opening Early (상체가 먼저 열리는 것에 대한 두려움)
+ ↓
+The Player Intentionally Holds The Chest Closed Through Impact.
+(상체가 열리면 안 된다는 의식으로 흉곽 회전을 의도적으로 억제한다.)
+ ↓
+Thorax Closed (P7)
+※ Movement Intent (안 도는)</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="7" t="inlineStr">
+        <is>
+          <t>■ 이후 나타날 가능성</t>
+        </is>
+      </c>
+      <c r="B55" s="8" t="inlineStr">
+        <is>
+          <t>[High Confidence]
+Thorax Closed (P7)
+ ↓
+Limited Thorax Rotation Directs The Club More From The Inside.
+(상체 회전이 부족하면 클럽이 더 안쪽에서 접근한다.)
+ ↓
+Club Path In-To-Out (P7) [Candidate]
+Thorax Closed (P7)
+ ↓
+Reduced Thorax Rotation Allows The Hands To Deliver Deeper Behind The Body.
+(상체 회전이 부족하면 손이 몸 뒤쪽 깊은 위치로 전달되기 쉽다.)
+ ↓
+Hand Depth Deep (P6)
+Thorax Closed (P7)
+ ↓
+Insufficient Thorax Rotation Pulls The Lead Arm Across The Body.
+(상체 회전이 부족하면 리드암이 몸쪽으로 당겨지며 접힌다.)
+ ↓
+Chicken Wing (P7)
+[Pattern Dependent]
+Thorax Closed (P7)
+ ↓
+If The Pelvis Continues Rotating While The Thorax Stays Closed, The Inside Delivery Becomes More Pronounced.
+(상체는 덜 돌고 골반만 계속 회전하면 인투아웃 전달이 더 커진다.)
+ ↓
+Club Path In-To-Out (P7) [Candidate] · 과도(Excessive)</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="7" t="inlineStr">
+        <is>
+          <t>■ Strong Co-occurrence</t>
+        </is>
+      </c>
+      <c r="B56" s="8" t="inlineStr">
+        <is>
+          <t>★★★★★  Early Extension (P6)
+★★★★★  Casting (P6)
+★★★★★  Club Path In-To-Out (P7)
+★★★★☆  Hand Depth Deep (P6)</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="7" t="inlineStr">
+        <is>
+          <t>■ 추가 검증 포인트</t>
+        </is>
+      </c>
+      <c r="B57" s="8" t="inlineStr">
+        <is>
+          <t>- 회전 부족이 Physical Limitation(못 도는)인가, Movement Intent(안 도는)인가?
+- 가동성·압력이동·시퀀스 문제인가?
+- '등을 지고/엎어치지 마라/몸을 참아라' 이미지의 영향인가?
+- Early Extension·Casting이 함께 나타나는가?
+- 골반은 계속 회전하는데 상체만 멈추는가?</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="7" t="inlineStr">
+        <is>
+          <t>■ 사고확장</t>
+        </is>
+      </c>
+      <c r="B58" s="8" t="inlineStr">
+        <is>
+          <t>- 많은 아마추어는 '상체를 오래 닫아야 한다'는 이미지로 흉곽 회전을 의도적으로 제한한다.
+- Closed Thorax는 회전 능력 부족보다 잘못된 움직임 이미지·보상 전략에서 발생하는 경우가 많다.
+- 골반과 흉곽의 회전 비율이 이후 Swing Path를 결정하는 중요한 요소가 된다.
+- Early Extension+Casting 동반형은 Closed Thorax가 높은 빈도로 함께 나타나는 하나의 Archetype.
+- ★LOCK 철학: 같은 Closed Thorax라도 Physical Limitation과 Movement Intent를 구분해 해석한다(코칭 방향이 달라짐).</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="8" t="inlineStr"/>
+      <c r="B59" s="8" t="inlineStr"/>
+    </row>
+    <row r="60">
+      <c r="A60" s="6" t="inlineStr">
+        <is>
+          <t>●</t>
+        </is>
+      </c>
+      <c r="B60" s="6" t="inlineStr">
+        <is>
+          <t>Standing Up (P7)  ·  몸 일어남  ·  Family: Posture / Axis Family  ·  Posture / Height · Rise (Pattern Feature)</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="7" t="inlineStr">
+        <is>
+          <t>■ 정의</t>
+        </is>
+      </c>
+      <c r="B61" s="8" t="inlineStr">
+        <is>
+          <t>임팩트(P7) 구간에서 척추 전경각이 소실되며 몸통 높이가 상승하는 현상. 관찰 대상은 척추각·몸통 높이(Height). Early Extension(골반 공간 변화)과 강한 Strong Co-occurrence를 가지나 관찰 대상이 다른 독립 Feature. 임팩트 반경(Radius)을 불안정하게 만드는 Hub.</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="7" t="inlineStr">
+        <is>
+          <t>■ 원인 추정</t>
+        </is>
+      </c>
+      <c r="B62" s="8" t="inlineStr">
+        <is>
+          <t>[High Confidence]
+Casting (P6, 캐스팅)
+ ↓
+Early Club Release Reduces Space For The Body To Stay Inclined.
+(클럽을 일찍 풀면서 척추각을 유지할 공간이 부족해진다.)
+ ↓
+Standing Up (P7)
+Closed Thorax (P7) (흉곽 회전 부족)
+ ↓
+Limited Thorax Rotation Encourages Vertical Extension To Complete The Swing.
+(상체 회전이 부족하면 회전을 대신해 몸을 세우는 보상이 나타난다.)
+ ↓
+Standing Up (P7)
+Hand Depth Deep (P6, 손 깊음)
+ ↓
+Deep Hand Delivery Reduces Available Space And Promotes Vertical Extension.
+(손이 깊게 전달되면 공간 확보를 위해 몸을 세우는 보상이 나타난다.)
+ ↓
+Standing Up (P7)
+Lead Pressure Excessive (P7) (리드측 압력 과다)
+ ↓
+The Body Rises To Relieve Excess Pressure On The Lead Side.
+(과도한 리드측 압력을 완화하기 위해 몸을 일으킨다.)
+ ↓
+Standing Up (P7)
+※ 보상
+[Pattern Dependent]
+Fat Contact Fear (뒷땅에 대한 두려움)
+ ↓
+Players Raise The Body To Avoid Striking The Ground.
+(뒷땅을 피하려는 의도로 몸을 세운다.)
+ ↓
+Standing Up (P7)
+※ 레슨 패턴</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="7" t="inlineStr">
+        <is>
+          <t>■ 이후 나타날 가능성</t>
+        </is>
+      </c>
+      <c r="B63" s="8" t="inlineStr">
+        <is>
+          <t>[High Confidence]
+Standing Up (P7)
+ ↓
+Standing Up Reduces Arm Space And Pushes The Handle Away From The Body.
+(몸이 일어나면서 팔 공간이 줄고 핸들이 몸에서 멀어진다.)
+ ↓
+Hand Distance Far From Body (P7)
+Standing Up (P7)
+ ↓
+Standing Up Reinforces Early Extension Rather Than Resolving It.
+(몸이 일어나는 패턴은 얼리 익스텐션을 더욱 고착시킨다.)
+ ↓
+Early Extension (P6)
+Standing Up (P7)
+ ↓
+Vertical Extension Reduces Available Arm Delivery Space.
+(몸이 세워지면서 팔이 지나갈 공간이 감소한다.)
+ ↓
+Chicken Wing (P7)  +  Trail Elbow Out (P7) [Candidate]
+[Pattern Dependent]
+Standing Up (P7)
+ ↓
+Losing Spine Inclination Makes Stable Face Control More Difficult.
+(척추각을 잃으면 페이스 제어가 불안정해진다.)
+ ↓
+Club Face Open (P7) / Club Face Closed (P7)</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="7" t="inlineStr">
+        <is>
+          <t>■ Strong Co-occurrence</t>
+        </is>
+      </c>
+      <c r="B64" s="8" t="inlineStr">
+        <is>
+          <t>★★★★★  Early Extension (P6)
+★★★★★  Casting (P6)
+★★★★☆  Hand Distance Far From Body (P7)
+★★★★☆  Hand Distance Close To Body (P7)</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="7" t="inlineStr">
+        <is>
+          <t>■ 추가 검증 포인트</t>
+        </is>
+      </c>
+      <c r="B65" s="8" t="inlineStr">
+        <is>
+          <t>- Standing Up은 임팩트 직전부터인가, 임팩트 이후인가?
+- 몸이 일어나는 원인이 공간 확보인가?
+- 손이 몸에서 멀어지는 현상이 동반되는가?
+- 뒷땅을 피하기 위한 보상 패턴인가?
+- Early Extension과 동일한 타이밍에서 발생하는가?</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="7" t="inlineStr">
+        <is>
+          <t>■ 사고확장</t>
+        </is>
+      </c>
+      <c r="B66" s="8" t="inlineStr">
+        <is>
+          <t>- Standing Up은 독립적 문제라기보다 '공간 확보를 위한 최후의 보상'인 경우가 많다.
+- 임팩트 반경(Radius)을 불안정하게 만드는 Feature이며, 그 결과 Heel/Toe/Thin/Shank 등 다양한 타점 문제가 발생한다.
+- ※ Heel · Toe · Thin · Shank 등 타점 결과는 Feature Chain이 아니라 Evidence Matrix에서 관리한다.
+- Early Extension이 골반 공간(Pelvic Space)의 변화라면 Standing Up은 척추각·몸통 높이의 변화로 구분한다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="8" t="inlineStr"/>
+      <c r="B67" s="8" t="inlineStr"/>
+    </row>
+    <row r="68">
+      <c r="A68" s="6" t="inlineStr">
+        <is>
+          <t>●</t>
+        </is>
+      </c>
+      <c r="B68" s="6" t="inlineStr">
+        <is>
+          <t>Forward Bend Excessive (P7)  ·  상체 과숙임  ·  Family: Posture / Axis Family  ·  Posture / Forward Bend · Excessive</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="7" t="inlineStr">
+        <is>
+          <t>■ 정의</t>
+        </is>
+      </c>
+      <c r="B69" s="8" t="inlineStr">
+        <is>
+          <t>임팩트(P7)에서 상체가 기준보다 과도하게 전방으로 숙여진 상태. 어드레스 대비 척추 전경각(Forward Bend)이 증가한 채 임팩트를 형성. Recovery Pattern과 Rotation Compensation 두 생성형이 있다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="7" t="inlineStr">
+        <is>
+          <t>■ 원인 추정</t>
+        </is>
+      </c>
+      <c r="B70" s="8" t="inlineStr">
+        <is>
+          <t>[High Confidence]
+Spine Angle Too Upright (P4, 백스윙 중 척추각 펴짐)
+ ↓
+The Player Re-Establishes Forward Bend To Reach The Ball.
+(볼에 도달하기 위해 상체를 다시 숙인다.)
+ ↓
+Forward Bend Excessive (P7)
+※ ① Recovery Pattern (대표)
+[Pattern Dependent]
+Spin-out (P6, 스핀아웃)
+ ↓
+Excessive Rotation Around The Trail Side Pulls The Upper Body Toward The Ball.
+(트레일측 축 회전이 과도해지며 상체가 볼 쪽으로 끌려 들어간다.)
+ ↓
+Forward Bend Excessive (P7)
+※ ② Rotation Compensation</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="7" t="inlineStr">
+        <is>
+          <t>■ 이후 나타날 가능성</t>
+        </is>
+      </c>
+      <c r="B71" s="8" t="inlineStr">
+        <is>
+          <t>[High Confidence]
+Forward Bend Excessive (P7)
+ ↓
+Forward Bending Moves The Hands Closer To The Body.
+(상체가 숙여지면서 손이 몸에 가까워진다.)
+ ↓
+Hand Distance Close To Body (P7)
+[Pattern Dependent]
+Forward Bend Excessive (P7)
+ ↓
+Reduced Arm Space Promotes A Steeper Delivery.
+(팔 공간이 감소하여 더 가파른 전달이 만들어진다.)
+ ↓
+Steep Shaft (P6)</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="7" t="inlineStr">
+        <is>
+          <t>■ Strong Co-occurrence</t>
+        </is>
+      </c>
+      <c r="B72" s="8" t="inlineStr">
+        <is>
+          <t>★★★★★  Spine Angle Too Upright (P4)
+★★★★★  Spin-out (P6)
+★★★★☆  Hand Distance Close To Body (P7)</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="7" t="inlineStr">
+        <is>
+          <t>■ 추가 검증 포인트</t>
+        </is>
+      </c>
+      <c r="B73" s="8" t="inlineStr">
+        <is>
+          <t>- P4에서 이미 척추각이 펴졌는가?
+- 다운스윙에서 상체가 다시 숙여지는 시점은 언제인가?
+- 숙임이 골반 굴곡인지 흉추 굴곡인지 구분이 필요한가?</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="7" t="inlineStr">
+        <is>
+          <t>■ 사고확장</t>
+        </is>
+      </c>
+      <c r="B74" s="8" t="inlineStr">
+        <is>
+          <t>- '상체 과숙임'은 두 생성형 가능: ① Recovery Pattern(P4에서 펴진 척추각을 임팩트 위해 다시 숙임) ② Rotation Compensation(스핀아웃/트레일축 과회전으로 축이 앞으로 무너짐).
+- 아마추어에서는 핵심 원인이 대체로 두 가지(척추각 회복·스핀아웃). 원인을 억지로 늘리기보다 강한 원인 2~3개를 명확히 정의한다.
+- 모든 Feature가 많은 원인을 가질 필요는 없다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="8" t="inlineStr"/>
+      <c r="B75" s="8" t="inlineStr"/>
+    </row>
+    <row r="76">
+      <c r="A76" s="6" t="inlineStr">
+        <is>
+          <t>●</t>
+        </is>
+      </c>
+      <c r="B76" s="6" t="inlineStr">
+        <is>
+          <t>Side Bend Excessive (P7)  ·  측굴 과다  ·  Family: Posture / Axis Family  ·  Thorax / Side Bend · Excessive</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" s="7" t="inlineStr">
+        <is>
+          <t>■ 정의</t>
+        </is>
+      </c>
+      <c r="B77" s="8" t="inlineStr">
+        <is>
+          <t>임팩트(P7)에서 상체의 트레일측 측면 굴곡(Side Bend)이 기준보다 과도하게 증가한 상태. 회전축·머리 위치 유지 보상으로 자주 나타난다. Amateur/Elite 생성형을 Player Type 태그로 구분한다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" s="7" t="inlineStr">
+        <is>
+          <t>■ 원인 추정</t>
+        </is>
+      </c>
+      <c r="B78" s="8" t="inlineStr">
+        <is>
+          <t>[High Confidence]
+Early Extension (P6, 얼리 익스텐션)
+ ↓
+Loss Of Pelvic Depth Increases Trail-Side Bend To Preserve Head Position And Swing Axis.
+(골반 깊이가 소실되면서 머리 위치와 스윙축을 유지하기 위해 측굴이 증가한다.)
+ ↓
+Side Bend Excessive (P7)
+※ [Player Type: Amateur]
+Open Pelvis (P7, 임팩트 시 골반 과오픈)
+ ↓
+Maintaining Spine Inclination Requires Greater Side Bend As Pelvic Rotation Increases.
+(골반 회전이 증가할수록 척추각을 유지하기 위해 더 많은 측굴이 요구된다.)
+ ↓
+Side Bend Excessive (P7)
+[Pattern Dependent]
+High Vertical Force Delivery (강한 수직력 전달)
+ ↓
+High Vertical Force Delivery Increases Side Bend To Match The Arm Rotation Radius.
+(강한 수직력 전달에서 팔의 회전 반경에 맞추기 위해 측굴이 증가한다.)
+ ↓
+Side Bend Excessive (P7)
+※ [Player Type: Elite]
+'Keep The Head Back' Image (머리를 뒤에 남기려는 이미지)
+ ↓
+Keeping The Head Back While The Lower Body Moves Forward Develops Side Bend To Connect The Upper And Lower Body.
+(하체는 앞으로 이동하고 머리는 뒤에 남기면서 상하체를 연결하기 위해 측굴이 형성된다.)
+ ↓
+Side Bend Excessive (P7)</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" s="7" t="inlineStr">
+        <is>
+          <t>■ 이후 나타날 가능성</t>
+        </is>
+      </c>
+      <c r="B79" s="8" t="inlineStr">
+        <is>
+          <t>[High Confidence]
+Side Bend Excessive (P7)
+ ↓
+Increased Side Bend Moves The Handle Closer To The Body.
+(측굴 증가로 손이 몸에 가까워진다.)
+ ↓
+Hand Distance Close To Body (P7)
+Side Bend Excessive (P7)
+ ↓
+Increased Side Bend Leaves The Trail Elbow Behind The Body.
+(측굴 증가로 트레일 팔꿈치가 몸보다 뒤처진다.)
+ ↓
+Trail Elbow Behind Body (P6)
+[Pattern Dependent]
+Side Bend Excessive (P7)
+ ↓
+Increased Side Bend Steepens The Delivery Path.
+(측굴 증가로 팔의 전달 경로가 더 가파르게 형성된다.)
+ ↓
+Steep Shaft (P6)</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" s="7" t="inlineStr">
+        <is>
+          <t>■ Strong Co-occurrence</t>
+        </is>
+      </c>
+      <c r="B80" s="8" t="inlineStr">
+        <is>
+          <t>★★★★★  Early Extension (P6)
+★★★★★  Hand Distance Close To Body (P7)
+★★★★☆  Trail Elbow Behind Body (P6)
+★★★★☆  Steep Shaft (P6)</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" s="7" t="inlineStr">
+        <is>
+          <t>■ 추가 검증 포인트</t>
+        </is>
+      </c>
+      <c r="B81" s="8" t="inlineStr">
+        <is>
+          <t>- 아마추어형(EE 보상·슬라이딩·머리 뒤 남기기)인가, 엘리트형(높은 탑·강한 수직력·능동 측굴)인가?
+- 골반 깊이 소실이 선행하는가?
+- 머리 위치·스윙축 유지를 위한 보상인가?</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" s="7" t="inlineStr">
+        <is>
+          <t>■ 사고확장</t>
+        </is>
+      </c>
+      <c r="B82" s="8" t="inlineStr">
+        <is>
+          <t>- 결과(Excessive Side Bend)는 같아도 생성 메커니즘은 아마추어와 선수에서 완전히 다르다.
+- [Player Type 태그] Amateur Pattern / Elite Pattern으로 해석 맥락(Context)을 부여한다. Feature 자체는 바꾸지 않는다.
+- 이 태그로 AI가 '아마추어형 Side Bend' vs '엘리트형 Side Bend'를 구분해 더 정확히 추론할 수 있다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" s="8" t="inlineStr"/>
+      <c r="B83" s="8" t="inlineStr"/>
+    </row>
+    <row r="84">
+      <c r="A84" s="6" t="inlineStr">
+        <is>
+          <t>●</t>
+        </is>
+      </c>
+      <c r="B84" s="6" t="inlineStr">
+        <is>
+          <t>Lead Pressure Excessive (P7)  ·  리드측 압력 과다  ·  Family: Pressure Family  ·  Pressure / Location · Lead · Excessive</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" s="7" t="inlineStr">
+        <is>
+          <t>■ 정의</t>
+        </is>
+      </c>
+      <c r="B85" s="8" t="inlineStr">
+        <is>
+          <t>임팩트(P7) 순간 압력이 정상 범위보다 과도하게 리드측(리드발)에 집중된 상태. 압력의 좌우 분포를 관찰. Rotation/Slide/Standing Up-driven으로 세분되며 Pressure Control Failure의 중간 Hub.</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" s="7" t="inlineStr">
+        <is>
+          <t>■ 원인 추정</t>
+        </is>
+      </c>
+      <c r="B86" s="8" t="inlineStr">
+        <is>
+          <t>[High Confidence]
+Slide (슬라이드)
+ ↓
+Excessive Lateral Shift Moves Pressure Too Far Onto The Lead Side.
+(과도한 슬라이드가 압력을 리드측으로 과도하게 이동시킨다.)
+ ↓
+Lead Pressure Excessive (P7)
+Open Pelvis (P7, 임팩트 시 골반 과오픈)
+ ↓
+Continued Pelvic Rotation Keeps Pressure Loaded On The Lead Side.
+(지속적인 골반 회전은 리드측 압력을 계속 유지한다.)
+ ↓
+Lead Pressure Excessive (P7)
+[Pattern Dependent]
+Standing Up (P7, 몸 일어남)
+ ↓
+Pushing Up Through The Lead Leg During Extension Increases Lead Side Pressure.
+(몸을 일으키는 과정에서 리드측을 강하게 밀어내며 압력이 증가한다.)
+ ↓
+Lead Pressure Excessive (P7)
+※ 패턴 의존
+[High Confidence]
+Trail Pressure Insufficient (P4, 트레일측 압력 부족)
+ ↓
+Insufficient Early-Phase Loading Forces Overcompensated Pressure Transfer In The Later Phases.
+(초기 구간에서 하중이 부족하면 후반 구간에서 과보상성 압력 이동이 발생한다.)
+ ↓
+Lead Pressure Excessive (P7)
+★ P4→P7 Pressure Chain
+[Pattern Dependent]
+Lead Hip Mobility Restriction / Glute·Adductor Inhibition (리드 고관절 가동성·둔근·내전근 저하)
+ ↓
+Poor Lead Side Stability Prevents Efficient Pressure Acceptance Through The Lead Heel.
+(리드측 안정성이 부족하면 압력을 뒤꿈치로 안정적으로 받아들이지 못하고 전족부에 집중된다.)
+ ↓
+Lead Pressure Excessive (P7)
+Open Thorax (P5, 상체 과회전)
+ ↓
+Aggressive Upper Body Rotation During Transition Drives Pressure Prematurely Onto The Lead Side.
+(전환 구간에서 상체를 급하게 회전시키면 압력이 리드측으로 조기에 이동한다.)
+ ↓
+Lead Pressure Excessive (P7)</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" s="7" t="inlineStr">
+        <is>
+          <t>■ 이후 나타날 가능성</t>
+        </is>
+      </c>
+      <c r="B87" s="8" t="inlineStr">
+        <is>
+          <t>[High Confidence]
+Lead Pressure Excessive (P7)
+ ↓
+Excessive Forward Pressure Reduces Rotational Freedom.
+(리드측 압력이 과도하면 회전의 자유도가 감소한다.)
+ ↓
+Pelvis Closed (P7)
+※ 추론
+Lead Pressure Excessive (P7)
+ ↓
+The Body Rises To Relieve Excess Pressure On The Lead Side.
+(과도한 리드측 압력을 완화하기 위해 몸을 일으킨다.)
+ ↓
+Standing Up (P7)</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" s="7" t="inlineStr">
+        <is>
+          <t>■ Strong Co-occurrence</t>
+        </is>
+      </c>
+      <c r="B88" s="8" t="inlineStr">
+        <is>
+          <t>★★★★★  Slide (슬라이드)
+★★★★★  Standing Up (P7)</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" s="7" t="inlineStr">
+        <is>
+          <t>■ 추가 검증 포인트</t>
+        </is>
+      </c>
+      <c r="B89" s="8" t="inlineStr">
+        <is>
+          <t>- 압력이 '얼마나'보다 '언제·어떻게' 형성됐는가?
+- Rotation-driven / Slide-driven / Standing Up-driven 중 무엇인가?
+- 백스윙(P4)에서 트레일측 압력이 충분히 형성됐는가?
+- 리드측 안정성(고관절·둔근)은 충분한가?</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" s="7" t="inlineStr">
+        <is>
+          <t>■ 사고확장</t>
+        </is>
+      </c>
+      <c r="B90" s="8" t="inlineStr">
+        <is>
+          <t>- Lead Pressure 자체는 좋고 나쁨이 아니라 '언제·어떻게' 형성됐는지가 중요하다.
+- Excessive Lead Pressure는 독립 문제가 아니라 Pressure Control Failure의 중간 Hub Feature.
+- ★재사용 Pressure Chain: Trail Pressure Insufficient (P4) → Lead Pressure Excessive (P7) → Standing Up (P7). P4와 P7을 직접 연결하는 축.
+- '초기 압력을 만들지 못하면 후반부 과보상으로 압력이 이동한다'는 일반 원리로 확장 가능.</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" s="8" t="inlineStr"/>
+      <c r="B91" s="8" t="inlineStr"/>
+    </row>
+    <row r="92">
+      <c r="A92" s="5" t="inlineStr">
+        <is>
+          <t>③ Arm / Hand Delivery (팔·손 전달)</t>
+        </is>
+      </c>
+      <c r="B92" s="5" t="inlineStr"/>
+    </row>
+    <row r="93">
+      <c r="A93" s="6" t="inlineStr">
+        <is>
+          <t>●</t>
+        </is>
+      </c>
+      <c r="B93" s="6" t="inlineStr">
+        <is>
+          <t>Hand Distance Close To Body (P7)  ·  손이 몸에 너무 가까움  ·  Family: Hand Position Family  ·  Hands / Distance · Close To Body</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" s="7" t="inlineStr">
+        <is>
+          <t>■ 정의</t>
+        </is>
+      </c>
+      <c r="B94" s="8" t="inlineStr">
+        <is>
+          <t>임팩트(P6~P7) 구간에서 손이 몸통(Torso)에 기준보다 과도하게 가까운 상태. 스윙 반경(Radius) 감소의 결과로 자주 나타난다. Distance는 Torso(몸) 기준.</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" s="7" t="inlineStr">
+        <is>
+          <t>■ 원인 추정</t>
+        </is>
+      </c>
+      <c r="B95" s="8" t="inlineStr">
+        <is>
+          <t>[High Confidence]
+Setup Hands Close (P1 Setup, 셋업 시 손이 가까움)
+ ↓
+A Close Hand Position At Address Is Maintained Throughout The Swing.
+(셋업에서 손이 몸에 가까우면 그 관계가 스윙 내내 유지된다.)
+ ↓
+Hand Distance Close To Body (P7)
+※ Setup Influence
+Chicken Wing (P7, 치킨윙)
+ ↓
+Lead Arm Flexion Pulls The Handle Closer To The Body Through Impact.
+(리드암이 접히면서 손이 몸쪽으로 당겨진다.)
+ ↓
+Hand Distance Close To Body (P7)
+Hand Depth Deep (P6, 손 깊음)
+ ↓
+Deep Hand Delivery Reduces The Distance Between The Hands And The Torso.
+(손이 깊게 전달되면서 몸과 손의 거리가 가까워진다.)
+ ↓
+Hand Distance Close To Body (P7)
+Late Arm (P6, 팔 하강 지연)
+ ↓
+Delayed Arm Delivery Traps The Hands Closer To The Body.
+(팔 전달이 늦어지면서 손이 몸 가까이 갇힌다.)
+ ↓
+Hand Distance Close To Body (P7)
+[Pattern Dependent]
+Trail Elbow Flexion (트레일 팔꿈치 과굴곡)
+ ↓
+Excessive Trail Elbow Flexion Reduces Swing Radius.
+(트레일 팔꿈치가 과도하게 굽혀지면 스윙 반경이 감소한다.)
+ ↓
+Hand Distance Close To Body (P7)
+Standing Up (P7, 몸 일어남)
+ ↓
+Vertical Extension Can Reduce Arm Radius Depending On The Compensation Pattern.
+(몸을 세우는 과정에서 보상 방식에 따라 팔 반경이 감소할 수 있다.)
+ ↓
+Hand Distance Close To Body (P7)
+※ 패턴 의존</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" s="7" t="inlineStr">
+        <is>
+          <t>■ 이후 나타날 가능성</t>
+        </is>
+      </c>
+      <c r="B96" s="8" t="inlineStr">
+        <is>
+          <t>[High Confidence]
+Hand Distance Close To Body (P7)
+ ↓
+Reduced Arm Radius Directs The Club More From The Inside.
+(팔 반경이 감소하면 클럽이 더 안쪽에서 접근한다.)
+ ↓
+Club Path In-To-Out (P7) [Candidate]
+Hand Distance Close To Body (P7)
+ ↓
+Reduced Swing Radius Restricts Lead Arm Extension.
+(스윙 반경이 감소하면서 리드암을 충분히 펼 공간이 부족해진다.)
+ ↓
+Chicken Wing (P7)</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" s="7" t="inlineStr">
+        <is>
+          <t>■ Strong Co-occurrence</t>
+        </is>
+      </c>
+      <c r="B97" s="8" t="inlineStr">
+        <is>
+          <t>★★★★★  Chicken Wing (P7)
+★★★★★  Hand Depth Deep (P6)
+★★★★★  Late Arm (P6)</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" s="7" t="inlineStr">
+        <is>
+          <t>■ 추가 검증 포인트</t>
+        </is>
+      </c>
+      <c r="B98" s="8" t="inlineStr">
+        <is>
+          <t>- 셋업부터 손이 몸에 가까운 구조인가?
+- P4부터 이미 손이 몸 가까이 전달되는가?
+- 리드암이 임팩트에서 접히는가?
+- 팔 하강 지연으로 손이 몸에 갇히는가?
+- 스윙 반경 감소가 원인인가, 회전 부족이 원인인가?
+- 토우 타점이 반복적으로 나타나는가? (→ Evidence Matrix)</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" s="7" t="inlineStr">
+        <is>
+          <t>■ 사고확장</t>
+        </is>
+      </c>
+      <c r="B99" s="8" t="inlineStr">
+        <is>
+          <t>- Hand Distance Close는 독립 문제가 아니라 스윙 반경(Swing Radius) 감소의 결과인 경우가 많다.
+- 생성 원인은 Setup / Deep Hands / Chicken Wing / Late Arm 등 다양하다.
+- '왜 스윙 반경이 줄었는가'를 해석하는 것이 Chain의 핵심.
+- 향후 Swing Radius를 Derived Parameter로 관리하면 Close/Far를 하나의 공통 메커니즘으로 설명 가능.</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" s="8" t="inlineStr"/>
+      <c r="B100" s="8" t="inlineStr"/>
+    </row>
+    <row r="101">
+      <c r="A101" s="6" t="inlineStr">
+        <is>
+          <t>●</t>
+        </is>
+      </c>
+      <c r="B101" s="6" t="inlineStr">
+        <is>
+          <t>Hand Distance Far From Body (P7)  ·  손이 몸에서 너무 멂  ·  Family: Hand Position Family  ·  Hands / Distance · Far From Body</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" s="7" t="inlineStr">
+        <is>
+          <t>■ 정의</t>
+        </is>
+      </c>
+      <c r="B102" s="8" t="inlineStr">
+        <is>
+          <t>임팩트(P6~P7) 구간에서 손이 몸통(Torso)에서 기준보다 과도하게 멀어진 상태. 스윙 반경 증가의 결과. Face Control 전략에 따라 이후 Chain이 분기(Branch)한다. Distance는 Torso(몸) 기준.</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" s="7" t="inlineStr">
+        <is>
+          <t>■ 원인 추정</t>
+        </is>
+      </c>
+      <c r="B103" s="8" t="inlineStr">
+        <is>
+          <t>[High Confidence]
+Setup Hands Far (P1 Setup, 셋업 시 손이 멂)
+ ↓
+The Initial Hand Distance At Address Is Maintained Throughout The Swing.
+(셋업에서 형성된 손과 몸의 거리가 스윙 내내 유지된다.)
+ ↓
+Hand Distance Far From Body (P7)
+※ Setup Influence
+Excessive In-To-Out (Club Path In-To-Out (P7), 과도한 인투아웃)
+ ↓
+An Excessive Inside Delivery Pushes The Hands Away From The Torso Through Impact.
+(과도한 인투아웃 전달은 손을 몸에서 멀어지게 만든다.)
+ ↓
+Hand Distance Far From Body (P7)
+Early Extension (P6, 얼리 익스텐션)
+ ↓
+Loss Of Pelvic Space Forces The Arms Away From The Body.
+(골반 공간을 잃으면서 팔이 몸에서 멀어지는 보상이 나타난다.)
+ ↓
+Hand Distance Far From Body (P7)
+[Pattern Dependent]
+Standing Up (P7, 몸 일어남)
+ ↓
+Some Standing-Up Compensation Patterns Increase Swing Radius Through Impact.
+(몸을 세우는 일부 보상 패턴에서는 스윙 반경이 증가한다.)
+ ↓
+Hand Distance Far From Body (P7)
+※ 패턴 의존</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" s="7" t="inlineStr">
+        <is>
+          <t>■ 이후 나타날 가능성</t>
+        </is>
+      </c>
+      <c r="B104" s="8" t="inlineStr">
+        <is>
+          <t>[High Confidence]
+Hand Distance Far From Body (P7)
+ ↓
+An Increased Swing Radius Makes Stable Clubface Control More Difficult.
+(스윙 반경이 증가하면 페이스를 안정적으로 제어하기 어려워진다.)
+ ↓
+Club Face Open (P7)
+── Branch (분기) ──
+The Chosen Compensation Strategy Determines The Subsequent Chain.
+(선택된 보상 전략이 이후 Chain을 결정한다.)
+[Pattern Dependent]
+Hand Distance Far From Body (P7)
+ ↓
+Players Actively Increase Clubface Closure To Prevent The Ball From Starting Right.
+(우측으로 밀리는 것을 보상하기 위해 적극적으로 페이스를 닫는다.)
+ ↓
+Club Face Closed (P7)
+※ Release Compensation</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" s="7" t="inlineStr">
+        <is>
+          <t>■ Strong Co-occurrence</t>
+        </is>
+      </c>
+      <c r="B105" s="8" t="inlineStr">
+        <is>
+          <t>★★★★★  Early Extension (P6)
+★★★★☆  Standing Up (P7)
+★★★★☆  Club Face Open (P7)
+★★★★☆  Club Path In-To-Out (P7) · Excessive</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" s="7" t="inlineStr">
+        <is>
+          <t>■ 추가 검증 포인트</t>
+        </is>
+      </c>
+      <c r="B106" s="8" t="inlineStr">
+        <is>
+          <t>- 셋업부터 손이 멀었는가?
+- 과도한 In-To-Out이 손을 밀어내는가?
+- 골반 공간 소실(EE)로 팔이 밀려나는가?
+- Face Control을 어떻게 하는가(무보상 vs 적극 릴리즈)?
+- 힐/생크 타점이 반복되는가? (→ Evidence Matrix)</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" s="7" t="inlineStr">
+        <is>
+          <t>■ 사고확장</t>
+        </is>
+      </c>
+      <c r="B107" s="8" t="inlineStr">
+        <is>
+          <t>- Hand Distance Far는 동일 Feature라도 Face Control 전략에 따라 Outcome이 분기하는 Branch Hub.
+- 무보상형: Club Face Open 유지. 적극 릴리즈형: Club Face Closed로 적응.
+- 이 분기가 이후 Archetype을 가른다: (EE형→Hand Far→Heel→Shank) vs (Excessive In-To-Out형→Hand Far→Face Open→Release Comp).
+- 같은 Hand Far라도 생성 원인이 다르면 전혀 다른 골퍼가 된다(핵심 해석 포인트).</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" s="8" t="inlineStr"/>
+      <c r="B108" s="8" t="inlineStr"/>
+    </row>
+    <row r="109">
+      <c r="A109" s="6" t="inlineStr">
+        <is>
+          <t>●</t>
+        </is>
+      </c>
+      <c r="B109" s="6" t="inlineStr">
+        <is>
+          <t>Chicken Wing (P7)  ·  치킨윙  ·  Family: Arm Delivery Family  ·  Arm / Lead Arm Extension · Loss (Pattern Feature)</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" s="7" t="inlineStr">
+        <is>
+          <t>■ 정의</t>
+        </is>
+      </c>
+      <c r="B110" s="8" t="inlineStr">
+        <is>
+          <t>임팩트(P7~P8) 이후 리드암이 정상적으로 신전되지 못하고 굴곡되며 접히는 패턴. 리드암의 신전 유지 여부를 관찰. 단순 팔꿈치 굴곡이 아닌 임팩트 이후 팔 전달 패턴. 회전 부족·분절 시퀀스 이상을 나타내는 대표 보상이며 Path+Face를 동시에 바꾸는 중간 Hub.</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" s="7" t="inlineStr">
+        <is>
+          <t>■ 원인 추정</t>
+        </is>
+      </c>
+      <c r="B111" s="8" t="inlineStr">
+        <is>
+          <t>[High Confidence]
+Late Arm (P6, 팔 하강 지연)
+ ↓
+Delayed Arm Delivery Prevents Full Lead Arm Extension Through Impact.
+(팔 전달이 늦어지면서 임팩트 이후 리드암이 충분히 신전되지 못한다.)
+ ↓
+Chicken Wing (P7)
+Hand Distance Close To Body (P7, 손이 몸에 가까움)
+ ↓
+Reduced Swing Radius Restricts Lead Arm Extension.
+(스윙 반경이 감소하면서 리드암을 충분히 펼 공간이 부족해진다.)
+ ↓
+Chicken Wing (P7)
+Thorax Open (P7, 임팩트 시 흉곽 과오픈)
+ ↓
+The Thorax Rotates Ahead Of The Arms, Leaving The Lead Arm Trapped Across The Chest.
+(상체 회전이 팔 전달보다 앞서면서 리드암이 가슴 앞에 갇힌다.)
+ ↓
+Chicken Wing (P7)
+Thorax Closed (P7, 흉곽 부족회전)
+ ↓
+Insufficient Thorax Rotation Pulls The Lead Arm Across The Body.
+(상체 회전이 부족하면 리드암이 몸쪽으로 당겨지며 접힌다.)
+ ↓
+Chicken Wing (P7)
+Closed Pelvis (P7, 골반 부족회전)
+ ↓
+Limited Pelvic Rotation Reduces Space For Lead Arm Extension.
+(골반 회전이 부족하면 리드암이 펴질 공간이 부족해진다.)
+ ↓
+Chicken Wing (P7)
+Arm Dominant Pattern (Coaching)
+ ↓
+An Arm-Dominant Delivery Limits Proper Body Rotation Through Impact.
+(팔 위주의 전달은 정상적인 몸 회전을 방해한다.)
+ ↓
+Chicken Wing (P7)
+[Pattern Dependent]
+Standing Up (P7, 몸 일어남)
+ ↓
+Vertical Extension Reduces Available Arm Delivery Space.
+(몸이 세워지면서 팔이 지나갈 공간이 감소한다.)
+ ↓
+Chicken Wing (P7)
+Club Face Open (P7, 임팩트 시 클럽페이스 오픈)
+ ↓
+Players Fold The Lead Arm To Help Close The Clubface.
+(열린 페이스를 닫기 위해 리드암을 접는 보상이 나타난다.)
+ ↓
+Chicken Wing (P7)
+※ 보상
+Late/Minimal Wrist Set (P2~P4, 코킹 부족)
+ ↓
+Without Proper Wrist Set And Arm Fold In The Backswing, The Segments Cannot Re-Extend Through Impact.
+(백스윙에서 적절한 코킹과 팔 접힘이 없으면 임팩트에서 각 분절이 자연스럽게 펴지지 못한다.)
+ ↓
+Chicken Wing (P7)
+★ Proper Fold→Proper Extension</t>
+        </is>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" s="7" t="inlineStr">
+        <is>
+          <t>■ 이후 나타날 가능성</t>
+        </is>
+      </c>
+      <c r="B112" s="8" t="inlineStr">
+        <is>
+          <t>[High Confidence]
+Chicken Wing (P7)
+ ↓
+Lead Arm Flexion Pulls The Handle Closer To The Body Through Impact.
+(리드암이 접히면서 손이 몸쪽으로 당겨진다.)
+ ↓
+Hand Distance Close To Body (P7)
+Chicken Wing (P7)
+ ↓
+Restricted Arm Extension Promotes Early Club Release.
+(팔 신전이 제한되면 클럽을 일찍 풀게 된다.)
+ ↓
+Casting (P6)
+[Pattern Dependent]
+Chicken Wing (P7)
+ ↓
+Limited Lead Arm Extension Directs The Club More Across The Ball.
+(리드암이 충분히 펴지지 못하면 클럽이 볼을 가로지르는 방향으로 접근하기 쉽다.)
+ ↓
+Club Path Out-To-In (P7) [Candidate]
+── Branch (분기) ──
+The Chosen Compensation Strategy Determines The Subsequent Chain.
+(선택된 보상 전략이 이후 Chain을 결정한다.)
+[Pattern Dependent]
+Chicken Wing (P7)
+ ↓
+Incomplete Lead Arm Extension Reduces Stable Club Release.
+(팔이 충분히 펴지지 못하면 릴리즈가 불안정해질 수 있다.)
+ ↓
+Club Face Open (P7)
+※ ① No Compensation
+Chicken Wing (P7)
+ ↓
+Players Close The Clubface Aggressively To Compensate For The Chicken Wing.
+(치킨윙을 보상하기 위해 임팩트에서 페이스를 적극적으로 닫는다.)
+ ↓
+Club Face Closed (P7)
+※ ② Face Compensation</t>
+        </is>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" s="7" t="inlineStr">
+        <is>
+          <t>■ Strong Co-occurrence</t>
+        </is>
+      </c>
+      <c r="B113" s="8" t="inlineStr">
+        <is>
+          <t>★★★★★  Thorax Closed (P7)
+★★★★★  Closed Pelvis (P7)
+★★★★★  Arm Dominant Pattern (Coaching)
+★★★★☆  Casting (P6)
+★★★★☆  Club Path Out-To-In (P7)
+★★★★☆  Club Face Open (P7)</t>
+        </is>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" s="7" t="inlineStr">
+        <is>
+          <t>■ 추가 검증 포인트</t>
+        </is>
+      </c>
+      <c r="B114" s="8" t="inlineStr">
+        <is>
+          <t>- 치킨윙이 상체 회전 부족에 의한 것인가?
+- 골반 회전 부족으로 팔이 접힌 것인가?
+- 팔 주도 스윙이 동반되는가?
+- 백스윙에서 코킹·오른팔 굴곡이 충분했는가?
+- 캐스팅이 함께 발생하는가?
+- 치킨윙 이후 아웃투인 스윙패스가 형성되는가?</t>
+        </is>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" s="7" t="inlineStr">
+        <is>
+          <t>■ 사고확장</t>
+        </is>
+      </c>
+      <c r="B115" s="8" t="inlineStr">
+        <is>
+          <t>- Chicken Wing은 팔 자체의 문제가 아니라 상·하체 회전 부족을 보상하는 대표 결과 Feature.
+- '백스윙에서 제대로 접혀야 다운스윙에서 제대로 펴진다' — Proper Fold → Proper Extension 시퀀스 원리(P2~P4 → P7~P8). Casting·Early Release로도 확장.
+- Chicken Wing은 Ball Flight를 직접 만드는 게 아니라 Swing Path와 Face Control을 동시에 바꾸는 중간 Hub.
+- '치킨윙=슬라이스'가 아니다. Path를 바꾸고 Face 보상 전략에 따라 Ball Flight가 갈라진다(Branch).</t>
+        </is>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" s="8" t="inlineStr"/>
+      <c r="B116" s="8" t="inlineStr"/>
+    </row>
+    <row r="117">
+      <c r="A117" s="5" t="inlineStr">
+        <is>
+          <t>④ Modifier Features (해석 보조)</t>
+        </is>
+      </c>
+      <c r="B117" s="5" t="inlineStr"/>
+    </row>
+    <row r="118">
+      <c r="A118" s="9" t="inlineStr">
+        <is>
+          <t>◆ Modifier</t>
+        </is>
+      </c>
+      <c r="B118" s="9" t="inlineStr">
+        <is>
+          <t>Lead Wrist Flexion (P7)  ·  리드 손목 굴곡  ·  Family: Wrist Modifier Family  ·  Wrist / Flexion (Modifier)</t>
+        </is>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" s="7" t="inlineStr">
+        <is>
+          <t>■ 정의</t>
+        </is>
+      </c>
+      <c r="B119" s="8" t="inlineStr">
+        <is>
+          <t>임팩트(P7) 순간 리드 손목이 굴곡(Flexion)된 상태. 관찰 대상은 리드 손목의 굴곡 정도이며, 좋고 나쁨을 의미하지 않는 Observation Feature이다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" s="7" t="inlineStr">
+        <is>
+          <t>■ Modifier 특성</t>
+        </is>
+      </c>
+      <c r="B120" s="8" t="inlineStr">
+        <is>
+          <t>Lead Wrist Flexion은 단독으로는 문제를 의미하지 않는다. Grip, Club Face, Release Pattern, Swing Intent 등 다른 Feature와 함께 해석되어야 한다. 원인/이후 가능성/Strong Co-occurrence보다 대표 해석 사례(Context)를 우선한다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" s="7" t="inlineStr">
+        <is>
+          <t>■ 대표 해석 사례</t>
+        </is>
+      </c>
+      <c r="B121" s="8" t="inlineStr">
+        <is>
+          <t>- Strong Grip + Lead Wrist Flexion → 일반적으로 자연스러운 임팩트 형태일 가능성이 높다.
+- Strong Grip + Excessive Lead Wrist Flexion → Club Face Closed 경향 증가 → Hook 가능성 증가.
+- Weak Grip + Lead Wrist Flexion → 열린 페이스를 보상하기 위한 전략일 가능성이 있다.
+- Club Face Open + Lead Wrist Flexion → 페이스를 Square로 만들기 위한 보상 패턴일 가능성이 있다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" s="7" t="inlineStr">
+        <is>
+          <t>■ 관련 Feature</t>
+        </is>
+      </c>
+      <c r="B122" s="8" t="inlineStr">
+        <is>
+          <t>- Strong Grip (P1 Setup)
+- Weak Grip (P1 Setup)
+- Club Face Open (P7)
+- Club Face Closed (P7)
+- Release Pattern</t>
+        </is>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" s="7" t="inlineStr">
+        <is>
+          <t>■ 사고확장</t>
+        </is>
+      </c>
+      <c r="B123" s="8" t="inlineStr">
+        <is>
+          <t>- Lead Wrist Flexion은 독립 문제 Feature가 아니라 다른 Observation의 의미를 변화시키는 Modifier Feature.
+- 동일 Flexion이라도 Grip·Release 전략에 따라 정상 동작이 될 수도, 과보상 패턴이 될 수도 있다.
+- AI가 '추론 대상이 아니라 해석 보조 Feature'로 이해하도록 Context-dependent Modifier로 관리한다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" s="8" t="inlineStr"/>
+      <c r="B124" s="8" t="inlineStr"/>
+    </row>
+    <row r="125">
+      <c r="A125" s="9" t="inlineStr">
+        <is>
+          <t>◆ Modifier</t>
+        </is>
+      </c>
+      <c r="B125" s="9" t="inlineStr">
+        <is>
+          <t>Lead Wrist Extension (P7)  ·  리드 손목 신전  ·  Family: Wrist Modifier Family  ·  Wrist / Extension (Modifier)</t>
+        </is>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" s="7" t="inlineStr">
+        <is>
+          <t>■ 정의</t>
+        </is>
+      </c>
+      <c r="B126" s="8" t="inlineStr">
+        <is>
+          <t>임팩트(P7) 순간 리드 손목이 신전(Extension)된 상태. 관찰 대상은 리드 손목의 신전 정도이며, 좋고 나쁨을 의미하지 않는 Observation Feature이다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" s="7" t="inlineStr">
+        <is>
+          <t>■ Modifier 특성</t>
+        </is>
+      </c>
+      <c r="B127" s="8" t="inlineStr">
+        <is>
+          <t>Lead Wrist Extension 역시 단독으로는 문제를 의미하지 않는다. Grip, Club Face, Release Pattern, Swing Intent 등과 함께 해석해야 한다. DOH에서는 Context-dependent Modifier Feature로 관리한다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" s="7" t="inlineStr">
+        <is>
+          <t>■ 대표 해석 사례</t>
+        </is>
+      </c>
+      <c r="B128" s="8" t="inlineStr">
+        <is>
+          <t>- Weak Grip + Lead Wrist Extension → Club Face Open 가능성 증가 → Push / Slice 가능성 증가.
+- Strong Grip + Lead Wrist Extension → 스트롱 그립의 닫힌 페이스를 완화하는 전략일 가능성이 있다.
+- Club Face Closed + Lead Wrist Extension → 닫힌 페이스를 보상하기 위한 움직임일 가능성이 있다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" s="7" t="inlineStr">
+        <is>
+          <t>■ 관련 Feature</t>
+        </is>
+      </c>
+      <c r="B129" s="8" t="inlineStr">
+        <is>
+          <t>- Strong Grip (P1 Setup)
+- Weak Grip (P1 Setup)
+- Club Face Open (P7)
+- Club Face Closed (P7)
+- Release Pattern</t>
+        </is>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" s="7" t="inlineStr">
+        <is>
+          <t>■ 사고확장</t>
+        </is>
+      </c>
+      <c r="B130" s="8" t="inlineStr">
+        <is>
+          <t>- Lead Wrist Extension도 독립 문제 Feature가 아니다.
+- 동일 손목 형태라도 Grip·Club Face 상태에 따라 완전히 다른 의미를 가질 수 있다.
+- 따라서 Context-dependent Modifier Feature로 관리한다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" s="8" t="inlineStr"/>
+      <c r="B131" s="8" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1731,7 +3652,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F108"/>
+  <dimension ref="A1:F121"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -5063,6 +6984,373 @@
         </is>
       </c>
     </row>
+    <row r="109">
+      <c r="A109" s="2" t="inlineStr">
+        <is>
+          <t>CMP</t>
+        </is>
+      </c>
+      <c r="B109" s="2" t="inlineStr">
+        <is>
+          <t>The Chosen Compensation Strategy Determines The Subsequent Chain.</t>
+        </is>
+      </c>
+      <c r="C109" s="2" t="inlineStr">
+        <is>
+          <t>선택된 보상 전략이 이후 Chain을 결정한다.</t>
+        </is>
+      </c>
+      <c r="D109" s="2" t="inlineStr"/>
+      <c r="E109" s="2" t="inlineStr">
+        <is>
+          <t>club_face_open_p7
+club_face_closed_p7
+hand_distance_far_p7
+chicken_wing_p7</t>
+        </is>
+      </c>
+      <c r="F109" s="2" t="inlineStr">
+        <is>
+          <t>★Branch Chain 분기 원인 표준 문장. 보상 전략 분기 지점에 삽입.</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" s="8" t="inlineStr">
+        <is>
+          <t>PRS</t>
+        </is>
+      </c>
+      <c r="B110" s="8" t="inlineStr">
+        <is>
+          <t>Earlier Lead Side Loading Allows Continued Pelvic Rotation.</t>
+        </is>
+      </c>
+      <c r="C110" s="8" t="inlineStr">
+        <is>
+          <t>리드측 압력이 충분하면 골반 회전이 계속 진행될 수 있다.</t>
+        </is>
+      </c>
+      <c r="D110" s="8" t="inlineStr"/>
+      <c r="E110" s="8" t="inlineStr">
+        <is>
+          <t>pelvis_open_p7</t>
+        </is>
+      </c>
+      <c r="F110" s="8" t="inlineStr">
+        <is>
+          <t>P7 Stage2 추가.</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" s="8" t="inlineStr">
+        <is>
+          <t>PST</t>
+        </is>
+      </c>
+      <c r="B111" s="8" t="inlineStr">
+        <is>
+          <t>Some Players Lose Pelvic Depth While Continuing To Rotate.</t>
+        </is>
+      </c>
+      <c r="C111" s="8" t="inlineStr">
+        <is>
+          <t>골반이 계속 회전하는 과정에서 깊이를 잃는 패턴이 나타날 수 있다.</t>
+        </is>
+      </c>
+      <c r="D111" s="8" t="inlineStr"/>
+      <c r="E111" s="8" t="inlineStr">
+        <is>
+          <t>pelvis_open_p7</t>
+        </is>
+      </c>
+      <c r="F111" s="8" t="inlineStr">
+        <is>
+          <t>P7 Stage2 추가. Open Pelvis→Early Extension(패턴).</t>
+        </is>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" s="8" t="inlineStr">
+        <is>
+          <t>ROT</t>
+        </is>
+      </c>
+      <c r="B112" s="8" t="inlineStr">
+        <is>
+          <t>Excessive Lateral Motion Reduces Available Pelvic Rotation.</t>
+        </is>
+      </c>
+      <c r="C112" s="8" t="inlineStr">
+        <is>
+          <t>과도한 측면 이동은 골반 회전을 감소시킨다.</t>
+        </is>
+      </c>
+      <c r="D112" s="8" t="inlineStr"/>
+      <c r="E112" s="8" t="inlineStr">
+        <is>
+          <t>pelvis_closed_p7</t>
+        </is>
+      </c>
+      <c r="F112" s="8" t="inlineStr">
+        <is>
+          <t>P7 Stage2 추가. Slide→Closed Pelvis.</t>
+        </is>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" s="8" t="inlineStr">
+        <is>
+          <t>ROT</t>
+        </is>
+      </c>
+      <c r="B113" s="8" t="inlineStr">
+        <is>
+          <t>Excessive Lateral Motion Interrupts Rotational Motion.</t>
+        </is>
+      </c>
+      <c r="C113" s="8" t="inlineStr">
+        <is>
+          <t>과도한 슬라이드는 회전 동작을 방해할 수 있다.</t>
+        </is>
+      </c>
+      <c r="D113" s="8" t="inlineStr"/>
+      <c r="E113" s="8" t="inlineStr">
+        <is>
+          <t>thorax_closed_p7</t>
+        </is>
+      </c>
+      <c r="F113" s="8" t="inlineStr">
+        <is>
+          <t>P7 Stage2 추가. Slide→Closed Thorax.</t>
+        </is>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" s="8" t="inlineStr">
+        <is>
+          <t>ROT</t>
+        </is>
+      </c>
+      <c r="B114" s="8" t="inlineStr">
+        <is>
+          <t>Loss Of Pelvic Space Restricts Continued Thorax Rotation.</t>
+        </is>
+      </c>
+      <c r="C114" s="8" t="inlineStr">
+        <is>
+          <t>골반 공간을 잃으면서 상체 회전을 끝까지 이어가기 어려워진다.</t>
+        </is>
+      </c>
+      <c r="D114" s="8" t="inlineStr"/>
+      <c r="E114" s="8" t="inlineStr">
+        <is>
+          <t>thorax_closed_p7</t>
+        </is>
+      </c>
+      <c r="F114" s="8" t="inlineStr">
+        <is>
+          <t>P7 Stage2 추가. Early Extension→Closed Thorax.</t>
+        </is>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" s="8" t="inlineStr">
+        <is>
+          <t>CLB</t>
+        </is>
+      </c>
+      <c r="B115" s="8" t="inlineStr">
+        <is>
+          <t>Early Club Release Reduces The Need For Continued Thorax Rotation.</t>
+        </is>
+      </c>
+      <c r="C115" s="8" t="inlineStr">
+        <is>
+          <t>클럽을 일찍 풀면서 상체 회전을 지속할 필요성이 감소한다.</t>
+        </is>
+      </c>
+      <c r="D115" s="8" t="inlineStr"/>
+      <c r="E115" s="8" t="inlineStr">
+        <is>
+          <t>thorax_closed_p7</t>
+        </is>
+      </c>
+      <c r="F115" s="8" t="inlineStr">
+        <is>
+          <t>P7 Stage2 추가. Casting→Closed Thorax.</t>
+        </is>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" s="8" t="inlineStr">
+        <is>
+          <t>ROT</t>
+        </is>
+      </c>
+      <c r="B116" s="8" t="inlineStr">
+        <is>
+          <t>Early Release Combined With Loss Of Pelvic Space Greatly Limits Thorax Rotation Through Impact.</t>
+        </is>
+      </c>
+      <c r="C116" s="8" t="inlineStr">
+        <is>
+          <t>캐스팅과 얼리 익스텐션이 함께 나타나면 임팩트까지 상체 회전이 크게 제한된다.</t>
+        </is>
+      </c>
+      <c r="D116" s="8" t="inlineStr"/>
+      <c r="E116" s="8" t="inlineStr">
+        <is>
+          <t>thorax_closed_p7</t>
+        </is>
+      </c>
+      <c r="F116" s="8" t="inlineStr">
+        <is>
+          <t>P7 Stage2 추가. Casting+EE 복합→Closed Thorax.</t>
+        </is>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" s="8" t="inlineStr">
+        <is>
+          <t>ROT</t>
+        </is>
+      </c>
+      <c r="B117" s="8" t="inlineStr">
+        <is>
+          <t>The Player Intentionally Holds The Chest Closed Through Impact.</t>
+        </is>
+      </c>
+      <c r="C117" s="8" t="inlineStr">
+        <is>
+          <t>상체가 열리면 안 된다는 의식으로 흉곽 회전을 의도적으로 억제한다.</t>
+        </is>
+      </c>
+      <c r="D117" s="8" t="inlineStr"/>
+      <c r="E117" s="8" t="inlineStr">
+        <is>
+          <t>thorax_closed_p7</t>
+        </is>
+      </c>
+      <c r="F117" s="8" t="inlineStr">
+        <is>
+          <t>P7 Stage2 추가. Movement Intent(안 도는)형.</t>
+        </is>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" s="8" t="inlineStr">
+        <is>
+          <t>SPC</t>
+        </is>
+      </c>
+      <c r="B118" s="8" t="inlineStr">
+        <is>
+          <t>Reduced Thorax Rotation Allows The Hands To Deliver Deeper Behind The Body.</t>
+        </is>
+      </c>
+      <c r="C118" s="8" t="inlineStr">
+        <is>
+          <t>상체 회전이 부족하면 손이 몸 뒤쪽 깊은 위치로 전달되기 쉽다.</t>
+        </is>
+      </c>
+      <c r="D118" s="8" t="inlineStr"/>
+      <c r="E118" s="8" t="inlineStr">
+        <is>
+          <t>thorax_closed_p7</t>
+        </is>
+      </c>
+      <c r="F118" s="8" t="inlineStr">
+        <is>
+          <t>P7 Stage2 추가. Closed Thorax→Hand Depth Deep.</t>
+        </is>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" s="8" t="inlineStr">
+        <is>
+          <t>SPC</t>
+        </is>
+      </c>
+      <c r="B119" s="8" t="inlineStr">
+        <is>
+          <t>Vertical Extension Can Reduce Arm Radius Depending On The Compensation Pattern.</t>
+        </is>
+      </c>
+      <c r="C119" s="8" t="inlineStr">
+        <is>
+          <t>몸을 세우는 과정에서 보상 방식에 따라 팔 반경이 감소할 수 있다.</t>
+        </is>
+      </c>
+      <c r="D119" s="8" t="inlineStr"/>
+      <c r="E119" s="8" t="inlineStr">
+        <is>
+          <t>hand_distance_close_p7</t>
+        </is>
+      </c>
+      <c r="F119" s="8" t="inlineStr">
+        <is>
+          <t>P7 Stage2 추가. Standing Up→Hand Distance Close(패턴).</t>
+        </is>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" s="8" t="inlineStr">
+        <is>
+          <t>CLB</t>
+        </is>
+      </c>
+      <c r="B120" s="8" t="inlineStr">
+        <is>
+          <t>Limited Lead Arm Extension Directs The Club More Across The Ball.</t>
+        </is>
+      </c>
+      <c r="C120" s="8" t="inlineStr">
+        <is>
+          <t>리드암이 충분히 펴지지 못하면 클럽이 볼을 가로지르는 방향으로 접근하기 쉽다.</t>
+        </is>
+      </c>
+      <c r="D120" s="8" t="inlineStr"/>
+      <c r="E120" s="8" t="inlineStr">
+        <is>
+          <t>chicken_wing_p7</t>
+        </is>
+      </c>
+      <c r="F120" s="8" t="inlineStr">
+        <is>
+          <t>P7 Stage2 추가. Chicken Wing→Out-To-In.</t>
+        </is>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" s="8" t="inlineStr">
+        <is>
+          <t>CLB</t>
+        </is>
+      </c>
+      <c r="B121" s="8" t="inlineStr">
+        <is>
+          <t>Incomplete Lead Arm Extension Reduces Stable Club Release.</t>
+        </is>
+      </c>
+      <c r="C121" s="8" t="inlineStr">
+        <is>
+          <t>팔이 충분히 펴지지 못하면 릴리즈가 불안정해질 수 있다.</t>
+        </is>
+      </c>
+      <c r="D121" s="8" t="inlineStr"/>
+      <c r="E121" s="8" t="inlineStr">
+        <is>
+          <t>chicken_wing_p7</t>
+        </is>
+      </c>
+      <c r="F121" s="8" t="inlineStr">
+        <is>
+          <t>P7 Stage2 추가. Chicken Wing→Face Open(No Comp).</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -5074,16 +7362,17 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G17"/>
+  <dimension ref="A1:H17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
-    <col width="26" customWidth="1" min="2" max="2"/>
+    <col width="30" customWidth="1" min="2" max="2"/>
     <col width="16" customWidth="1" min="3" max="3"/>
-    <col width="66" customWidth="1" min="4" max="4"/>
+    <col width="62" customWidth="1" min="4" max="4"/>
     <col width="12" customWidth="1" min="5" max="5"/>
     <col width="20" customWidth="1" min="6" max="6"/>
-    <col width="40" customWidth="1" min="7" max="7"/>
+    <col width="18" customWidth="1" min="7" max="7"/>
+    <col width="38" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -5114,10 +7403,15 @@
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
+          <t>Family</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
           <t>Layer/Status</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>비고</t>
         </is>
@@ -5151,10 +7445,15 @@
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
+          <t>Hand Position Family</t>
+        </is>
+      </c>
+      <c r="G2" s="2" t="inlineStr">
+        <is>
           <t>Core</t>
         </is>
       </c>
-      <c r="G2" s="2" t="inlineStr">
+      <c r="H2" s="2" t="inlineStr">
         <is>
           <t>Impact Geometry. Handle Position Family 중심(Hub) 후보. [Ref: Ball/Target Line]</t>
         </is>
@@ -5188,10 +7487,15 @@
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
+          <t>Club Face Family</t>
+        </is>
+      </c>
+      <c r="G3" s="2" t="inlineStr">
+        <is>
           <t>Core</t>
         </is>
       </c>
-      <c r="G3" s="2" t="inlineStr">
+      <c r="H3" s="2" t="inlineStr">
         <is>
           <t>Hub Feature. 보상전략 3분기(Rotation/Hand Release/No Comp). [Ref: Target Line]</t>
         </is>
@@ -5225,10 +7529,15 @@
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
+          <t>Club Face Family</t>
+        </is>
+      </c>
+      <c r="G4" s="2" t="inlineStr">
+        <is>
           <t>Core</t>
         </is>
       </c>
-      <c r="G4" s="2" t="inlineStr">
+      <c r="H4" s="2" t="inlineStr">
         <is>
           <t>Hub Feature. 보상전략 3분기(Path/Counter/No Comp). [Ref: Target Line]</t>
         </is>
@@ -5262,10 +7571,15 @@
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
+          <t>Pelvis Rotation Family</t>
+        </is>
+      </c>
+      <c r="G5" s="2" t="inlineStr">
+        <is>
           <t>Core</t>
         </is>
       </c>
-      <c r="G5" s="2" t="inlineStr">
+      <c r="H5" s="2" t="inlineStr">
         <is>
           <t>Hub Feature. Pivot-driven vs Spin-out-driven 구분. [Ref: Target Line]</t>
         </is>
@@ -5299,10 +7613,15 @@
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
+          <t>Pelvis Rotation Family</t>
+        </is>
+      </c>
+      <c r="G6" s="2" t="inlineStr">
+        <is>
           <t>Core</t>
         </is>
       </c>
-      <c r="G6" s="2" t="inlineStr">
+      <c r="H6" s="2" t="inlineStr">
         <is>
           <t>Physical Limitation vs Movement Intent 구분. [Ref: Target Line]</t>
         </is>
@@ -5336,10 +7655,15 @@
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
+          <t>Thorax Rotation Family</t>
+        </is>
+      </c>
+      <c r="G7" s="2" t="inlineStr">
+        <is>
           <t>Core</t>
         </is>
       </c>
-      <c r="G7" s="2" t="inlineStr">
+      <c r="H7" s="2" t="inlineStr">
         <is>
           <t>Hub Feature. Rotation/Compensation/Spin-out-driven. [Ref: Target Line]</t>
         </is>
@@ -5373,10 +7697,15 @@
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
+          <t>Thorax Rotation Family</t>
+        </is>
+      </c>
+      <c r="G8" s="2" t="inlineStr">
+        <is>
           <t>Core</t>
         </is>
       </c>
-      <c r="G8" s="2" t="inlineStr">
+      <c r="H8" s="2" t="inlineStr">
         <is>
           <t>★LOCK 철학: Physical Limitation vs Movement Intent. [Ref: Target Line]</t>
         </is>
@@ -5410,10 +7739,15 @@
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
+          <t>Posture / Axis Family</t>
+        </is>
+      </c>
+      <c r="G9" s="2" t="inlineStr">
+        <is>
           <t>Core</t>
         </is>
       </c>
-      <c r="G9" s="2" t="inlineStr">
+      <c r="H9" s="2" t="inlineStr">
         <is>
           <t>Pattern Feature(명칭 유지). 임팩트 반경(Radius) 불안정 Hub. [Ref: 척추각/몸통 높이]</t>
         </is>
@@ -5447,10 +7781,15 @@
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
+          <t>Posture / Axis Family</t>
+        </is>
+      </c>
+      <c r="G10" s="2" t="inlineStr">
+        <is>
           <t>Core</t>
         </is>
       </c>
-      <c r="G10" s="2" t="inlineStr">
+      <c r="H10" s="2" t="inlineStr">
         <is>
           <t>[Ref: 척추 전경각(Forward Bend)]</t>
         </is>
@@ -5484,10 +7823,15 @@
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
+          <t>Posture / Axis Family</t>
+        </is>
+      </c>
+      <c r="G11" s="2" t="inlineStr">
+        <is>
           <t>Core</t>
         </is>
       </c>
-      <c r="G11" s="2" t="inlineStr">
+      <c r="H11" s="2" t="inlineStr">
         <is>
           <t>Player Type 태그(Amateur/Elite). [Ref: 트레일측 측굴]</t>
         </is>
@@ -5521,10 +7865,15 @@
       </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
+          <t>Pressure Family</t>
+        </is>
+      </c>
+      <c r="G12" s="2" t="inlineStr">
+        <is>
           <t>Core</t>
         </is>
       </c>
-      <c r="G12" s="2" t="inlineStr">
+      <c r="H12" s="2" t="inlineStr">
         <is>
           <t>P4 Trail Pressure Insufficient→P7 Pressure Chain 핵심. [Ref: 좌우 압력 분포]</t>
         </is>
@@ -5558,10 +7907,15 @@
       </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
+          <t>Hand Position Family</t>
+        </is>
+      </c>
+      <c r="G13" s="2" t="inlineStr">
+        <is>
           <t>Core</t>
         </is>
       </c>
-      <c r="G13" s="2" t="inlineStr">
+      <c r="H13" s="2" t="inlineStr">
         <is>
           <t>임팩트 반경 감소 Hub→Toe/In-To-Out. [Ref: Torso]</t>
         </is>
@@ -5595,10 +7949,15 @@
       </c>
       <c r="F14" s="2" t="inlineStr">
         <is>
+          <t>Hand Position Family</t>
+        </is>
+      </c>
+      <c r="G14" s="2" t="inlineStr">
+        <is>
           <t>Core</t>
         </is>
       </c>
-      <c r="G14" s="2" t="inlineStr">
+      <c r="H14" s="2" t="inlineStr">
         <is>
           <t>Branch Chain Hub→Heel/Shank 또는 Push Draw. [Ref: Torso]</t>
         </is>
@@ -5632,10 +7991,15 @@
       </c>
       <c r="F15" s="2" t="inlineStr">
         <is>
+          <t>Arm Delivery Family</t>
+        </is>
+      </c>
+      <c r="G15" s="2" t="inlineStr">
+        <is>
           <t>Core</t>
         </is>
       </c>
-      <c r="G15" s="2" t="inlineStr">
+      <c r="H15" s="2" t="inlineStr">
         <is>
           <t>Pattern Feature(명칭 유지). 회전 부족·분절 시퀀스 이상의 대표 보상. Path+Face 동시 변화 Hub.</t>
         </is>
@@ -5669,10 +8033,15 @@
       </c>
       <c r="F16" s="2" t="inlineStr">
         <is>
+          <t>Wrist Modifier Family</t>
+        </is>
+      </c>
+      <c r="G16" s="2" t="inlineStr">
+        <is>
           <t>Modifier</t>
         </is>
       </c>
-      <c r="G16" s="2" t="inlineStr">
+      <c r="H16" s="2" t="inlineStr">
         <is>
           <t>5-섹션 템플릿(원인/이후 없음). Context-dependent.</t>
         </is>
@@ -5706,10 +8075,15 @@
       </c>
       <c r="F17" s="2" t="inlineStr">
         <is>
+          <t>Wrist Modifier Family</t>
+        </is>
+      </c>
+      <c r="G17" s="2" t="inlineStr">
+        <is>
           <t>Modifier</t>
         </is>
       </c>
-      <c r="G17" s="2" t="inlineStr">
+      <c r="H17" s="2" t="inlineStr">
         <is>
           <t>5-섹션 템플릿(원인/이후 없음). Context-dependent.</t>
         </is>
@@ -6206,7 +8580,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B49"/>
+  <dimension ref="A1:B51"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -6365,239 +8739,247 @@
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>동일 Feature라도 보상 전략에 따라 이후 Chain이 분기하면 단일 결과로 단정하지 않고 Branch Chain으로 작성한다.</t>
+          <t>동일 Feature라도 보상 전략에 따라 이후 Chain이 분기하면 단일 결과로 단정하지 않고 Branch Chain으로 작성한다. 분기 지점에는 분기 원인을 설명하는 Mechanism 한 줄을 삽입한 뒤 각 Branch를 나열한다. (표준 문장: The Chosen Compensation Strategy Determines The Subsequent Chain.)</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>⑧ Confidence 등급</t>
+          <t>⑧ Confidence 등급(3단계)</t>
         </is>
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>[High Confidence]=생체역학적으로 확실 · [Medium Confidence]=레슨상 자주 · [Low Confidence / Pattern Dependent] 또는 ※추론=특정 유형. 원인/이후 Chain에 등급을 명시한다.</t>
+          <t>[High Confidence]=생체역학적으로 확실 · [Pattern Dependent]=특정 유형/패턴에서 관찰 · [Low Confidence]=약한 추론. 원인/이후 Chain에 등급을 명시한다.</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>⑨ Feature 신설 3원칙</t>
+          <t>⑨-2 Chain 종료 규칙</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>새 Feature는 ①Observation이 다른가 ②새 Chain을 생성하는가 ③새 추론 정보(Information Gain)를 주는가 를 모두 만족할 때만 만든다. 아니면 기존 Feature 통합을 우선한다. 애매하면 임의 결정 없이 질문 후 진행한다.</t>
+          <t>Feature Chain은 Feature → Mechanism → Feature 에서 종료한다(Candidate/Derived Parameter 노드 포함 가능). Ball Flight·Impact Strike·Ground Contact(Evidence Layer)는 Chain에 포함하지 않고 Evidence Matrix에서만 관리한다.</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="2" t="inlineStr"/>
-      <c r="B17" s="2" t="inlineStr"/>
+      <c r="A17" s="2" t="inlineStr">
+        <is>
+          <t>⑩-2 Feature Family</t>
+        </is>
+      </c>
+      <c r="B17" s="2" t="inlineStr">
+        <is>
+          <t>모든 Feature Header에 Family 필드를 두어 Object 분류를 명확히 한다. Family: Hand Position · Club Face · Pelvis Rotation · Thorax Rotation · Posture/Axis · Pressure · Arm Delivery · Wrist Modifier.</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>Coordinate Reference Vocabulary (Axis 기준점)</t>
-        </is>
-      </c>
-      <c r="B18" s="2" t="inlineStr"/>
+          <t>⑨ Feature 신설 3원칙</t>
+        </is>
+      </c>
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t>새 Feature는 ①Observation이 다른가 ②새 Chain을 생성하는가 ③새 추론 정보(Information Gain)를 주는가 를 모두 만족할 때만 만든다. 아니면 기존 Feature 통합을 우선한다. 애매하면 임의 결정 없이 질문 후 진행한다.</t>
+        </is>
+      </c>
     </row>
     <row r="19">
-      <c r="A19" s="2" t="inlineStr">
-        <is>
-          <t>Direction (Forward / Backward)</t>
-        </is>
-      </c>
-      <c r="B19" s="2" t="inlineStr">
-        <is>
-          <t>Ball / Target Line 기준</t>
-        </is>
-      </c>
+      <c r="A19" s="2" t="inlineStr"/>
+      <c r="B19" s="2" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>Lateral (In / Out)</t>
-        </is>
-      </c>
-      <c r="B20" s="2" t="inlineStr">
-        <is>
-          <t>Target Line 기준</t>
-        </is>
-      </c>
+          <t>Coordinate Reference Vocabulary (Axis 기준점)</t>
+        </is>
+      </c>
+      <c r="B20" s="2" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>Rotation (Open / Closed)</t>
+          <t>Direction (Forward / Backward)</t>
         </is>
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>Target Line 기준</t>
+          <t>Ball / Target Line 기준</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>Distance (Close To Body / Far From Body)</t>
+          <t>Lateral (In / Out)</t>
         </is>
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>Torso(몸) 기준</t>
+          <t>Target Line 기준</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>Depth (Deep / Shallow)</t>
+          <t>Rotation (Open / Closed)</t>
         </is>
       </c>
       <c r="B23" s="2" t="inlineStr">
         <is>
-          <t>Thorax(몸 회전) 기준</t>
+          <t>Target Line 기준</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>Height (High / Low)</t>
+          <t>Distance (Close To Body / Far From Body)</t>
         </is>
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t>척추각 / 몸통 높이 기준</t>
+          <t>Torso(몸) 기준</t>
         </is>
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="2" t="inlineStr"/>
-      <c r="B25" s="2" t="inlineStr"/>
+      <c r="A25" s="2" t="inlineStr">
+        <is>
+          <t>Depth (Deep / Shallow)</t>
+        </is>
+      </c>
+      <c r="B25" s="2" t="inlineStr">
+        <is>
+          <t>Thorax(몸 회전) 기준</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>Mechanism Categories (P7)</t>
-        </is>
-      </c>
-      <c r="B26" s="2" t="inlineStr"/>
+          <t>Height (High / Low)</t>
+        </is>
+      </c>
+      <c r="B26" s="2" t="inlineStr">
+        <is>
+          <t>척추각 / 몸통 높이 기준</t>
+        </is>
+      </c>
     </row>
     <row r="27">
-      <c r="A27" s="2" t="inlineStr">
-        <is>
-          <t>ROT</t>
-        </is>
-      </c>
-      <c r="B27" s="2" t="inlineStr">
-        <is>
-          <t>Rotation — 골반/흉곽 회전(Amount·Timing·Velocity·Axis)</t>
-        </is>
-      </c>
+      <c r="A27" s="2" t="inlineStr"/>
+      <c r="B27" s="2" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>PRS</t>
-        </is>
-      </c>
-      <c r="B28" s="2" t="inlineStr">
-        <is>
-          <t>Pressure — 리드/트레일 하중 및 압력 분포</t>
-        </is>
-      </c>
+          <t>Mechanism Categories (P7)</t>
+        </is>
+      </c>
+      <c r="B28" s="2" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
         <is>
-          <t>ARM</t>
+          <t>ROT</t>
         </is>
       </c>
       <c r="B29" s="2" t="inlineStr">
         <is>
-          <t>Arm Delivery — 팔·손·팔꿈치의 전달과 신전</t>
+          <t>Rotation — 골반/흉곽 회전(Amount·Timing·Velocity·Axis)</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>CLB</t>
+          <t>PRS</t>
         </is>
       </c>
       <c r="B30" s="2" t="inlineStr">
         <is>
-          <t>Club Delivery — 페이스 방향·경로(Path)·릴리즈·로프트</t>
+          <t>Pressure — 리드/트레일 하중 및 압력 분포</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
         <is>
-          <t>SPC</t>
+          <t>ARM</t>
         </is>
       </c>
       <c r="B31" s="2" t="inlineStr">
         <is>
-          <t>Space — 몸-팔 전달 공간 및 스윙 반경(Radius)</t>
+          <t>Arm Delivery — 팔·손·팔꿈치의 전달과 신전</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>LOD</t>
+          <t>CLB</t>
         </is>
       </c>
       <c r="B32" s="2" t="inlineStr">
         <is>
-          <t>Loading — 리드/트레일측 하중 수용과 안정</t>
+          <t>Club Delivery — 페이스 방향·경로(Path)·릴리즈·로프트</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
         <is>
-          <t>CMP</t>
+          <t>SPC</t>
         </is>
       </c>
       <c r="B33" s="2" t="inlineStr">
         <is>
-          <t>Compensation — 페이스·회전·손·몸의 보상 동작</t>
+          <t>Space — 몸-팔 전달 공간 및 스윙 반경(Radius)</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>PST</t>
+          <t>LOD</t>
         </is>
       </c>
       <c r="B34" s="2" t="inlineStr">
         <is>
-          <t>Posture / Axis — 척추각·측굴·전경·몸통 높이(신규, P7에서 신설)</t>
+          <t>Loading — 리드/트레일측 하중 수용과 안정</t>
         </is>
       </c>
     </row>
     <row r="35">
-      <c r="A35" s="2" t="inlineStr"/>
-      <c r="B35" s="2" t="inlineStr"/>
+      <c r="A35" s="2" t="inlineStr">
+        <is>
+          <t>CMP</t>
+        </is>
+      </c>
+      <c r="B35" s="2" t="inlineStr">
+        <is>
+          <t>Compensation — 페이스·회전·손·몸의 보상 동작</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>Player Type 태그(신규)</t>
+          <t>PST</t>
         </is>
       </c>
       <c r="B36" s="2" t="inlineStr">
         <is>
-          <t>같은 Feature라도 생성 메커니즘이 선수/아마추어에서 다를 때 [Player Type: Amateur/Elite] 태그로 해석 맥락(Context)을 부여한다. Feature 자체는 바꾸지 않는다. (예: Side Bend Excessive (P7))</t>
+          <t>Posture / Axis — 척추각·측굴·전경·몸통 높이(신규, P7에서 신설)</t>
         </is>
       </c>
     </row>
@@ -6608,134 +8990,150 @@
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>Role Taxonomy (DOH Object Roles)</t>
+          <t>Player Type 태그(신규)</t>
         </is>
       </c>
       <c r="B38" s="2" t="inlineStr">
         <is>
-          <t>역할을 명확히 분리한다. 규모가 커질수록 합치지 말고 유지한다.</t>
+          <t>같은 Feature라도 생성 메커니즘이 선수/아마추어에서 다를 때 [Player Type: Amateur/Elite] 태그로 해석 맥락(Context)을 부여한다. Feature 자체는 바꾸지 않는다. (예: Side Bend Excessive (P7))</t>
         </is>
       </c>
     </row>
     <row r="39">
-      <c r="A39" s="2" t="inlineStr">
-        <is>
-          <t>Core Feature</t>
-        </is>
-      </c>
-      <c r="B39" s="2" t="inlineStr">
-        <is>
-          <t>독립적으로 관찰되는 문제/현상 Feature. 6-섹션 템플릿.</t>
-        </is>
-      </c>
+      <c r="A39" s="2" t="inlineStr"/>
+      <c r="B39" s="2" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>Modifier Feature</t>
+          <t>Role Taxonomy (DOH Object Roles)</t>
         </is>
       </c>
       <c r="B40" s="2" t="inlineStr">
         <is>
-          <t>다른 Feature의 해석을 바꾸는 보조 Feature. 5-섹션 템플릿(원인/이후/Strong Co-occurrence 없음).</t>
+          <t>역할을 명확히 분리한다. 규모가 커질수록 합치지 말고 유지한다.</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
         <is>
-          <t>Setup Influence</t>
+          <t>Core Feature</t>
         </is>
       </c>
       <c r="B41" s="2" t="inlineStr">
         <is>
-          <t>P1 Setup에서 기원하는 영향 요인(예: Grip Strong/Weak). 후속 Phase에서 새로 만들지 않고 참조한다.</t>
+          <t>독립적으로 관찰되는 문제/현상 Feature. 6-섹션 템플릿.</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>Coaching Knowledge</t>
+          <t>Modifier Feature</t>
         </is>
       </c>
       <c r="B42" s="2" t="inlineStr">
         <is>
-          <t>여러 Feature 종합 해석·레슨 이미지·조건부 지식(예: Arm Dominant Pattern). 별도 시트.</t>
+          <t>다른 Feature의 해석을 바꾸는 보조 Feature. 5-섹션 템플릿(원인/이후/Strong Co-occurrence 없음).</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
         <is>
-          <t>Candidate Concepts</t>
+          <t>Setup Influence</t>
         </is>
       </c>
       <c r="B43" s="2" t="inlineStr">
         <is>
-          <t>Feature화가 애매한 개념. 'DOH Candidate Concepts' 시트에 선등록(Repeated 공백).</t>
+          <t>P1 Setup에서 기원하는 영향 요인(예: Grip Strong/Weak). 후속 Phase에서 새로 만들지 않고 참조한다.</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
         <is>
-          <t>Biomechanical Concepts</t>
+          <t>Coaching Knowledge</t>
         </is>
       </c>
       <c r="B44" s="2" t="inlineStr">
         <is>
-          <t>생체역학 개념·Injury Risk 등(예: Lumbar Stress). Mechanism/Note로 관리.</t>
+          <t>여러 Feature 종합 해석·레슨 이미지·조건부 지식(예: Arm Dominant Pattern). 별도 시트.</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
         <is>
-          <t>Derived Parameters</t>
+          <t>Candidate Concepts</t>
         </is>
       </c>
       <c r="B45" s="2" t="inlineStr">
         <is>
-          <t>계산·조합으로 산출되는 값(예: Dynamic Loft). 별도 시트.</t>
+          <t>Feature화가 애매한 개념. 'DOH Candidate Concepts' 시트에 선등록(Repeated 공백).</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
         <is>
-          <t>PST</t>
+          <t>Biomechanical Concepts</t>
         </is>
       </c>
       <c r="B46" s="2" t="inlineStr">
         <is>
-          <t>Posture/Axis Mechanism 카테고리(척추각·측굴·전경·몸통 높이). CMP와 합치지 않고 유지(LOCK).</t>
+          <t>생체역학 개념·Injury Risk 등(예: Lumbar Stress). Mechanism/Note로 관리.</t>
         </is>
       </c>
     </row>
     <row r="47">
-      <c r="A47" s="2" t="inlineStr"/>
-      <c r="B47" s="2" t="inlineStr"/>
+      <c r="A47" s="2" t="inlineStr">
+        <is>
+          <t>Derived Parameters</t>
+        </is>
+      </c>
+      <c r="B47" s="2" t="inlineStr">
+        <is>
+          <t>계산·조합으로 산출되는 값(예: Dynamic Loft). 별도 시트.</t>
+        </is>
+      </c>
     </row>
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
         <is>
+          <t>PST</t>
+        </is>
+      </c>
+      <c r="B48" s="2" t="inlineStr">
+        <is>
+          <t>Posture/Axis Mechanism 카테고리(척추각·측굴·전경·몸통 높이). CMP와 합치지 않고 유지(LOCK).</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="2" t="inlineStr"/>
+      <c r="B49" s="2" t="inlineStr"/>
+    </row>
+    <row r="50">
+      <c r="A50" s="2" t="inlineStr">
+        <is>
           <t>⑩ Candidate 우선 원칙</t>
         </is>
       </c>
-      <c r="B48" s="2" t="inlineStr">
+      <c r="B50" s="2" t="inlineStr">
         <is>
           <t>Stage 2 등 이후 작업에서 새 개념/Mechanism 구조/Knowledge Structure가 나오면 억지로 Feature를 만들지 말고 Candidate Concepts 시트에 먼저 등록한다. Definition·First Found·Status·Example만 작성하고 Repeated는 비워둔다.</t>
         </is>
       </c>
     </row>
-    <row r="49">
-      <c r="A49" s="2" t="inlineStr">
+    <row r="51">
+      <c r="A51" s="2" t="inlineStr">
         <is>
           <t>⑪ Dictionary 수정 정책(LOCK)</t>
         </is>
       </c>
-      <c r="B49" s="2" t="inlineStr">
+      <c r="B51" s="2" t="inlineStr">
         <is>
           <t>현재 Dictionary는 유지. P1~P4 진행 중에는 '추가'만 하고 수정은 최소화한다. P4 완료 후 Dictionary Refactoring을 1회 일괄 수행한다.</t>
         </is>
@@ -7225,7 +9623,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O21"/>
+  <dimension ref="A1:O22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -7246,77 +9644,77 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="9" t="inlineStr">
+      <c r="A1" s="10" t="inlineStr">
         <is>
           <t>Feature</t>
         </is>
       </c>
-      <c r="B1" s="9" t="inlineStr">
+      <c r="B1" s="10" t="inlineStr">
         <is>
           <t>Heel</t>
         </is>
       </c>
-      <c r="C1" s="9" t="inlineStr">
+      <c r="C1" s="10" t="inlineStr">
         <is>
           <t>Toe</t>
         </is>
       </c>
-      <c r="D1" s="9" t="inlineStr">
+      <c r="D1" s="10" t="inlineStr">
         <is>
           <t>High Face</t>
         </is>
       </c>
-      <c r="E1" s="9" t="inlineStr">
+      <c r="E1" s="10" t="inlineStr">
         <is>
           <t>Low Face</t>
         </is>
       </c>
-      <c r="F1" s="9" t="inlineStr">
+      <c r="F1" s="10" t="inlineStr">
         <is>
           <t>Slice</t>
         </is>
       </c>
-      <c r="G1" s="9" t="inlineStr">
+      <c r="G1" s="10" t="inlineStr">
         <is>
           <t>Hook</t>
         </is>
       </c>
-      <c r="H1" s="9" t="inlineStr">
+      <c r="H1" s="10" t="inlineStr">
         <is>
           <t>Push</t>
         </is>
       </c>
-      <c r="I1" s="9" t="inlineStr">
+      <c r="I1" s="10" t="inlineStr">
         <is>
           <t>Pull</t>
         </is>
       </c>
-      <c r="J1" s="9" t="inlineStr">
+      <c r="J1" s="10" t="inlineStr">
         <is>
           <t>Fade</t>
         </is>
       </c>
-      <c r="K1" s="9" t="inlineStr">
+      <c r="K1" s="10" t="inlineStr">
         <is>
           <t>Draw</t>
         </is>
       </c>
-      <c r="L1" s="9" t="inlineStr">
+      <c r="L1" s="10" t="inlineStr">
         <is>
           <t>Fat</t>
         </is>
       </c>
-      <c r="M1" s="9" t="inlineStr">
+      <c r="M1" s="10" t="inlineStr">
         <is>
           <t>Thin</t>
         </is>
       </c>
-      <c r="N1" s="9" t="inlineStr">
+      <c r="N1" s="10" t="inlineStr">
         <is>
           <t>Top</t>
         </is>
       </c>
-      <c r="O1" s="9" t="inlineStr">
+      <c r="O1" s="10" t="inlineStr">
         <is>
           <t>Chunk</t>
         </is>
@@ -7675,7 +10073,14 @@
     <row r="21">
       <c r="A21" s="4" t="inlineStr">
         <is>
-          <t>이 Matrix는 Feature를 설명하는 것이 아니라, 회원의 Ball Flight·Contact·Strike로부터 Feature를 역추론하는 Evidence Layer이다.</t>
+          <t>이 Matrix는 Feature 설명이 아니라, 회원의 Ball Flight·Contact·Strike로부터 Feature를 역추론하는 Evidence Layer이다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="4" t="inlineStr">
+        <is>
+          <t>Feature Chain(원인/이후)은 Feature에서 종료하며, Ball Flight·Contact는 여기(Evidence Matrix)에서만 관리한다.</t>
         </is>
       </c>
     </row>
@@ -7690,7 +10095,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F17"/>
+  <dimension ref="A1:F18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -7873,67 +10278,95 @@
       </c>
       <c r="F6" s="2" t="inlineStr"/>
     </row>
-    <row r="8">
-      <c r="A8" s="3" t="inlineStr">
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>Forward Shaft Lean (P7)</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>임팩트에서 샤프트가 타깃 방향으로 기운(전경) 상태. 핸들 선행(Hand Direction Forward)의 기하학적 표현이며 손 위치 Feature와는 구분한다.</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>P7 (2026-07-08)</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>candidate-feature</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="inlineStr">
+        <is>
+          <t>Hand Direction Forward (P7) → Forward Shaft Lean (P7)</t>
+        </is>
+      </c>
+      <c r="F7" s="2" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="3" t="inlineStr">
         <is>
           <t>── DOH Candidate Concepts 운영 규칙 ──</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="4" t="inlineStr">
-        <is>
-          <t>Stage 2 작업 중 새로운 Feature를 만들기 애매한 개념 / 새로운 Mechanism 구조 / 새로운 Knowledge Structure가 발견되면, 억지로 Feature를 만들지 말고 이 시트에 먼저 등록한다.</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="4" t="inlineStr">
         <is>
+          <t>Stage 2 작업 중 새로운 Feature를 만들기 애매한 개념 / 새로운 Mechanism 구조 / 새로운 Knowledge Structure가 발견되면, 억지로 Feature를 만들지 말고 이 시트에 먼저 등록한다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
           <t>Candidate는 Definition · First Found · Status · Example 만 작성하고 Repeated는 비워둔다. (반복 관찰이 누적되면 Repeated를 채우고 승격 검토)</t>
         </is>
       </c>
     </row>
-    <row r="11">
-      <c r="A11" s="4" t="inlineStr"/>
-    </row>
     <row r="12">
-      <c r="A12" s="3" t="inlineStr">
+      <c r="A12" s="4" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="3" t="inlineStr">
         <is>
           <t>── 후보 노드 재분류 로그 (원칙3: 계층별 분류) ──</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="4" t="inlineStr">
-        <is>
-          <t>Dynamic Loft Low / High → Derived Parameters 시트 (계산·조합값).</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="4" t="inlineStr">
         <is>
-          <t>Arm Dominant Pattern → DOH Coaching Knowledge 시트 (여러 Feature 종합 해석).</t>
+          <t>Dynamic Loft Low / High → Derived Parameters 시트 (계산·조합값).</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="4" t="inlineStr">
         <is>
-          <t>Lead Arm Against Chest → Chicken Wing (P7)에 통합 (원칙 ⑨: 독립 Information Gain 없음).</t>
+          <t>Arm Dominant Pattern → DOH Coaching Knowledge 시트 (여러 Feature 종합 해석).</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="4" t="inlineStr">
         <is>
-          <t>Grip Strong / Weak → P1 Setup Influence 참조 (P7 신규 Feature 아님).</t>
+          <t>Lead Arm Against Chest → Chicken Wing (P7)에 통합 (원칙 ⑨: 독립 Information Gain 없음).</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="4" t="inlineStr">
+        <is>
+          <t>Grip Strong / Weak → P1 Setup Influence 참조 (P7 신규 Feature 아님).</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="4" t="inlineStr">
         <is>
           <t>Trail Wrist / Forearm 계열 → P8 Release 단계에서 재검토 (현재 독립 Feature 아님).</t>
         </is>

</xml_diff>

<commit_message>
chore(P7): Todo 시트 Stage 2 완료 상태 갱신
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01AdDd8hWZsADEXdqNySEqXP
</commit_message>
<xml_diff>
--- a/DOH_P7.xlsx
+++ b/DOH_P7.xlsx
@@ -3258,7 +3258,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D19"/>
+  <dimension ref="A1:D20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -3514,12 +3514,12 @@
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>todo</t>
+          <t>done</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>Dictionary 기준 문장만 사용.</t>
+          <t>Dictionary 기준 문장만 사용(무결성 검증 통과).</t>
         </is>
       </c>
     </row>
@@ -3536,10 +3536,14 @@
       </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
-          <t>todo</t>
-        </is>
-      </c>
-      <c r="D13" s="2" t="inlineStr"/>
+          <t>done</t>
+        </is>
+      </c>
+      <c r="D13" s="2" t="inlineStr">
+        <is>
+          <t>Lead Wrist Flexion/Extension.</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
@@ -3549,35 +3553,39 @@
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>각 Feature 우측 Evidence Matrix 컬럼 구조(별점 제외)</t>
+          <t>Evidence Matrix 컬럼 구조(별도 시트, 별점 제외)</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>todo</t>
-        </is>
-      </c>
-      <c r="D14" s="2" t="inlineStr"/>
+          <t>done</t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="inlineStr">
+        <is>
+          <t>16 Feature × 14 Outcome.</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>Evidence Matrix 별점 일괄 부여</t>
+          <t>반영: Chain 종료 규칙 · Branch Mechanism · Confidence 3단계 · Family</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
         <is>
-          <t>todo</t>
+          <t>done</t>
         </is>
       </c>
       <c r="D15" s="2" t="inlineStr">
         <is>
-          <t>P1~P8 설계 완료 후 별도 세션.</t>
+          <t>프로토타입 피드백 5건 전량 반영.</t>
         </is>
       </c>
     </row>
@@ -3589,43 +3597,51 @@
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
+          <t>Evidence Matrix 별점 일괄 부여</t>
+        </is>
+      </c>
+      <c r="C16" s="2" t="inlineStr">
+        <is>
+          <t>todo</t>
+        </is>
+      </c>
+      <c r="D16" s="2" t="inlineStr">
+        <is>
+          <t>P1~P8 설계 완료 후 별도 세션.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="B17" s="2" t="inlineStr">
+        <is>
           <t>HTML/JSON 변환</t>
         </is>
       </c>
-      <c r="C16" s="2" t="inlineStr">
+      <c r="C17" s="2" t="inlineStr">
         <is>
           <t>todo</t>
         </is>
       </c>
-      <c r="D16" s="2" t="inlineStr">
+      <c r="D17" s="2" t="inlineStr">
         <is>
           <t>P1~P8 LOCK 후 일괄.</t>
         </is>
       </c>
     </row>
-    <row r="17">
-      <c r="A17" s="2" t="inlineStr"/>
-      <c r="B17" s="2" t="inlineStr"/>
-      <c r="C17" s="2" t="inlineStr"/>
-      <c r="D17" s="2" t="inlineStr">
+    <row r="18">
+      <c r="A18" s="2" t="inlineStr"/>
+      <c r="B18" s="2" t="inlineStr"/>
+      <c r="C18" s="2" t="inlineStr"/>
+      <c r="D18" s="2" t="inlineStr">
         <is>
           <t> </t>
         </is>
       </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="2" t="inlineStr">
-        <is>
-          <t>참고</t>
-        </is>
-      </c>
-      <c r="B18" s="2" t="inlineStr">
-        <is>
-          <t>작업 순서: Dictionary LOCK → Feature 6-섹션 → Evidence Matrix 별점 → HTML/JSON</t>
-        </is>
-      </c>
-      <c r="C18" s="2" t="inlineStr"/>
-      <c r="D18" s="2" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
@@ -3635,11 +3651,25 @@
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>동일 의미=동일 문장, 동일 Mechanism=동일 문장, 동일 Feature=동일 이름</t>
+          <t>작업 순서: Dictionary LOCK → Feature 6-섹션 → Evidence Matrix 별점 → HTML/JSON</t>
         </is>
       </c>
       <c r="C19" s="2" t="inlineStr"/>
       <c r="D19" s="2" t="inlineStr"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="inlineStr">
+        <is>
+          <t>참고</t>
+        </is>
+      </c>
+      <c r="B20" s="2" t="inlineStr">
+        <is>
+          <t>동일 의미=동일 문장, 동일 Mechanism=동일 문장, 동일 Feature=동일 이름</t>
+        </is>
+      </c>
+      <c r="C20" s="2" t="inlineStr"/>
+      <c r="D20" s="2" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>